<commit_message>
Spot Hire Planner improvements: single-month filter, asset grouping, consistent colors
</commit_message>
<xml_diff>
--- a/uploads/Asset_Activity_Tracker_MASTER.xlsx
+++ b/uploads/Asset_Activity_Tracker_MASTER.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eu001-sp.shell.com/sites/UGPTDWGOMSupplyChain/Shared Documents/SC Delivery/Logistics New Ways of Working/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8828" documentId="8_{8BED3E6F-E7C2-45EA-AB2B-C6B0456C2E64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B711C60B-ECB9-4E9D-B31F-35C84BC9D311}"/>
+  <xr:revisionPtr revIDLastSave="8844" documentId="8_{8BED3E6F-E7C2-45EA-AB2B-C6B0456C2E64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B5878055-B7A9-4B9D-A15C-A979FE1DE677}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38520" yWindow="-4590" windowWidth="38640" windowHeight="21120" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="11_17_2025 Spot Hire Update" sheetId="2" r:id="rId1"/>
@@ -4736,6 +4736,15 @@
     <xf numFmtId="14" fontId="10" fillId="15" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="31" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="31" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="31" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="19" fillId="34" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -4745,13 +4754,139 @@
     <xf numFmtId="0" fontId="19" fillId="34" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="31" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="31" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="31" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="19" fillId="34" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="31" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="22" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="22" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="22" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="22" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="22" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="22" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="18" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="18" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="18" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="18" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="18" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="18" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="18" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="18" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="31" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="31" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="31" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="13" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
@@ -4763,6 +4898,42 @@
     <xf numFmtId="0" fontId="21" fillId="13" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="22" fillId="34" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="34" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="34" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="31" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="31" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="31" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="16" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="16" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="16" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="10" fillId="13" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="10" fillId="15" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="10" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="21" fillId="34" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -4793,175 +4964,7 @@
     <xf numFmtId="14" fontId="10" fillId="29" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="10" fillId="15" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="10" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="16" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="16" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="16" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="10" fillId="13" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="22" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="22" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="22" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="31" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="31" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="31" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="34" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="34" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="34" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="31" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="31" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="31" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="18" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="18" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="18" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="18" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="18" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="18" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="18" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="18" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="22" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="22" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="22" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="18" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="18" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="18" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="18" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="18" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="18" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="18" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="18" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="31" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="34" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="10" fillId="15" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
@@ -5022,9 +5025,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
@@ -29340,56 +29340,56 @@
       <c r="D7" s="40"/>
       <c r="E7" s="40"/>
       <c r="F7" s="40"/>
-      <c r="G7" s="475">
+      <c r="G7" s="532">
         <v>2026</v>
       </c>
-      <c r="H7" s="475"/>
-      <c r="I7" s="475"/>
-      <c r="J7" s="475"/>
-      <c r="K7" s="475"/>
-      <c r="L7" s="475"/>
-      <c r="M7" s="475"/>
-      <c r="N7" s="475"/>
-      <c r="O7" s="475"/>
-      <c r="P7" s="475"/>
-      <c r="Q7" s="475"/>
-      <c r="R7" s="475"/>
-      <c r="S7" s="475"/>
-      <c r="T7" s="475"/>
-      <c r="U7" s="475"/>
-      <c r="V7" s="475"/>
-      <c r="W7" s="475"/>
-      <c r="X7" s="475"/>
-      <c r="Y7" s="475"/>
-      <c r="Z7" s="475"/>
-      <c r="AA7" s="475"/>
-      <c r="AB7" s="475"/>
-      <c r="AC7" s="475"/>
-      <c r="AD7" s="475"/>
-      <c r="AE7" s="475"/>
-      <c r="AF7" s="475"/>
-      <c r="AG7" s="475"/>
-      <c r="AH7" s="475"/>
-      <c r="AI7" s="475"/>
-      <c r="AJ7" s="475"/>
-      <c r="AK7" s="475"/>
-      <c r="AL7" s="475"/>
-      <c r="AM7" s="475"/>
-      <c r="AN7" s="475"/>
-      <c r="AO7" s="475"/>
-      <c r="AP7" s="475"/>
-      <c r="AQ7" s="475"/>
-      <c r="AR7" s="475"/>
-      <c r="AS7" s="475"/>
-      <c r="AT7" s="475"/>
-      <c r="AU7" s="475"/>
-      <c r="AV7" s="475"/>
-      <c r="AW7" s="475"/>
-      <c r="AX7" s="475"/>
-      <c r="AY7" s="475"/>
-      <c r="AZ7" s="475"/>
-      <c r="BA7" s="475"/>
-      <c r="BB7" s="475"/>
+      <c r="H7" s="532"/>
+      <c r="I7" s="532"/>
+      <c r="J7" s="532"/>
+      <c r="K7" s="532"/>
+      <c r="L7" s="532"/>
+      <c r="M7" s="532"/>
+      <c r="N7" s="532"/>
+      <c r="O7" s="532"/>
+      <c r="P7" s="532"/>
+      <c r="Q7" s="532"/>
+      <c r="R7" s="532"/>
+      <c r="S7" s="532"/>
+      <c r="T7" s="532"/>
+      <c r="U7" s="532"/>
+      <c r="V7" s="532"/>
+      <c r="W7" s="532"/>
+      <c r="X7" s="532"/>
+      <c r="Y7" s="532"/>
+      <c r="Z7" s="532"/>
+      <c r="AA7" s="532"/>
+      <c r="AB7" s="532"/>
+      <c r="AC7" s="532"/>
+      <c r="AD7" s="532"/>
+      <c r="AE7" s="532"/>
+      <c r="AF7" s="532"/>
+      <c r="AG7" s="532"/>
+      <c r="AH7" s="532"/>
+      <c r="AI7" s="532"/>
+      <c r="AJ7" s="532"/>
+      <c r="AK7" s="532"/>
+      <c r="AL7" s="532"/>
+      <c r="AM7" s="532"/>
+      <c r="AN7" s="532"/>
+      <c r="AO7" s="532"/>
+      <c r="AP7" s="532"/>
+      <c r="AQ7" s="532"/>
+      <c r="AR7" s="532"/>
+      <c r="AS7" s="532"/>
+      <c r="AT7" s="532"/>
+      <c r="AU7" s="532"/>
+      <c r="AV7" s="532"/>
+      <c r="AW7" s="532"/>
+      <c r="AX7" s="532"/>
+      <c r="AY7" s="532"/>
+      <c r="AZ7" s="532"/>
+      <c r="BA7" s="532"/>
+      <c r="BB7" s="532"/>
     </row>
     <row r="8" spans="1:71" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="40"/>
@@ -29400,78 +29400,78 @@
       <c r="D8" s="40"/>
       <c r="E8" s="40"/>
       <c r="F8" s="40"/>
-      <c r="G8" s="487" t="s">
+      <c r="G8" s="526" t="s">
         <v>72</v>
       </c>
-      <c r="H8" s="487"/>
-      <c r="I8" s="487"/>
-      <c r="J8" s="487"/>
-      <c r="K8" s="482" t="s">
+      <c r="H8" s="526"/>
+      <c r="I8" s="526"/>
+      <c r="J8" s="526"/>
+      <c r="K8" s="527" t="s">
         <v>73</v>
       </c>
-      <c r="L8" s="482"/>
-      <c r="M8" s="482"/>
-      <c r="N8" s="482"/>
-      <c r="O8" s="483" t="s">
+      <c r="L8" s="527"/>
+      <c r="M8" s="527"/>
+      <c r="N8" s="527"/>
+      <c r="O8" s="528" t="s">
         <v>74</v>
       </c>
-      <c r="P8" s="483"/>
-      <c r="Q8" s="483"/>
-      <c r="R8" s="483"/>
-      <c r="S8" s="481" t="s">
+      <c r="P8" s="528"/>
+      <c r="Q8" s="528"/>
+      <c r="R8" s="528"/>
+      <c r="S8" s="538" t="s">
         <v>75</v>
       </c>
-      <c r="T8" s="481"/>
-      <c r="U8" s="481"/>
-      <c r="V8" s="481"/>
-      <c r="W8" s="482" t="s">
+      <c r="T8" s="538"/>
+      <c r="U8" s="538"/>
+      <c r="V8" s="538"/>
+      <c r="W8" s="527" t="s">
         <v>76</v>
       </c>
-      <c r="X8" s="482"/>
-      <c r="Y8" s="482"/>
-      <c r="Z8" s="482"/>
-      <c r="AA8" s="483" t="s">
+      <c r="X8" s="527"/>
+      <c r="Y8" s="527"/>
+      <c r="Z8" s="527"/>
+      <c r="AA8" s="528" t="s">
         <v>77</v>
       </c>
-      <c r="AB8" s="483"/>
-      <c r="AC8" s="483"/>
-      <c r="AD8" s="483"/>
-      <c r="AE8" s="480" t="s">
+      <c r="AB8" s="528"/>
+      <c r="AC8" s="528"/>
+      <c r="AD8" s="528"/>
+      <c r="AE8" s="537" t="s">
         <v>78</v>
       </c>
-      <c r="AF8" s="480"/>
-      <c r="AG8" s="480"/>
-      <c r="AH8" s="480"/>
-      <c r="AI8" s="476" t="s">
+      <c r="AF8" s="537"/>
+      <c r="AG8" s="537"/>
+      <c r="AH8" s="537"/>
+      <c r="AI8" s="533" t="s">
         <v>79</v>
       </c>
-      <c r="AJ8" s="476"/>
-      <c r="AK8" s="476"/>
-      <c r="AL8" s="476"/>
-      <c r="AM8" s="477" t="s">
+      <c r="AJ8" s="533"/>
+      <c r="AK8" s="533"/>
+      <c r="AL8" s="533"/>
+      <c r="AM8" s="534" t="s">
         <v>80</v>
       </c>
-      <c r="AN8" s="477"/>
-      <c r="AO8" s="477"/>
-      <c r="AP8" s="477"/>
-      <c r="AQ8" s="476" t="s">
+      <c r="AN8" s="534"/>
+      <c r="AO8" s="534"/>
+      <c r="AP8" s="534"/>
+      <c r="AQ8" s="533" t="s">
         <v>81</v>
       </c>
-      <c r="AR8" s="476"/>
-      <c r="AS8" s="476"/>
-      <c r="AT8" s="476"/>
-      <c r="AU8" s="477" t="s">
+      <c r="AR8" s="533"/>
+      <c r="AS8" s="533"/>
+      <c r="AT8" s="533"/>
+      <c r="AU8" s="534" t="s">
         <v>82</v>
       </c>
-      <c r="AV8" s="477"/>
-      <c r="AW8" s="477"/>
-      <c r="AX8" s="477"/>
-      <c r="AY8" s="476" t="s">
+      <c r="AV8" s="534"/>
+      <c r="AW8" s="534"/>
+      <c r="AX8" s="534"/>
+      <c r="AY8" s="533" t="s">
         <v>83</v>
       </c>
-      <c r="AZ8" s="476"/>
-      <c r="BA8" s="476"/>
-      <c r="BB8" s="476"/>
+      <c r="AZ8" s="533"/>
+      <c r="BA8" s="533"/>
+      <c r="BB8" s="533"/>
       <c r="BC8" s="8"/>
       <c r="BD8" s="8"/>
       <c r="BE8" s="8"/>
@@ -29688,42 +29688,42 @@
       <c r="P10" s="231"/>
       <c r="Q10" s="231"/>
       <c r="R10" s="378"/>
-      <c r="S10" s="484"/>
-      <c r="T10" s="485"/>
-      <c r="U10" s="485"/>
-      <c r="V10" s="485"/>
-      <c r="W10" s="485"/>
-      <c r="X10" s="485"/>
-      <c r="Y10" s="485"/>
-      <c r="Z10" s="485"/>
-      <c r="AA10" s="485"/>
-      <c r="AB10" s="485"/>
-      <c r="AC10" s="485"/>
-      <c r="AD10" s="486"/>
-      <c r="AE10" s="478"/>
-      <c r="AF10" s="479"/>
-      <c r="AG10" s="479"/>
-      <c r="AH10" s="479"/>
-      <c r="AI10" s="479"/>
-      <c r="AJ10" s="479"/>
-      <c r="AK10" s="479"/>
-      <c r="AL10" s="479"/>
-      <c r="AM10" s="479"/>
-      <c r="AN10" s="479"/>
-      <c r="AO10" s="479"/>
-      <c r="AP10" s="479"/>
-      <c r="AQ10" s="478"/>
-      <c r="AR10" s="479"/>
-      <c r="AS10" s="479"/>
-      <c r="AT10" s="479"/>
-      <c r="AU10" s="479"/>
-      <c r="AV10" s="479"/>
-      <c r="AW10" s="479"/>
-      <c r="AX10" s="479"/>
-      <c r="AY10" s="479"/>
-      <c r="AZ10" s="479"/>
-      <c r="BA10" s="479"/>
-      <c r="BB10" s="479"/>
+      <c r="S10" s="523"/>
+      <c r="T10" s="524"/>
+      <c r="U10" s="524"/>
+      <c r="V10" s="524"/>
+      <c r="W10" s="524"/>
+      <c r="X10" s="524"/>
+      <c r="Y10" s="524"/>
+      <c r="Z10" s="524"/>
+      <c r="AA10" s="524"/>
+      <c r="AB10" s="524"/>
+      <c r="AC10" s="524"/>
+      <c r="AD10" s="525"/>
+      <c r="AE10" s="535"/>
+      <c r="AF10" s="536"/>
+      <c r="AG10" s="536"/>
+      <c r="AH10" s="536"/>
+      <c r="AI10" s="536"/>
+      <c r="AJ10" s="536"/>
+      <c r="AK10" s="536"/>
+      <c r="AL10" s="536"/>
+      <c r="AM10" s="536"/>
+      <c r="AN10" s="536"/>
+      <c r="AO10" s="536"/>
+      <c r="AP10" s="536"/>
+      <c r="AQ10" s="535"/>
+      <c r="AR10" s="536"/>
+      <c r="AS10" s="536"/>
+      <c r="AT10" s="536"/>
+      <c r="AU10" s="536"/>
+      <c r="AV10" s="536"/>
+      <c r="AW10" s="536"/>
+      <c r="AX10" s="536"/>
+      <c r="AY10" s="536"/>
+      <c r="AZ10" s="536"/>
+      <c r="BA10" s="536"/>
+      <c r="BB10" s="536"/>
       <c r="BC10" s="9"/>
       <c r="BD10" s="9"/>
       <c r="BE10" s="9"/>
@@ -31063,7 +31063,7 @@
     </row>
     <row r="31" spans="1:54" x14ac:dyDescent="0.25">
       <c r="A31" s="150"/>
-      <c r="B31" s="503"/>
+      <c r="B31" s="480"/>
       <c r="C31" s="116" t="s">
         <v>44</v>
       </c>
@@ -31127,7 +31127,7 @@
     </row>
     <row r="32" spans="1:54" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="150"/>
-      <c r="B32" s="503"/>
+      <c r="B32" s="480"/>
       <c r="C32" s="363" t="s">
         <v>44</v>
       </c>
@@ -31191,7 +31191,7 @@
     </row>
     <row r="33" spans="1:54" x14ac:dyDescent="0.25">
       <c r="A33" s="150"/>
-      <c r="B33" s="504"/>
+      <c r="B33" s="481"/>
       <c r="C33" s="363" t="s">
         <v>44</v>
       </c>
@@ -31584,7 +31584,7 @@
     </row>
     <row r="39" spans="1:54" x14ac:dyDescent="0.25">
       <c r="A39" s="150"/>
-      <c r="B39" s="536" t="s">
+      <c r="B39" s="507" t="s">
         <v>118</v>
       </c>
       <c r="C39" s="116" t="s">
@@ -31650,7 +31650,7 @@
     </row>
     <row r="40" spans="1:54" x14ac:dyDescent="0.25">
       <c r="A40" s="150"/>
-      <c r="B40" s="536"/>
+      <c r="B40" s="507"/>
       <c r="C40" s="116" t="s">
         <v>113</v>
       </c>
@@ -31714,7 +31714,7 @@
     </row>
     <row r="41" spans="1:54" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="150"/>
-      <c r="B41" s="536"/>
+      <c r="B41" s="507"/>
       <c r="C41" s="116" t="s">
         <v>113</v>
       </c>
@@ -31778,7 +31778,7 @@
     </row>
     <row r="42" spans="1:54" x14ac:dyDescent="0.25">
       <c r="A42" s="150"/>
-      <c r="B42" s="514" t="s">
+      <c r="B42" s="485" t="s">
         <v>122</v>
       </c>
       <c r="C42" s="223" t="s">
@@ -31844,7 +31844,7 @@
     </row>
     <row r="43" spans="1:54" x14ac:dyDescent="0.25">
       <c r="A43" s="150"/>
-      <c r="B43" s="514"/>
+      <c r="B43" s="485"/>
       <c r="C43" s="223" t="s">
         <v>113</v>
       </c>
@@ -31908,7 +31908,7 @@
     </row>
     <row r="44" spans="1:54" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="150"/>
-      <c r="B44" s="514"/>
+      <c r="B44" s="485"/>
       <c r="C44" s="223" t="s">
         <v>113</v>
       </c>
@@ -32231,49 +32231,49 @@
     </row>
     <row r="49" spans="1:54" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A49" s="150"/>
-      <c r="B49" s="515" t="s">
+      <c r="B49" s="486" t="s">
         <v>131</v>
       </c>
-      <c r="C49" s="516"/>
-      <c r="D49" s="516"/>
-      <c r="E49" s="516"/>
-      <c r="F49" s="517"/>
-      <c r="G49" s="491" t="s">
+      <c r="C49" s="487"/>
+      <c r="D49" s="487"/>
+      <c r="E49" s="487"/>
+      <c r="F49" s="488"/>
+      <c r="G49" s="482" t="s">
         <v>132</v>
       </c>
-      <c r="H49" s="492"/>
-      <c r="I49" s="492"/>
-      <c r="J49" s="493"/>
-      <c r="K49" s="491" t="s">
+      <c r="H49" s="483"/>
+      <c r="I49" s="483"/>
+      <c r="J49" s="484"/>
+      <c r="K49" s="482" t="s">
         <v>133</v>
       </c>
-      <c r="L49" s="492"/>
-      <c r="M49" s="492"/>
-      <c r="N49" s="493"/>
-      <c r="O49" s="491" t="s">
+      <c r="L49" s="483"/>
+      <c r="M49" s="483"/>
+      <c r="N49" s="484"/>
+      <c r="O49" s="482" t="s">
         <v>134</v>
       </c>
-      <c r="P49" s="492"/>
-      <c r="Q49" s="492"/>
-      <c r="R49" s="493"/>
-      <c r="S49" s="491" t="s">
+      <c r="P49" s="483"/>
+      <c r="Q49" s="483"/>
+      <c r="R49" s="484"/>
+      <c r="S49" s="482" t="s">
         <v>135</v>
       </c>
-      <c r="T49" s="492"/>
-      <c r="U49" s="492"/>
-      <c r="V49" s="493"/>
-      <c r="W49" s="491" t="s">
+      <c r="T49" s="483"/>
+      <c r="U49" s="483"/>
+      <c r="V49" s="484"/>
+      <c r="W49" s="482" t="s">
         <v>133</v>
       </c>
-      <c r="X49" s="492"/>
-      <c r="Y49" s="492"/>
-      <c r="Z49" s="493"/>
-      <c r="AA49" s="491" t="s">
+      <c r="X49" s="483"/>
+      <c r="Y49" s="483"/>
+      <c r="Z49" s="484"/>
+      <c r="AA49" s="482" t="s">
         <v>136</v>
       </c>
-      <c r="AB49" s="492"/>
-      <c r="AC49" s="492"/>
-      <c r="AD49" s="493"/>
+      <c r="AB49" s="483"/>
+      <c r="AC49" s="483"/>
+      <c r="AD49" s="484"/>
       <c r="AE49" s="192"/>
       <c r="AF49" s="192"/>
       <c r="AG49" s="192"/>
@@ -32301,49 +32301,49 @@
     </row>
     <row r="50" spans="1:54" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A50" s="150"/>
-      <c r="B50" s="488" t="s">
+      <c r="B50" s="508" t="s">
         <v>137</v>
       </c>
-      <c r="C50" s="489"/>
-      <c r="D50" s="489"/>
-      <c r="E50" s="489"/>
-      <c r="F50" s="490"/>
-      <c r="G50" s="469" t="s">
+      <c r="C50" s="509"/>
+      <c r="D50" s="509"/>
+      <c r="E50" s="509"/>
+      <c r="F50" s="510"/>
+      <c r="G50" s="514" t="s">
         <v>136</v>
       </c>
-      <c r="H50" s="470"/>
-      <c r="I50" s="470"/>
-      <c r="J50" s="471"/>
-      <c r="K50" s="469" t="s">
+      <c r="H50" s="515"/>
+      <c r="I50" s="515"/>
+      <c r="J50" s="516"/>
+      <c r="K50" s="514" t="s">
         <v>138</v>
       </c>
-      <c r="L50" s="470"/>
-      <c r="M50" s="470"/>
-      <c r="N50" s="471"/>
-      <c r="O50" s="488" t="s">
+      <c r="L50" s="515"/>
+      <c r="M50" s="515"/>
+      <c r="N50" s="516"/>
+      <c r="O50" s="508" t="s">
         <v>139</v>
       </c>
-      <c r="P50" s="489"/>
-      <c r="Q50" s="489"/>
-      <c r="R50" s="490"/>
-      <c r="S50" s="488" t="s">
+      <c r="P50" s="509"/>
+      <c r="Q50" s="509"/>
+      <c r="R50" s="510"/>
+      <c r="S50" s="508" t="s">
         <v>138</v>
       </c>
-      <c r="T50" s="489"/>
-      <c r="U50" s="489"/>
-      <c r="V50" s="490"/>
-      <c r="W50" s="488" t="s">
+      <c r="T50" s="509"/>
+      <c r="U50" s="509"/>
+      <c r="V50" s="510"/>
+      <c r="W50" s="508" t="s">
         <v>138</v>
       </c>
-      <c r="X50" s="489"/>
-      <c r="Y50" s="489"/>
-      <c r="Z50" s="490"/>
-      <c r="AA50" s="488" t="s">
+      <c r="X50" s="509"/>
+      <c r="Y50" s="509"/>
+      <c r="Z50" s="510"/>
+      <c r="AA50" s="508" t="s">
         <v>138</v>
       </c>
-      <c r="AB50" s="489"/>
-      <c r="AC50" s="489"/>
-      <c r="AD50" s="490"/>
+      <c r="AB50" s="509"/>
+      <c r="AC50" s="509"/>
+      <c r="AD50" s="510"/>
       <c r="AE50" s="192"/>
       <c r="AF50" s="192"/>
       <c r="AG50" s="192"/>
@@ -32371,45 +32371,45 @@
     </row>
     <row r="51" spans="1:54" ht="20.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A51" s="150"/>
-      <c r="B51" s="463" t="s">
+      <c r="B51" s="466" t="s">
         <v>140</v>
       </c>
-      <c r="C51" s="464"/>
-      <c r="D51" s="464"/>
-      <c r="E51" s="464"/>
-      <c r="F51" s="465"/>
-      <c r="G51" s="472" t="s">
+      <c r="C51" s="467"/>
+      <c r="D51" s="467"/>
+      <c r="E51" s="467"/>
+      <c r="F51" s="468"/>
+      <c r="G51" s="529" t="s">
         <v>141</v>
       </c>
-      <c r="H51" s="473"/>
-      <c r="I51" s="473"/>
-      <c r="J51" s="474"/>
-      <c r="K51" s="497" t="s">
+      <c r="H51" s="530"/>
+      <c r="I51" s="530"/>
+      <c r="J51" s="531"/>
+      <c r="K51" s="517" t="s">
         <v>142</v>
       </c>
-      <c r="L51" s="498"/>
-      <c r="M51" s="498"/>
-      <c r="N51" s="499"/>
-      <c r="O51" s="463" t="s">
+      <c r="L51" s="518"/>
+      <c r="M51" s="518"/>
+      <c r="N51" s="519"/>
+      <c r="O51" s="466" t="s">
         <v>143</v>
       </c>
-      <c r="P51" s="464"/>
-      <c r="Q51" s="464"/>
-      <c r="R51" s="465"/>
-      <c r="S51" s="463"/>
-      <c r="T51" s="464"/>
-      <c r="U51" s="464"/>
-      <c r="V51" s="465"/>
-      <c r="W51" s="463" t="s">
+      <c r="P51" s="467"/>
+      <c r="Q51" s="467"/>
+      <c r="R51" s="468"/>
+      <c r="S51" s="466"/>
+      <c r="T51" s="467"/>
+      <c r="U51" s="467"/>
+      <c r="V51" s="468"/>
+      <c r="W51" s="466" t="s">
         <v>143</v>
       </c>
-      <c r="X51" s="464"/>
-      <c r="Y51" s="464"/>
-      <c r="Z51" s="465"/>
-      <c r="AA51" s="463"/>
-      <c r="AB51" s="464"/>
-      <c r="AC51" s="464"/>
-      <c r="AD51" s="538"/>
+      <c r="X51" s="467"/>
+      <c r="Y51" s="467"/>
+      <c r="Z51" s="468"/>
+      <c r="AA51" s="466"/>
+      <c r="AB51" s="467"/>
+      <c r="AC51" s="467"/>
+      <c r="AD51" s="479"/>
       <c r="AE51" s="192"/>
       <c r="AF51" s="192"/>
       <c r="AG51" s="192"/>
@@ -32437,43 +32437,43 @@
     </row>
     <row r="52" spans="1:54" ht="43.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A52" s="150"/>
-      <c r="B52" s="466" t="s">
+      <c r="B52" s="463" t="s">
         <v>144</v>
       </c>
-      <c r="C52" s="467"/>
-      <c r="D52" s="467"/>
-      <c r="E52" s="467"/>
-      <c r="F52" s="468"/>
-      <c r="G52" s="494" t="s">
+      <c r="C52" s="464"/>
+      <c r="D52" s="464"/>
+      <c r="E52" s="464"/>
+      <c r="F52" s="465"/>
+      <c r="G52" s="511" t="s">
         <v>145</v>
       </c>
-      <c r="H52" s="495"/>
-      <c r="I52" s="495"/>
-      <c r="J52" s="496"/>
-      <c r="K52" s="500" t="s">
+      <c r="H52" s="512"/>
+      <c r="I52" s="512"/>
+      <c r="J52" s="513"/>
+      <c r="K52" s="520" t="s">
         <v>146</v>
       </c>
-      <c r="L52" s="501"/>
-      <c r="M52" s="501"/>
-      <c r="N52" s="502"/>
-      <c r="O52" s="500" t="s">
+      <c r="L52" s="521"/>
+      <c r="M52" s="521"/>
+      <c r="N52" s="522"/>
+      <c r="O52" s="520" t="s">
         <v>147</v>
       </c>
-      <c r="P52" s="501"/>
-      <c r="Q52" s="501"/>
-      <c r="R52" s="502"/>
-      <c r="S52" s="466"/>
-      <c r="T52" s="467"/>
-      <c r="U52" s="467"/>
-      <c r="V52" s="468"/>
-      <c r="W52" s="466"/>
-      <c r="X52" s="467"/>
-      <c r="Y52" s="467"/>
-      <c r="Z52" s="468"/>
-      <c r="AA52" s="466"/>
-      <c r="AB52" s="467"/>
-      <c r="AC52" s="467"/>
-      <c r="AD52" s="537"/>
+      <c r="P52" s="521"/>
+      <c r="Q52" s="521"/>
+      <c r="R52" s="522"/>
+      <c r="S52" s="463"/>
+      <c r="T52" s="464"/>
+      <c r="U52" s="464"/>
+      <c r="V52" s="465"/>
+      <c r="W52" s="463"/>
+      <c r="X52" s="464"/>
+      <c r="Y52" s="464"/>
+      <c r="Z52" s="465"/>
+      <c r="AA52" s="463"/>
+      <c r="AB52" s="464"/>
+      <c r="AC52" s="464"/>
+      <c r="AD52" s="478"/>
       <c r="AE52" s="192"/>
       <c r="AF52" s="192"/>
       <c r="AG52" s="192"/>
@@ -32501,49 +32501,49 @@
     </row>
     <row r="53" spans="1:54" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="150"/>
-      <c r="B53" s="518" t="s">
+      <c r="B53" s="489" t="s">
         <v>148</v>
       </c>
-      <c r="C53" s="519"/>
-      <c r="D53" s="519"/>
-      <c r="E53" s="519"/>
-      <c r="F53" s="520"/>
-      <c r="G53" s="527" t="s">
+      <c r="C53" s="490"/>
+      <c r="D53" s="490"/>
+      <c r="E53" s="490"/>
+      <c r="F53" s="491"/>
+      <c r="G53" s="498" t="s">
         <v>149</v>
       </c>
-      <c r="H53" s="528"/>
-      <c r="I53" s="528"/>
-      <c r="J53" s="529"/>
-      <c r="K53" s="527" t="s">
+      <c r="H53" s="499"/>
+      <c r="I53" s="499"/>
+      <c r="J53" s="500"/>
+      <c r="K53" s="498" t="s">
         <v>150</v>
       </c>
-      <c r="L53" s="528"/>
-      <c r="M53" s="528"/>
-      <c r="N53" s="529"/>
-      <c r="O53" s="505" t="s">
+      <c r="L53" s="499"/>
+      <c r="M53" s="499"/>
+      <c r="N53" s="500"/>
+      <c r="O53" s="469" t="s">
         <v>151</v>
       </c>
-      <c r="P53" s="506"/>
-      <c r="Q53" s="506"/>
-      <c r="R53" s="507"/>
-      <c r="S53" s="505" t="s">
+      <c r="P53" s="470"/>
+      <c r="Q53" s="470"/>
+      <c r="R53" s="471"/>
+      <c r="S53" s="469" t="s">
         <v>152</v>
       </c>
-      <c r="T53" s="506"/>
-      <c r="U53" s="506"/>
-      <c r="V53" s="507"/>
-      <c r="W53" s="505" t="s">
+      <c r="T53" s="470"/>
+      <c r="U53" s="470"/>
+      <c r="V53" s="471"/>
+      <c r="W53" s="469" t="s">
         <v>153</v>
       </c>
-      <c r="X53" s="506"/>
-      <c r="Y53" s="506"/>
-      <c r="Z53" s="507"/>
-      <c r="AA53" s="505" t="s">
+      <c r="X53" s="470"/>
+      <c r="Y53" s="470"/>
+      <c r="Z53" s="471"/>
+      <c r="AA53" s="469" t="s">
         <v>154</v>
       </c>
-      <c r="AB53" s="506"/>
-      <c r="AC53" s="506"/>
-      <c r="AD53" s="507"/>
+      <c r="AB53" s="470"/>
+      <c r="AC53" s="470"/>
+      <c r="AD53" s="471"/>
       <c r="AE53" s="150"/>
       <c r="AF53" s="150"/>
       <c r="AG53" s="150"/>
@@ -32573,35 +32573,35 @@
     </row>
     <row r="54" spans="1:54" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="150"/>
-      <c r="B54" s="521"/>
-      <c r="C54" s="522"/>
-      <c r="D54" s="522"/>
-      <c r="E54" s="522"/>
-      <c r="F54" s="523"/>
-      <c r="G54" s="530"/>
-      <c r="H54" s="531"/>
-      <c r="I54" s="531"/>
-      <c r="J54" s="532"/>
-      <c r="K54" s="530"/>
-      <c r="L54" s="531"/>
-      <c r="M54" s="531"/>
-      <c r="N54" s="532"/>
-      <c r="O54" s="508"/>
-      <c r="P54" s="509"/>
-      <c r="Q54" s="509"/>
-      <c r="R54" s="510"/>
-      <c r="S54" s="508"/>
-      <c r="T54" s="509"/>
-      <c r="U54" s="509"/>
-      <c r="V54" s="510"/>
-      <c r="W54" s="508"/>
-      <c r="X54" s="509"/>
-      <c r="Y54" s="509"/>
-      <c r="Z54" s="510"/>
-      <c r="AA54" s="508"/>
-      <c r="AB54" s="509"/>
-      <c r="AC54" s="509"/>
-      <c r="AD54" s="510"/>
+      <c r="B54" s="492"/>
+      <c r="C54" s="493"/>
+      <c r="D54" s="493"/>
+      <c r="E54" s="493"/>
+      <c r="F54" s="494"/>
+      <c r="G54" s="501"/>
+      <c r="H54" s="502"/>
+      <c r="I54" s="502"/>
+      <c r="J54" s="503"/>
+      <c r="K54" s="501"/>
+      <c r="L54" s="502"/>
+      <c r="M54" s="502"/>
+      <c r="N54" s="503"/>
+      <c r="O54" s="472"/>
+      <c r="P54" s="473"/>
+      <c r="Q54" s="473"/>
+      <c r="R54" s="474"/>
+      <c r="S54" s="472"/>
+      <c r="T54" s="473"/>
+      <c r="U54" s="473"/>
+      <c r="V54" s="474"/>
+      <c r="W54" s="472"/>
+      <c r="X54" s="473"/>
+      <c r="Y54" s="473"/>
+      <c r="Z54" s="474"/>
+      <c r="AA54" s="472"/>
+      <c r="AB54" s="473"/>
+      <c r="AC54" s="473"/>
+      <c r="AD54" s="474"/>
       <c r="AE54" s="150"/>
       <c r="AF54" s="150"/>
       <c r="AG54" s="150"/>
@@ -32628,35 +32628,35 @@
       <c r="BB54" s="150"/>
     </row>
     <row r="55" spans="1:54" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B55" s="521"/>
-      <c r="C55" s="522"/>
-      <c r="D55" s="522"/>
-      <c r="E55" s="522"/>
-      <c r="F55" s="523"/>
-      <c r="G55" s="530"/>
-      <c r="H55" s="531"/>
-      <c r="I55" s="531"/>
-      <c r="J55" s="532"/>
-      <c r="K55" s="530"/>
-      <c r="L55" s="531"/>
-      <c r="M55" s="531"/>
-      <c r="N55" s="532"/>
-      <c r="O55" s="508"/>
-      <c r="P55" s="509"/>
-      <c r="Q55" s="509"/>
-      <c r="R55" s="510"/>
-      <c r="S55" s="508"/>
-      <c r="T55" s="509"/>
-      <c r="U55" s="509"/>
-      <c r="V55" s="510"/>
-      <c r="W55" s="508"/>
-      <c r="X55" s="509"/>
-      <c r="Y55" s="509"/>
-      <c r="Z55" s="510"/>
-      <c r="AA55" s="508"/>
-      <c r="AB55" s="509"/>
-      <c r="AC55" s="509"/>
-      <c r="AD55" s="510"/>
+      <c r="B55" s="492"/>
+      <c r="C55" s="493"/>
+      <c r="D55" s="493"/>
+      <c r="E55" s="493"/>
+      <c r="F55" s="494"/>
+      <c r="G55" s="501"/>
+      <c r="H55" s="502"/>
+      <c r="I55" s="502"/>
+      <c r="J55" s="503"/>
+      <c r="K55" s="501"/>
+      <c r="L55" s="502"/>
+      <c r="M55" s="502"/>
+      <c r="N55" s="503"/>
+      <c r="O55" s="472"/>
+      <c r="P55" s="473"/>
+      <c r="Q55" s="473"/>
+      <c r="R55" s="474"/>
+      <c r="S55" s="472"/>
+      <c r="T55" s="473"/>
+      <c r="U55" s="473"/>
+      <c r="V55" s="474"/>
+      <c r="W55" s="472"/>
+      <c r="X55" s="473"/>
+      <c r="Y55" s="473"/>
+      <c r="Z55" s="474"/>
+      <c r="AA55" s="472"/>
+      <c r="AB55" s="473"/>
+      <c r="AC55" s="473"/>
+      <c r="AD55" s="474"/>
       <c r="AE55" s="150"/>
       <c r="AF55" s="150"/>
       <c r="AG55" s="150"/>
@@ -32683,447 +32683,478 @@
       <c r="BB55" s="150"/>
     </row>
     <row r="56" spans="1:54" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B56" s="521"/>
-      <c r="C56" s="522"/>
-      <c r="D56" s="522"/>
-      <c r="E56" s="522"/>
-      <c r="F56" s="523"/>
-      <c r="G56" s="530"/>
-      <c r="H56" s="531"/>
-      <c r="I56" s="531"/>
-      <c r="J56" s="532"/>
-      <c r="K56" s="530"/>
-      <c r="L56" s="531"/>
-      <c r="M56" s="531"/>
-      <c r="N56" s="532"/>
-      <c r="O56" s="508"/>
-      <c r="P56" s="509"/>
-      <c r="Q56" s="509"/>
-      <c r="R56" s="510"/>
-      <c r="S56" s="508"/>
-      <c r="T56" s="509"/>
-      <c r="U56" s="509"/>
-      <c r="V56" s="510"/>
-      <c r="W56" s="508"/>
-      <c r="X56" s="509"/>
-      <c r="Y56" s="509"/>
-      <c r="Z56" s="510"/>
-      <c r="AA56" s="508"/>
-      <c r="AB56" s="509"/>
-      <c r="AC56" s="509"/>
-      <c r="AD56" s="510"/>
+      <c r="B56" s="492"/>
+      <c r="C56" s="493"/>
+      <c r="D56" s="493"/>
+      <c r="E56" s="493"/>
+      <c r="F56" s="494"/>
+      <c r="G56" s="501"/>
+      <c r="H56" s="502"/>
+      <c r="I56" s="502"/>
+      <c r="J56" s="503"/>
+      <c r="K56" s="501"/>
+      <c r="L56" s="502"/>
+      <c r="M56" s="502"/>
+      <c r="N56" s="503"/>
+      <c r="O56" s="472"/>
+      <c r="P56" s="473"/>
+      <c r="Q56" s="473"/>
+      <c r="R56" s="474"/>
+      <c r="S56" s="472"/>
+      <c r="T56" s="473"/>
+      <c r="U56" s="473"/>
+      <c r="V56" s="474"/>
+      <c r="W56" s="472"/>
+      <c r="X56" s="473"/>
+      <c r="Y56" s="473"/>
+      <c r="Z56" s="474"/>
+      <c r="AA56" s="472"/>
+      <c r="AB56" s="473"/>
+      <c r="AC56" s="473"/>
+      <c r="AD56" s="474"/>
     </row>
     <row r="57" spans="1:54" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B57" s="521"/>
-      <c r="C57" s="522"/>
-      <c r="D57" s="522"/>
-      <c r="E57" s="522"/>
-      <c r="F57" s="523"/>
-      <c r="G57" s="530"/>
-      <c r="H57" s="531"/>
-      <c r="I57" s="531"/>
-      <c r="J57" s="532"/>
-      <c r="K57" s="530"/>
-      <c r="L57" s="531"/>
-      <c r="M57" s="531"/>
-      <c r="N57" s="532"/>
-      <c r="O57" s="508"/>
-      <c r="P57" s="509"/>
-      <c r="Q57" s="509"/>
-      <c r="R57" s="510"/>
-      <c r="S57" s="508"/>
-      <c r="T57" s="509"/>
-      <c r="U57" s="509"/>
-      <c r="V57" s="510"/>
-      <c r="W57" s="508"/>
-      <c r="X57" s="509"/>
-      <c r="Y57" s="509"/>
-      <c r="Z57" s="510"/>
-      <c r="AA57" s="508"/>
-      <c r="AB57" s="509"/>
-      <c r="AC57" s="509"/>
-      <c r="AD57" s="510"/>
+      <c r="B57" s="492"/>
+      <c r="C57" s="493"/>
+      <c r="D57" s="493"/>
+      <c r="E57" s="493"/>
+      <c r="F57" s="494"/>
+      <c r="G57" s="501"/>
+      <c r="H57" s="502"/>
+      <c r="I57" s="502"/>
+      <c r="J57" s="503"/>
+      <c r="K57" s="501"/>
+      <c r="L57" s="502"/>
+      <c r="M57" s="502"/>
+      <c r="N57" s="503"/>
+      <c r="O57" s="472"/>
+      <c r="P57" s="473"/>
+      <c r="Q57" s="473"/>
+      <c r="R57" s="474"/>
+      <c r="S57" s="472"/>
+      <c r="T57" s="473"/>
+      <c r="U57" s="473"/>
+      <c r="V57" s="474"/>
+      <c r="W57" s="472"/>
+      <c r="X57" s="473"/>
+      <c r="Y57" s="473"/>
+      <c r="Z57" s="474"/>
+      <c r="AA57" s="472"/>
+      <c r="AB57" s="473"/>
+      <c r="AC57" s="473"/>
+      <c r="AD57" s="474"/>
     </row>
     <row r="58" spans="1:54" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B58" s="521"/>
-      <c r="C58" s="522"/>
-      <c r="D58" s="522"/>
-      <c r="E58" s="522"/>
-      <c r="F58" s="523"/>
-      <c r="G58" s="530"/>
-      <c r="H58" s="531"/>
-      <c r="I58" s="531"/>
-      <c r="J58" s="532"/>
-      <c r="K58" s="530"/>
-      <c r="L58" s="531"/>
-      <c r="M58" s="531"/>
-      <c r="N58" s="532"/>
-      <c r="O58" s="508"/>
-      <c r="P58" s="509"/>
-      <c r="Q58" s="509"/>
-      <c r="R58" s="510"/>
-      <c r="S58" s="508"/>
-      <c r="T58" s="509"/>
-      <c r="U58" s="509"/>
-      <c r="V58" s="510"/>
-      <c r="W58" s="508"/>
-      <c r="X58" s="509"/>
-      <c r="Y58" s="509"/>
-      <c r="Z58" s="510"/>
-      <c r="AA58" s="508"/>
-      <c r="AB58" s="509"/>
-      <c r="AC58" s="509"/>
-      <c r="AD58" s="510"/>
+      <c r="B58" s="492"/>
+      <c r="C58" s="493"/>
+      <c r="D58" s="493"/>
+      <c r="E58" s="493"/>
+      <c r="F58" s="494"/>
+      <c r="G58" s="501"/>
+      <c r="H58" s="502"/>
+      <c r="I58" s="502"/>
+      <c r="J58" s="503"/>
+      <c r="K58" s="501"/>
+      <c r="L58" s="502"/>
+      <c r="M58" s="502"/>
+      <c r="N58" s="503"/>
+      <c r="O58" s="472"/>
+      <c r="P58" s="473"/>
+      <c r="Q58" s="473"/>
+      <c r="R58" s="474"/>
+      <c r="S58" s="472"/>
+      <c r="T58" s="473"/>
+      <c r="U58" s="473"/>
+      <c r="V58" s="474"/>
+      <c r="W58" s="472"/>
+      <c r="X58" s="473"/>
+      <c r="Y58" s="473"/>
+      <c r="Z58" s="474"/>
+      <c r="AA58" s="472"/>
+      <c r="AB58" s="473"/>
+      <c r="AC58" s="473"/>
+      <c r="AD58" s="474"/>
     </row>
     <row r="59" spans="1:54" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B59" s="521"/>
-      <c r="C59" s="522"/>
-      <c r="D59" s="522"/>
-      <c r="E59" s="522"/>
-      <c r="F59" s="523"/>
-      <c r="G59" s="530"/>
-      <c r="H59" s="531"/>
-      <c r="I59" s="531"/>
-      <c r="J59" s="532"/>
-      <c r="K59" s="530"/>
-      <c r="L59" s="531"/>
-      <c r="M59" s="531"/>
-      <c r="N59" s="532"/>
-      <c r="O59" s="508"/>
-      <c r="P59" s="509"/>
-      <c r="Q59" s="509"/>
-      <c r="R59" s="510"/>
-      <c r="S59" s="508"/>
-      <c r="T59" s="509"/>
-      <c r="U59" s="509"/>
-      <c r="V59" s="510"/>
-      <c r="W59" s="508"/>
-      <c r="X59" s="509"/>
-      <c r="Y59" s="509"/>
-      <c r="Z59" s="510"/>
-      <c r="AA59" s="508"/>
-      <c r="AB59" s="509"/>
-      <c r="AC59" s="509"/>
-      <c r="AD59" s="510"/>
+      <c r="B59" s="492"/>
+      <c r="C59" s="493"/>
+      <c r="D59" s="493"/>
+      <c r="E59" s="493"/>
+      <c r="F59" s="494"/>
+      <c r="G59" s="501"/>
+      <c r="H59" s="502"/>
+      <c r="I59" s="502"/>
+      <c r="J59" s="503"/>
+      <c r="K59" s="501"/>
+      <c r="L59" s="502"/>
+      <c r="M59" s="502"/>
+      <c r="N59" s="503"/>
+      <c r="O59" s="472"/>
+      <c r="P59" s="473"/>
+      <c r="Q59" s="473"/>
+      <c r="R59" s="474"/>
+      <c r="S59" s="472"/>
+      <c r="T59" s="473"/>
+      <c r="U59" s="473"/>
+      <c r="V59" s="474"/>
+      <c r="W59" s="472"/>
+      <c r="X59" s="473"/>
+      <c r="Y59" s="473"/>
+      <c r="Z59" s="474"/>
+      <c r="AA59" s="472"/>
+      <c r="AB59" s="473"/>
+      <c r="AC59" s="473"/>
+      <c r="AD59" s="474"/>
     </row>
     <row r="60" spans="1:54" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B60" s="521"/>
-      <c r="C60" s="522"/>
-      <c r="D60" s="522"/>
-      <c r="E60" s="522"/>
-      <c r="F60" s="523"/>
-      <c r="G60" s="530"/>
-      <c r="H60" s="531"/>
-      <c r="I60" s="531"/>
-      <c r="J60" s="532"/>
-      <c r="K60" s="530"/>
-      <c r="L60" s="531"/>
-      <c r="M60" s="531"/>
-      <c r="N60" s="532"/>
-      <c r="O60" s="508"/>
-      <c r="P60" s="509"/>
-      <c r="Q60" s="509"/>
-      <c r="R60" s="510"/>
-      <c r="S60" s="508"/>
-      <c r="T60" s="509"/>
-      <c r="U60" s="509"/>
-      <c r="V60" s="510"/>
-      <c r="W60" s="508"/>
-      <c r="X60" s="509"/>
-      <c r="Y60" s="509"/>
-      <c r="Z60" s="510"/>
-      <c r="AA60" s="508"/>
-      <c r="AB60" s="509"/>
-      <c r="AC60" s="509"/>
-      <c r="AD60" s="510"/>
+      <c r="B60" s="492"/>
+      <c r="C60" s="493"/>
+      <c r="D60" s="493"/>
+      <c r="E60" s="493"/>
+      <c r="F60" s="494"/>
+      <c r="G60" s="501"/>
+      <c r="H60" s="502"/>
+      <c r="I60" s="502"/>
+      <c r="J60" s="503"/>
+      <c r="K60" s="501"/>
+      <c r="L60" s="502"/>
+      <c r="M60" s="502"/>
+      <c r="N60" s="503"/>
+      <c r="O60" s="472"/>
+      <c r="P60" s="473"/>
+      <c r="Q60" s="473"/>
+      <c r="R60" s="474"/>
+      <c r="S60" s="472"/>
+      <c r="T60" s="473"/>
+      <c r="U60" s="473"/>
+      <c r="V60" s="474"/>
+      <c r="W60" s="472"/>
+      <c r="X60" s="473"/>
+      <c r="Y60" s="473"/>
+      <c r="Z60" s="474"/>
+      <c r="AA60" s="472"/>
+      <c r="AB60" s="473"/>
+      <c r="AC60" s="473"/>
+      <c r="AD60" s="474"/>
     </row>
     <row r="61" spans="1:54" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B61" s="521"/>
-      <c r="C61" s="522"/>
-      <c r="D61" s="522"/>
-      <c r="E61" s="522"/>
-      <c r="F61" s="523"/>
-      <c r="G61" s="530"/>
-      <c r="H61" s="531"/>
-      <c r="I61" s="531"/>
-      <c r="J61" s="532"/>
-      <c r="K61" s="530"/>
-      <c r="L61" s="531"/>
-      <c r="M61" s="531"/>
-      <c r="N61" s="532"/>
-      <c r="O61" s="508"/>
-      <c r="P61" s="509"/>
-      <c r="Q61" s="509"/>
-      <c r="R61" s="510"/>
-      <c r="S61" s="508"/>
-      <c r="T61" s="509"/>
-      <c r="U61" s="509"/>
-      <c r="V61" s="510"/>
-      <c r="W61" s="508"/>
-      <c r="X61" s="509"/>
-      <c r="Y61" s="509"/>
-      <c r="Z61" s="510"/>
-      <c r="AA61" s="508"/>
-      <c r="AB61" s="509"/>
-      <c r="AC61" s="509"/>
-      <c r="AD61" s="510"/>
+      <c r="B61" s="492"/>
+      <c r="C61" s="493"/>
+      <c r="D61" s="493"/>
+      <c r="E61" s="493"/>
+      <c r="F61" s="494"/>
+      <c r="G61" s="501"/>
+      <c r="H61" s="502"/>
+      <c r="I61" s="502"/>
+      <c r="J61" s="503"/>
+      <c r="K61" s="501"/>
+      <c r="L61" s="502"/>
+      <c r="M61" s="502"/>
+      <c r="N61" s="503"/>
+      <c r="O61" s="472"/>
+      <c r="P61" s="473"/>
+      <c r="Q61" s="473"/>
+      <c r="R61" s="474"/>
+      <c r="S61" s="472"/>
+      <c r="T61" s="473"/>
+      <c r="U61" s="473"/>
+      <c r="V61" s="474"/>
+      <c r="W61" s="472"/>
+      <c r="X61" s="473"/>
+      <c r="Y61" s="473"/>
+      <c r="Z61" s="474"/>
+      <c r="AA61" s="472"/>
+      <c r="AB61" s="473"/>
+      <c r="AC61" s="473"/>
+      <c r="AD61" s="474"/>
     </row>
     <row r="62" spans="1:54" ht="52.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B62" s="521"/>
-      <c r="C62" s="522"/>
-      <c r="D62" s="522"/>
-      <c r="E62" s="522"/>
-      <c r="F62" s="523"/>
-      <c r="G62" s="530"/>
-      <c r="H62" s="531"/>
-      <c r="I62" s="531"/>
-      <c r="J62" s="532"/>
-      <c r="K62" s="530"/>
-      <c r="L62" s="531"/>
-      <c r="M62" s="531"/>
-      <c r="N62" s="532"/>
-      <c r="O62" s="508"/>
-      <c r="P62" s="509"/>
-      <c r="Q62" s="509"/>
-      <c r="R62" s="510"/>
-      <c r="S62" s="508"/>
-      <c r="T62" s="509"/>
-      <c r="U62" s="509"/>
-      <c r="V62" s="510"/>
-      <c r="W62" s="508"/>
-      <c r="X62" s="509"/>
-      <c r="Y62" s="509"/>
-      <c r="Z62" s="510"/>
-      <c r="AA62" s="508"/>
-      <c r="AB62" s="509"/>
-      <c r="AC62" s="509"/>
-      <c r="AD62" s="510"/>
+      <c r="B62" s="492"/>
+      <c r="C62" s="493"/>
+      <c r="D62" s="493"/>
+      <c r="E62" s="493"/>
+      <c r="F62" s="494"/>
+      <c r="G62" s="501"/>
+      <c r="H62" s="502"/>
+      <c r="I62" s="502"/>
+      <c r="J62" s="503"/>
+      <c r="K62" s="501"/>
+      <c r="L62" s="502"/>
+      <c r="M62" s="502"/>
+      <c r="N62" s="503"/>
+      <c r="O62" s="472"/>
+      <c r="P62" s="473"/>
+      <c r="Q62" s="473"/>
+      <c r="R62" s="474"/>
+      <c r="S62" s="472"/>
+      <c r="T62" s="473"/>
+      <c r="U62" s="473"/>
+      <c r="V62" s="474"/>
+      <c r="W62" s="472"/>
+      <c r="X62" s="473"/>
+      <c r="Y62" s="473"/>
+      <c r="Z62" s="474"/>
+      <c r="AA62" s="472"/>
+      <c r="AB62" s="473"/>
+      <c r="AC62" s="473"/>
+      <c r="AD62" s="474"/>
     </row>
     <row r="63" spans="1:54" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B63" s="521"/>
-      <c r="C63" s="522"/>
-      <c r="D63" s="522"/>
-      <c r="E63" s="522"/>
-      <c r="F63" s="523"/>
-      <c r="G63" s="530"/>
-      <c r="H63" s="531"/>
-      <c r="I63" s="531"/>
-      <c r="J63" s="532"/>
-      <c r="K63" s="530"/>
-      <c r="L63" s="531"/>
-      <c r="M63" s="531"/>
-      <c r="N63" s="532"/>
-      <c r="O63" s="508"/>
-      <c r="P63" s="509"/>
-      <c r="Q63" s="509"/>
-      <c r="R63" s="510"/>
-      <c r="S63" s="508"/>
-      <c r="T63" s="509"/>
-      <c r="U63" s="509"/>
-      <c r="V63" s="510"/>
-      <c r="W63" s="508"/>
-      <c r="X63" s="509"/>
-      <c r="Y63" s="509"/>
-      <c r="Z63" s="510"/>
-      <c r="AA63" s="508"/>
-      <c r="AB63" s="509"/>
-      <c r="AC63" s="509"/>
-      <c r="AD63" s="510"/>
+      <c r="B63" s="492"/>
+      <c r="C63" s="493"/>
+      <c r="D63" s="493"/>
+      <c r="E63" s="493"/>
+      <c r="F63" s="494"/>
+      <c r="G63" s="501"/>
+      <c r="H63" s="502"/>
+      <c r="I63" s="502"/>
+      <c r="J63" s="503"/>
+      <c r="K63" s="501"/>
+      <c r="L63" s="502"/>
+      <c r="M63" s="502"/>
+      <c r="N63" s="503"/>
+      <c r="O63" s="472"/>
+      <c r="P63" s="473"/>
+      <c r="Q63" s="473"/>
+      <c r="R63" s="474"/>
+      <c r="S63" s="472"/>
+      <c r="T63" s="473"/>
+      <c r="U63" s="473"/>
+      <c r="V63" s="474"/>
+      <c r="W63" s="472"/>
+      <c r="X63" s="473"/>
+      <c r="Y63" s="473"/>
+      <c r="Z63" s="474"/>
+      <c r="AA63" s="472"/>
+      <c r="AB63" s="473"/>
+      <c r="AC63" s="473"/>
+      <c r="AD63" s="474"/>
     </row>
     <row r="64" spans="1:54" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B64" s="521"/>
-      <c r="C64" s="522"/>
-      <c r="D64" s="522"/>
-      <c r="E64" s="522"/>
-      <c r="F64" s="523"/>
-      <c r="G64" s="530"/>
-      <c r="H64" s="531"/>
-      <c r="I64" s="531"/>
-      <c r="J64" s="532"/>
-      <c r="K64" s="530"/>
-      <c r="L64" s="531"/>
-      <c r="M64" s="531"/>
-      <c r="N64" s="532"/>
-      <c r="O64" s="508"/>
-      <c r="P64" s="509"/>
-      <c r="Q64" s="509"/>
-      <c r="R64" s="510"/>
-      <c r="S64" s="508"/>
-      <c r="T64" s="509"/>
-      <c r="U64" s="509"/>
-      <c r="V64" s="510"/>
-      <c r="W64" s="508"/>
-      <c r="X64" s="509"/>
-      <c r="Y64" s="509"/>
-      <c r="Z64" s="510"/>
-      <c r="AA64" s="508"/>
-      <c r="AB64" s="509"/>
-      <c r="AC64" s="509"/>
-      <c r="AD64" s="510"/>
+      <c r="B64" s="492"/>
+      <c r="C64" s="493"/>
+      <c r="D64" s="493"/>
+      <c r="E64" s="493"/>
+      <c r="F64" s="494"/>
+      <c r="G64" s="501"/>
+      <c r="H64" s="502"/>
+      <c r="I64" s="502"/>
+      <c r="J64" s="503"/>
+      <c r="K64" s="501"/>
+      <c r="L64" s="502"/>
+      <c r="M64" s="502"/>
+      <c r="N64" s="503"/>
+      <c r="O64" s="472"/>
+      <c r="P64" s="473"/>
+      <c r="Q64" s="473"/>
+      <c r="R64" s="474"/>
+      <c r="S64" s="472"/>
+      <c r="T64" s="473"/>
+      <c r="U64" s="473"/>
+      <c r="V64" s="474"/>
+      <c r="W64" s="472"/>
+      <c r="X64" s="473"/>
+      <c r="Y64" s="473"/>
+      <c r="Z64" s="474"/>
+      <c r="AA64" s="472"/>
+      <c r="AB64" s="473"/>
+      <c r="AC64" s="473"/>
+      <c r="AD64" s="474"/>
     </row>
     <row r="65" spans="2:30" ht="67.150000000000006" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B65" s="521"/>
-      <c r="C65" s="522"/>
-      <c r="D65" s="522"/>
-      <c r="E65" s="522"/>
-      <c r="F65" s="523"/>
-      <c r="G65" s="530"/>
-      <c r="H65" s="531"/>
-      <c r="I65" s="531"/>
-      <c r="J65" s="532"/>
-      <c r="K65" s="530"/>
-      <c r="L65" s="531"/>
-      <c r="M65" s="531"/>
-      <c r="N65" s="532"/>
-      <c r="O65" s="508"/>
-      <c r="P65" s="509"/>
-      <c r="Q65" s="509"/>
-      <c r="R65" s="510"/>
-      <c r="S65" s="508"/>
-      <c r="T65" s="509"/>
-      <c r="U65" s="509"/>
-      <c r="V65" s="510"/>
-      <c r="W65" s="508"/>
-      <c r="X65" s="509"/>
-      <c r="Y65" s="509"/>
-      <c r="Z65" s="510"/>
-      <c r="AA65" s="508"/>
-      <c r="AB65" s="509"/>
-      <c r="AC65" s="509"/>
-      <c r="AD65" s="510"/>
+      <c r="B65" s="492"/>
+      <c r="C65" s="493"/>
+      <c r="D65" s="493"/>
+      <c r="E65" s="493"/>
+      <c r="F65" s="494"/>
+      <c r="G65" s="501"/>
+      <c r="H65" s="502"/>
+      <c r="I65" s="502"/>
+      <c r="J65" s="503"/>
+      <c r="K65" s="501"/>
+      <c r="L65" s="502"/>
+      <c r="M65" s="502"/>
+      <c r="N65" s="503"/>
+      <c r="O65" s="472"/>
+      <c r="P65" s="473"/>
+      <c r="Q65" s="473"/>
+      <c r="R65" s="474"/>
+      <c r="S65" s="472"/>
+      <c r="T65" s="473"/>
+      <c r="U65" s="473"/>
+      <c r="V65" s="474"/>
+      <c r="W65" s="472"/>
+      <c r="X65" s="473"/>
+      <c r="Y65" s="473"/>
+      <c r="Z65" s="474"/>
+      <c r="AA65" s="472"/>
+      <c r="AB65" s="473"/>
+      <c r="AC65" s="473"/>
+      <c r="AD65" s="474"/>
     </row>
     <row r="66" spans="2:30" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B66" s="521"/>
-      <c r="C66" s="522"/>
-      <c r="D66" s="522"/>
-      <c r="E66" s="522"/>
-      <c r="F66" s="523"/>
-      <c r="G66" s="530"/>
-      <c r="H66" s="531"/>
-      <c r="I66" s="531"/>
-      <c r="J66" s="532"/>
-      <c r="K66" s="530"/>
-      <c r="L66" s="531"/>
-      <c r="M66" s="531"/>
-      <c r="N66" s="532"/>
-      <c r="O66" s="508"/>
-      <c r="P66" s="509"/>
-      <c r="Q66" s="509"/>
-      <c r="R66" s="510"/>
-      <c r="S66" s="508"/>
-      <c r="T66" s="509"/>
-      <c r="U66" s="509"/>
-      <c r="V66" s="510"/>
-      <c r="W66" s="508"/>
-      <c r="X66" s="509"/>
-      <c r="Y66" s="509"/>
-      <c r="Z66" s="510"/>
-      <c r="AA66" s="508"/>
-      <c r="AB66" s="509"/>
-      <c r="AC66" s="509"/>
-      <c r="AD66" s="510"/>
+      <c r="B66" s="492"/>
+      <c r="C66" s="493"/>
+      <c r="D66" s="493"/>
+      <c r="E66" s="493"/>
+      <c r="F66" s="494"/>
+      <c r="G66" s="501"/>
+      <c r="H66" s="502"/>
+      <c r="I66" s="502"/>
+      <c r="J66" s="503"/>
+      <c r="K66" s="501"/>
+      <c r="L66" s="502"/>
+      <c r="M66" s="502"/>
+      <c r="N66" s="503"/>
+      <c r="O66" s="472"/>
+      <c r="P66" s="473"/>
+      <c r="Q66" s="473"/>
+      <c r="R66" s="474"/>
+      <c r="S66" s="472"/>
+      <c r="T66" s="473"/>
+      <c r="U66" s="473"/>
+      <c r="V66" s="474"/>
+      <c r="W66" s="472"/>
+      <c r="X66" s="473"/>
+      <c r="Y66" s="473"/>
+      <c r="Z66" s="474"/>
+      <c r="AA66" s="472"/>
+      <c r="AB66" s="473"/>
+      <c r="AC66" s="473"/>
+      <c r="AD66" s="474"/>
     </row>
     <row r="67" spans="2:30" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B67" s="521"/>
-      <c r="C67" s="522"/>
-      <c r="D67" s="522"/>
-      <c r="E67" s="522"/>
-      <c r="F67" s="523"/>
-      <c r="G67" s="530"/>
-      <c r="H67" s="531"/>
-      <c r="I67" s="531"/>
-      <c r="J67" s="532"/>
-      <c r="K67" s="530"/>
-      <c r="L67" s="531"/>
-      <c r="M67" s="531"/>
-      <c r="N67" s="532"/>
-      <c r="O67" s="508"/>
-      <c r="P67" s="509"/>
-      <c r="Q67" s="509"/>
-      <c r="R67" s="510"/>
-      <c r="S67" s="508"/>
-      <c r="T67" s="509"/>
-      <c r="U67" s="509"/>
-      <c r="V67" s="510"/>
-      <c r="W67" s="508"/>
-      <c r="X67" s="509"/>
-      <c r="Y67" s="509"/>
-      <c r="Z67" s="510"/>
-      <c r="AA67" s="508"/>
-      <c r="AB67" s="509"/>
-      <c r="AC67" s="509"/>
-      <c r="AD67" s="510"/>
+      <c r="B67" s="492"/>
+      <c r="C67" s="493"/>
+      <c r="D67" s="493"/>
+      <c r="E67" s="493"/>
+      <c r="F67" s="494"/>
+      <c r="G67" s="501"/>
+      <c r="H67" s="502"/>
+      <c r="I67" s="502"/>
+      <c r="J67" s="503"/>
+      <c r="K67" s="501"/>
+      <c r="L67" s="502"/>
+      <c r="M67" s="502"/>
+      <c r="N67" s="503"/>
+      <c r="O67" s="472"/>
+      <c r="P67" s="473"/>
+      <c r="Q67" s="473"/>
+      <c r="R67" s="474"/>
+      <c r="S67" s="472"/>
+      <c r="T67" s="473"/>
+      <c r="U67" s="473"/>
+      <c r="V67" s="474"/>
+      <c r="W67" s="472"/>
+      <c r="X67" s="473"/>
+      <c r="Y67" s="473"/>
+      <c r="Z67" s="474"/>
+      <c r="AA67" s="472"/>
+      <c r="AB67" s="473"/>
+      <c r="AC67" s="473"/>
+      <c r="AD67" s="474"/>
     </row>
     <row r="68" spans="2:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B68" s="521"/>
-      <c r="C68" s="522"/>
-      <c r="D68" s="522"/>
-      <c r="E68" s="522"/>
-      <c r="F68" s="523"/>
-      <c r="G68" s="530"/>
-      <c r="H68" s="531"/>
-      <c r="I68" s="531"/>
-      <c r="J68" s="532"/>
-      <c r="K68" s="530"/>
-      <c r="L68" s="531"/>
-      <c r="M68" s="531"/>
-      <c r="N68" s="532"/>
-      <c r="O68" s="508"/>
-      <c r="P68" s="509"/>
-      <c r="Q68" s="509"/>
-      <c r="R68" s="510"/>
-      <c r="S68" s="508"/>
-      <c r="T68" s="509"/>
-      <c r="U68" s="509"/>
-      <c r="V68" s="510"/>
-      <c r="W68" s="508"/>
-      <c r="X68" s="509"/>
-      <c r="Y68" s="509"/>
-      <c r="Z68" s="510"/>
-      <c r="AA68" s="508"/>
-      <c r="AB68" s="509"/>
-      <c r="AC68" s="509"/>
-      <c r="AD68" s="510"/>
+      <c r="B68" s="492"/>
+      <c r="C68" s="493"/>
+      <c r="D68" s="493"/>
+      <c r="E68" s="493"/>
+      <c r="F68" s="494"/>
+      <c r="G68" s="501"/>
+      <c r="H68" s="502"/>
+      <c r="I68" s="502"/>
+      <c r="J68" s="503"/>
+      <c r="K68" s="501"/>
+      <c r="L68" s="502"/>
+      <c r="M68" s="502"/>
+      <c r="N68" s="503"/>
+      <c r="O68" s="472"/>
+      <c r="P68" s="473"/>
+      <c r="Q68" s="473"/>
+      <c r="R68" s="474"/>
+      <c r="S68" s="472"/>
+      <c r="T68" s="473"/>
+      <c r="U68" s="473"/>
+      <c r="V68" s="474"/>
+      <c r="W68" s="472"/>
+      <c r="X68" s="473"/>
+      <c r="Y68" s="473"/>
+      <c r="Z68" s="474"/>
+      <c r="AA68" s="472"/>
+      <c r="AB68" s="473"/>
+      <c r="AC68" s="473"/>
+      <c r="AD68" s="474"/>
     </row>
     <row r="69" spans="2:30" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B69" s="524"/>
-      <c r="C69" s="525"/>
-      <c r="D69" s="525"/>
-      <c r="E69" s="525"/>
-      <c r="F69" s="526"/>
-      <c r="G69" s="533"/>
-      <c r="H69" s="534"/>
-      <c r="I69" s="534"/>
-      <c r="J69" s="535"/>
-      <c r="K69" s="533"/>
-      <c r="L69" s="534"/>
-      <c r="M69" s="534"/>
-      <c r="N69" s="535"/>
-      <c r="O69" s="511"/>
-      <c r="P69" s="512"/>
-      <c r="Q69" s="512"/>
-      <c r="R69" s="513"/>
-      <c r="S69" s="511"/>
-      <c r="T69" s="512"/>
-      <c r="U69" s="512"/>
-      <c r="V69" s="513"/>
-      <c r="W69" s="511"/>
-      <c r="X69" s="512"/>
-      <c r="Y69" s="512"/>
-      <c r="Z69" s="513"/>
-      <c r="AA69" s="511"/>
-      <c r="AB69" s="512"/>
-      <c r="AC69" s="512"/>
-      <c r="AD69" s="513"/>
+      <c r="B69" s="495"/>
+      <c r="C69" s="496"/>
+      <c r="D69" s="496"/>
+      <c r="E69" s="496"/>
+      <c r="F69" s="497"/>
+      <c r="G69" s="504"/>
+      <c r="H69" s="505"/>
+      <c r="I69" s="505"/>
+      <c r="J69" s="506"/>
+      <c r="K69" s="504"/>
+      <c r="L69" s="505"/>
+      <c r="M69" s="505"/>
+      <c r="N69" s="506"/>
+      <c r="O69" s="475"/>
+      <c r="P69" s="476"/>
+      <c r="Q69" s="476"/>
+      <c r="R69" s="477"/>
+      <c r="S69" s="475"/>
+      <c r="T69" s="476"/>
+      <c r="U69" s="476"/>
+      <c r="V69" s="477"/>
+      <c r="W69" s="475"/>
+      <c r="X69" s="476"/>
+      <c r="Y69" s="476"/>
+      <c r="Z69" s="477"/>
+      <c r="AA69" s="475"/>
+      <c r="AB69" s="476"/>
+      <c r="AC69" s="476"/>
+      <c r="AD69" s="477"/>
     </row>
   </sheetData>
   <mergeCells count="59">
-    <mergeCell ref="W52:Z52"/>
-    <mergeCell ref="W51:Z51"/>
-    <mergeCell ref="W53:Z69"/>
-    <mergeCell ref="AA52:AD52"/>
-    <mergeCell ref="AA51:AD51"/>
-    <mergeCell ref="AA53:AD69"/>
+    <mergeCell ref="B51:F51"/>
+    <mergeCell ref="B52:F52"/>
+    <mergeCell ref="G50:J50"/>
+    <mergeCell ref="G51:J51"/>
+    <mergeCell ref="G7:BB7"/>
+    <mergeCell ref="AQ8:AT8"/>
+    <mergeCell ref="AU8:AX8"/>
+    <mergeCell ref="AY8:BB8"/>
+    <mergeCell ref="AQ10:BB10"/>
+    <mergeCell ref="AE8:AH8"/>
+    <mergeCell ref="AI8:AL8"/>
+    <mergeCell ref="AM8:AP8"/>
+    <mergeCell ref="AE10:AP10"/>
+    <mergeCell ref="S8:V8"/>
+    <mergeCell ref="W8:Z8"/>
+    <mergeCell ref="AA8:AD8"/>
+    <mergeCell ref="S10:AD10"/>
+    <mergeCell ref="G8:J8"/>
+    <mergeCell ref="K8:N8"/>
+    <mergeCell ref="O8:R8"/>
+    <mergeCell ref="AA50:AD50"/>
+    <mergeCell ref="S50:V50"/>
+    <mergeCell ref="W50:Z50"/>
+    <mergeCell ref="AA49:AD49"/>
+    <mergeCell ref="W49:Z49"/>
+    <mergeCell ref="S49:V49"/>
+    <mergeCell ref="O49:R49"/>
+    <mergeCell ref="K49:N49"/>
+    <mergeCell ref="G52:J52"/>
+    <mergeCell ref="O51:R51"/>
+    <mergeCell ref="O50:R50"/>
+    <mergeCell ref="K50:N50"/>
+    <mergeCell ref="S51:V51"/>
+    <mergeCell ref="S52:V52"/>
+    <mergeCell ref="K51:N51"/>
+    <mergeCell ref="K52:N52"/>
+    <mergeCell ref="O52:R52"/>
     <mergeCell ref="B15:B20"/>
     <mergeCell ref="B21:B25"/>
     <mergeCell ref="B30:B33"/>
@@ -33140,43 +33171,12 @@
     <mergeCell ref="B34:B35"/>
     <mergeCell ref="B37:B38"/>
     <mergeCell ref="B50:F50"/>
-    <mergeCell ref="G52:J52"/>
-    <mergeCell ref="O51:R51"/>
-    <mergeCell ref="O50:R50"/>
-    <mergeCell ref="K50:N50"/>
-    <mergeCell ref="S51:V51"/>
-    <mergeCell ref="S52:V52"/>
-    <mergeCell ref="K51:N51"/>
-    <mergeCell ref="K52:N52"/>
-    <mergeCell ref="O52:R52"/>
-    <mergeCell ref="S10:AD10"/>
-    <mergeCell ref="G8:J8"/>
-    <mergeCell ref="K8:N8"/>
-    <mergeCell ref="O8:R8"/>
-    <mergeCell ref="AA50:AD50"/>
-    <mergeCell ref="S50:V50"/>
-    <mergeCell ref="W50:Z50"/>
-    <mergeCell ref="AA49:AD49"/>
-    <mergeCell ref="W49:Z49"/>
-    <mergeCell ref="S49:V49"/>
-    <mergeCell ref="O49:R49"/>
-    <mergeCell ref="K49:N49"/>
-    <mergeCell ref="B51:F51"/>
-    <mergeCell ref="B52:F52"/>
-    <mergeCell ref="G50:J50"/>
-    <mergeCell ref="G51:J51"/>
-    <mergeCell ref="G7:BB7"/>
-    <mergeCell ref="AQ8:AT8"/>
-    <mergeCell ref="AU8:AX8"/>
-    <mergeCell ref="AY8:BB8"/>
-    <mergeCell ref="AQ10:BB10"/>
-    <mergeCell ref="AE8:AH8"/>
-    <mergeCell ref="AI8:AL8"/>
-    <mergeCell ref="AM8:AP8"/>
-    <mergeCell ref="AE10:AP10"/>
-    <mergeCell ref="S8:V8"/>
-    <mergeCell ref="W8:Z8"/>
-    <mergeCell ref="AA8:AD8"/>
+    <mergeCell ref="W52:Z52"/>
+    <mergeCell ref="W51:Z51"/>
+    <mergeCell ref="W53:Z69"/>
+    <mergeCell ref="AA52:AD52"/>
+    <mergeCell ref="AA51:AD51"/>
+    <mergeCell ref="AA53:AD69"/>
   </mergeCells>
   <phoneticPr fontId="15" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -33337,24 +33337,24 @@
       <c r="D7" s="40"/>
       <c r="E7" s="40"/>
       <c r="F7" s="40"/>
-      <c r="G7" s="545" t="s">
+      <c r="G7" s="546" t="s">
         <v>74</v>
       </c>
-      <c r="H7" s="546"/>
-      <c r="I7" s="546"/>
-      <c r="J7" s="547"/>
-      <c r="K7" s="542" t="s">
+      <c r="H7" s="547"/>
+      <c r="I7" s="547"/>
+      <c r="J7" s="548"/>
+      <c r="K7" s="543" t="s">
         <v>75</v>
       </c>
-      <c r="L7" s="543"/>
-      <c r="M7" s="543"/>
-      <c r="N7" s="544"/>
-      <c r="O7" s="539" t="s">
+      <c r="L7" s="544"/>
+      <c r="M7" s="544"/>
+      <c r="N7" s="545"/>
+      <c r="O7" s="540" t="s">
         <v>76</v>
       </c>
-      <c r="P7" s="540"/>
-      <c r="Q7" s="540"/>
-      <c r="R7" s="541"/>
+      <c r="P7" s="541"/>
+      <c r="Q7" s="541"/>
+      <c r="R7" s="542"/>
     </row>
     <row r="8" spans="2:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B8" s="167"/>
@@ -33547,7 +33547,7 @@
       <c r="R13" s="224"/>
     </row>
     <row r="14" spans="2:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="552" t="s">
+      <c r="B14" s="553" t="s">
         <v>159</v>
       </c>
       <c r="C14" s="146" t="s">
@@ -33576,7 +33576,7 @@
       <c r="R14" s="266"/>
     </row>
     <row r="15" spans="2:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="553"/>
+      <c r="B15" s="554"/>
       <c r="C15" s="228" t="s">
         <v>93</v>
       </c>
@@ -33603,7 +33603,7 @@
       <c r="R15" s="267"/>
     </row>
     <row r="16" spans="2:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="552" t="s">
+      <c r="B16" s="553" t="s">
         <v>160</v>
       </c>
       <c r="C16" s="263" t="s">
@@ -33632,7 +33632,7 @@
       <c r="R16" s="264"/>
     </row>
     <row r="17" spans="2:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="554"/>
+      <c r="B17" s="555"/>
       <c r="C17" s="296" t="s">
         <v>27</v>
       </c>
@@ -33663,7 +33663,7 @@
       <c r="R17" s="271"/>
     </row>
     <row r="18" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B18" s="555" t="s">
+      <c r="B18" s="556" t="s">
         <v>161</v>
       </c>
       <c r="C18" s="122" t="s">
@@ -33692,7 +33692,7 @@
       <c r="R18" s="266"/>
     </row>
     <row r="19" spans="2:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="556"/>
+      <c r="B19" s="557"/>
       <c r="C19" s="123" t="s">
         <v>38</v>
       </c>
@@ -33721,7 +33721,7 @@
       <c r="R19" s="266"/>
     </row>
     <row r="20" spans="2:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="555" t="s">
+      <c r="B20" s="556" t="s">
         <v>162</v>
       </c>
       <c r="C20" s="119" t="s">
@@ -33750,7 +33750,7 @@
       <c r="R20" s="264"/>
     </row>
     <row r="21" spans="2:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="556"/>
+      <c r="B21" s="557"/>
       <c r="C21" s="284" t="s">
         <v>44</v>
       </c>
@@ -33808,7 +33808,7 @@
       <c r="R22" s="266"/>
     </row>
     <row r="23" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B23" s="557" t="s">
+      <c r="B23" s="558" t="s">
         <v>115</v>
       </c>
       <c r="C23" s="119" t="s">
@@ -33837,7 +33837,7 @@
       <c r="R23" s="264"/>
     </row>
     <row r="24" spans="2:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="558"/>
+      <c r="B24" s="559"/>
       <c r="C24" s="124" t="s">
         <v>20</v>
       </c>
@@ -33864,7 +33864,7 @@
       <c r="R24" s="281"/>
     </row>
     <row r="25" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B25" s="552" t="s">
+      <c r="B25" s="553" t="s">
         <v>163</v>
       </c>
       <c r="C25" s="119" t="s">
@@ -33893,7 +33893,7 @@
       <c r="R25" s="23"/>
     </row>
     <row r="26" spans="2:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="553"/>
+      <c r="B26" s="554"/>
       <c r="C26" s="124" t="s">
         <v>113</v>
       </c>
@@ -34007,455 +34007,442 @@
       <c r="R29" s="312"/>
     </row>
     <row r="30" spans="2:18" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B30" s="515" t="s">
+      <c r="B30" s="486" t="s">
         <v>131</v>
       </c>
-      <c r="C30" s="516"/>
-      <c r="D30" s="516"/>
-      <c r="E30" s="516"/>
-      <c r="F30" s="516"/>
-      <c r="G30" s="515" t="s">
+      <c r="C30" s="487"/>
+      <c r="D30" s="487"/>
+      <c r="E30" s="487"/>
+      <c r="F30" s="487"/>
+      <c r="G30" s="486" t="s">
         <v>134</v>
       </c>
-      <c r="H30" s="516"/>
-      <c r="I30" s="516"/>
-      <c r="J30" s="551"/>
-      <c r="K30" s="491" t="s">
+      <c r="H30" s="487"/>
+      <c r="I30" s="487"/>
+      <c r="J30" s="552"/>
+      <c r="K30" s="482" t="s">
         <v>135</v>
       </c>
-      <c r="L30" s="492"/>
-      <c r="M30" s="492"/>
-      <c r="N30" s="493"/>
-      <c r="O30" s="491"/>
-      <c r="P30" s="492"/>
-      <c r="Q30" s="492"/>
-      <c r="R30" s="493"/>
+      <c r="L30" s="483"/>
+      <c r="M30" s="483"/>
+      <c r="N30" s="484"/>
+      <c r="O30" s="482"/>
+      <c r="P30" s="483"/>
+      <c r="Q30" s="483"/>
+      <c r="R30" s="484"/>
     </row>
     <row r="31" spans="2:18" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B31" s="488" t="s">
+      <c r="B31" s="508" t="s">
         <v>137</v>
       </c>
-      <c r="C31" s="489"/>
-      <c r="D31" s="489"/>
-      <c r="E31" s="489"/>
-      <c r="F31" s="489"/>
-      <c r="G31" s="488" t="s">
+      <c r="C31" s="509"/>
+      <c r="D31" s="509"/>
+      <c r="E31" s="509"/>
+      <c r="F31" s="509"/>
+      <c r="G31" s="508" t="s">
         <v>139</v>
       </c>
-      <c r="H31" s="489"/>
-      <c r="I31" s="489"/>
-      <c r="J31" s="559"/>
-      <c r="K31" s="488" t="s">
+      <c r="H31" s="509"/>
+      <c r="I31" s="509"/>
+      <c r="J31" s="539"/>
+      <c r="K31" s="508" t="s">
         <v>138</v>
       </c>
-      <c r="L31" s="489"/>
-      <c r="M31" s="489"/>
-      <c r="N31" s="559"/>
-      <c r="O31" s="488" t="s">
+      <c r="L31" s="509"/>
+      <c r="M31" s="509"/>
+      <c r="N31" s="539"/>
+      <c r="O31" s="508" t="s">
         <v>138</v>
       </c>
-      <c r="P31" s="489"/>
-      <c r="Q31" s="489"/>
-      <c r="R31" s="559"/>
+      <c r="P31" s="509"/>
+      <c r="Q31" s="509"/>
+      <c r="R31" s="539"/>
     </row>
     <row r="32" spans="2:18" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B32" s="463" t="s">
+      <c r="B32" s="466" t="s">
         <v>140</v>
       </c>
-      <c r="C32" s="464"/>
-      <c r="D32" s="464"/>
-      <c r="E32" s="464"/>
-      <c r="F32" s="464"/>
-      <c r="G32" s="463" t="s">
+      <c r="C32" s="467"/>
+      <c r="D32" s="467"/>
+      <c r="E32" s="467"/>
+      <c r="F32" s="467"/>
+      <c r="G32" s="466" t="s">
         <v>143</v>
       </c>
-      <c r="H32" s="464"/>
-      <c r="I32" s="464"/>
-      <c r="J32" s="538"/>
-      <c r="K32" s="463" t="s">
+      <c r="H32" s="467"/>
+      <c r="I32" s="467"/>
+      <c r="J32" s="479"/>
+      <c r="K32" s="466" t="s">
         <v>142</v>
       </c>
-      <c r="L32" s="464"/>
-      <c r="M32" s="464"/>
-      <c r="N32" s="538"/>
-      <c r="O32" s="463" t="s">
+      <c r="L32" s="467"/>
+      <c r="M32" s="467"/>
+      <c r="N32" s="479"/>
+      <c r="O32" s="466" t="s">
         <v>142</v>
       </c>
-      <c r="P32" s="464"/>
-      <c r="Q32" s="464"/>
-      <c r="R32" s="538"/>
+      <c r="P32" s="467"/>
+      <c r="Q32" s="467"/>
+      <c r="R32" s="479"/>
     </row>
     <row r="33" spans="2:18" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B33" s="548" t="s">
+      <c r="B33" s="549" t="s">
         <v>144</v>
       </c>
-      <c r="C33" s="549"/>
-      <c r="D33" s="549"/>
-      <c r="E33" s="549"/>
-      <c r="F33" s="550"/>
-      <c r="G33" s="466" t="s">
+      <c r="C33" s="550"/>
+      <c r="D33" s="550"/>
+      <c r="E33" s="550"/>
+      <c r="F33" s="551"/>
+      <c r="G33" s="463" t="s">
         <v>147</v>
       </c>
-      <c r="H33" s="467"/>
-      <c r="I33" s="467"/>
-      <c r="J33" s="537"/>
-      <c r="K33" s="466" t="s">
+      <c r="H33" s="464"/>
+      <c r="I33" s="464"/>
+      <c r="J33" s="478"/>
+      <c r="K33" s="463" t="s">
         <v>165</v>
       </c>
-      <c r="L33" s="467"/>
-      <c r="M33" s="467"/>
-      <c r="N33" s="537"/>
-      <c r="O33" s="466"/>
-      <c r="P33" s="467"/>
-      <c r="Q33" s="467"/>
-      <c r="R33" s="537"/>
+      <c r="L33" s="464"/>
+      <c r="M33" s="464"/>
+      <c r="N33" s="478"/>
+      <c r="O33" s="463"/>
+      <c r="P33" s="464"/>
+      <c r="Q33" s="464"/>
+      <c r="R33" s="478"/>
     </row>
     <row r="34" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B34" s="518" t="s">
+      <c r="B34" s="489" t="s">
         <v>148</v>
       </c>
-      <c r="C34" s="519"/>
-      <c r="D34" s="519"/>
-      <c r="E34" s="519"/>
-      <c r="F34" s="520"/>
-      <c r="G34" s="505" t="s">
+      <c r="C34" s="490"/>
+      <c r="D34" s="490"/>
+      <c r="E34" s="490"/>
+      <c r="F34" s="491"/>
+      <c r="G34" s="469" t="s">
         <v>151</v>
       </c>
-      <c r="H34" s="506"/>
-      <c r="I34" s="506"/>
-      <c r="J34" s="507"/>
-      <c r="K34" s="505" t="s">
+      <c r="H34" s="470"/>
+      <c r="I34" s="470"/>
+      <c r="J34" s="471"/>
+      <c r="K34" s="469" t="s">
         <v>152</v>
       </c>
-      <c r="L34" s="506"/>
-      <c r="M34" s="506"/>
-      <c r="N34" s="507"/>
-      <c r="O34" s="505" t="s">
+      <c r="L34" s="470"/>
+      <c r="M34" s="470"/>
+      <c r="N34" s="471"/>
+      <c r="O34" s="469" t="s">
         <v>166</v>
       </c>
-      <c r="P34" s="506"/>
-      <c r="Q34" s="506"/>
-      <c r="R34" s="507"/>
+      <c r="P34" s="470"/>
+      <c r="Q34" s="470"/>
+      <c r="R34" s="471"/>
     </row>
     <row r="35" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B35" s="521"/>
-      <c r="C35" s="522"/>
-      <c r="D35" s="522"/>
-      <c r="E35" s="522"/>
-      <c r="F35" s="523"/>
-      <c r="G35" s="508"/>
-      <c r="H35" s="509"/>
-      <c r="I35" s="509"/>
-      <c r="J35" s="510"/>
-      <c r="K35" s="508"/>
-      <c r="L35" s="509"/>
-      <c r="M35" s="509"/>
-      <c r="N35" s="510"/>
-      <c r="O35" s="508"/>
-      <c r="P35" s="509"/>
-      <c r="Q35" s="509"/>
-      <c r="R35" s="510"/>
+      <c r="B35" s="492"/>
+      <c r="C35" s="493"/>
+      <c r="D35" s="493"/>
+      <c r="E35" s="493"/>
+      <c r="F35" s="494"/>
+      <c r="G35" s="472"/>
+      <c r="H35" s="473"/>
+      <c r="I35" s="473"/>
+      <c r="J35" s="474"/>
+      <c r="K35" s="472"/>
+      <c r="L35" s="473"/>
+      <c r="M35" s="473"/>
+      <c r="N35" s="474"/>
+      <c r="O35" s="472"/>
+      <c r="P35" s="473"/>
+      <c r="Q35" s="473"/>
+      <c r="R35" s="474"/>
     </row>
     <row r="36" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B36" s="521"/>
-      <c r="C36" s="522"/>
-      <c r="D36" s="522"/>
-      <c r="E36" s="522"/>
-      <c r="F36" s="523"/>
-      <c r="G36" s="508"/>
-      <c r="H36" s="509"/>
-      <c r="I36" s="509"/>
-      <c r="J36" s="510"/>
-      <c r="K36" s="508"/>
-      <c r="L36" s="509"/>
-      <c r="M36" s="509"/>
-      <c r="N36" s="510"/>
-      <c r="O36" s="508"/>
-      <c r="P36" s="509"/>
-      <c r="Q36" s="509"/>
-      <c r="R36" s="510"/>
+      <c r="B36" s="492"/>
+      <c r="C36" s="493"/>
+      <c r="D36" s="493"/>
+      <c r="E36" s="493"/>
+      <c r="F36" s="494"/>
+      <c r="G36" s="472"/>
+      <c r="H36" s="473"/>
+      <c r="I36" s="473"/>
+      <c r="J36" s="474"/>
+      <c r="K36" s="472"/>
+      <c r="L36" s="473"/>
+      <c r="M36" s="473"/>
+      <c r="N36" s="474"/>
+      <c r="O36" s="472"/>
+      <c r="P36" s="473"/>
+      <c r="Q36" s="473"/>
+      <c r="R36" s="474"/>
     </row>
     <row r="37" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B37" s="521"/>
-      <c r="C37" s="522"/>
-      <c r="D37" s="522"/>
-      <c r="E37" s="522"/>
-      <c r="F37" s="523"/>
-      <c r="G37" s="508"/>
-      <c r="H37" s="509"/>
-      <c r="I37" s="509"/>
-      <c r="J37" s="510"/>
-      <c r="K37" s="508"/>
-      <c r="L37" s="509"/>
-      <c r="M37" s="509"/>
-      <c r="N37" s="510"/>
-      <c r="O37" s="508"/>
-      <c r="P37" s="509"/>
-      <c r="Q37" s="509"/>
-      <c r="R37" s="510"/>
+      <c r="B37" s="492"/>
+      <c r="C37" s="493"/>
+      <c r="D37" s="493"/>
+      <c r="E37" s="493"/>
+      <c r="F37" s="494"/>
+      <c r="G37" s="472"/>
+      <c r="H37" s="473"/>
+      <c r="I37" s="473"/>
+      <c r="J37" s="474"/>
+      <c r="K37" s="472"/>
+      <c r="L37" s="473"/>
+      <c r="M37" s="473"/>
+      <c r="N37" s="474"/>
+      <c r="O37" s="472"/>
+      <c r="P37" s="473"/>
+      <c r="Q37" s="473"/>
+      <c r="R37" s="474"/>
     </row>
     <row r="38" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B38" s="521"/>
-      <c r="C38" s="522"/>
-      <c r="D38" s="522"/>
-      <c r="E38" s="522"/>
-      <c r="F38" s="523"/>
-      <c r="G38" s="508"/>
-      <c r="H38" s="509"/>
-      <c r="I38" s="509"/>
-      <c r="J38" s="510"/>
-      <c r="K38" s="508"/>
-      <c r="L38" s="509"/>
-      <c r="M38" s="509"/>
-      <c r="N38" s="510"/>
-      <c r="O38" s="508"/>
-      <c r="P38" s="509"/>
-      <c r="Q38" s="509"/>
-      <c r="R38" s="510"/>
+      <c r="B38" s="492"/>
+      <c r="C38" s="493"/>
+      <c r="D38" s="493"/>
+      <c r="E38" s="493"/>
+      <c r="F38" s="494"/>
+      <c r="G38" s="472"/>
+      <c r="H38" s="473"/>
+      <c r="I38" s="473"/>
+      <c r="J38" s="474"/>
+      <c r="K38" s="472"/>
+      <c r="L38" s="473"/>
+      <c r="M38" s="473"/>
+      <c r="N38" s="474"/>
+      <c r="O38" s="472"/>
+      <c r="P38" s="473"/>
+      <c r="Q38" s="473"/>
+      <c r="R38" s="474"/>
     </row>
     <row r="39" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B39" s="521"/>
-      <c r="C39" s="522"/>
-      <c r="D39" s="522"/>
-      <c r="E39" s="522"/>
-      <c r="F39" s="523"/>
-      <c r="G39" s="508"/>
-      <c r="H39" s="509"/>
-      <c r="I39" s="509"/>
-      <c r="J39" s="510"/>
-      <c r="K39" s="508"/>
-      <c r="L39" s="509"/>
-      <c r="M39" s="509"/>
-      <c r="N39" s="510"/>
-      <c r="O39" s="508"/>
-      <c r="P39" s="509"/>
-      <c r="Q39" s="509"/>
-      <c r="R39" s="510"/>
+      <c r="B39" s="492"/>
+      <c r="C39" s="493"/>
+      <c r="D39" s="493"/>
+      <c r="E39" s="493"/>
+      <c r="F39" s="494"/>
+      <c r="G39" s="472"/>
+      <c r="H39" s="473"/>
+      <c r="I39" s="473"/>
+      <c r="J39" s="474"/>
+      <c r="K39" s="472"/>
+      <c r="L39" s="473"/>
+      <c r="M39" s="473"/>
+      <c r="N39" s="474"/>
+      <c r="O39" s="472"/>
+      <c r="P39" s="473"/>
+      <c r="Q39" s="473"/>
+      <c r="R39" s="474"/>
     </row>
     <row r="40" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B40" s="521"/>
-      <c r="C40" s="522"/>
-      <c r="D40" s="522"/>
-      <c r="E40" s="522"/>
-      <c r="F40" s="523"/>
-      <c r="G40" s="508"/>
-      <c r="H40" s="509"/>
-      <c r="I40" s="509"/>
-      <c r="J40" s="510"/>
-      <c r="K40" s="508"/>
-      <c r="L40" s="509"/>
-      <c r="M40" s="509"/>
-      <c r="N40" s="510"/>
-      <c r="O40" s="508"/>
-      <c r="P40" s="509"/>
-      <c r="Q40" s="509"/>
-      <c r="R40" s="510"/>
+      <c r="B40" s="492"/>
+      <c r="C40" s="493"/>
+      <c r="D40" s="493"/>
+      <c r="E40" s="493"/>
+      <c r="F40" s="494"/>
+      <c r="G40" s="472"/>
+      <c r="H40" s="473"/>
+      <c r="I40" s="473"/>
+      <c r="J40" s="474"/>
+      <c r="K40" s="472"/>
+      <c r="L40" s="473"/>
+      <c r="M40" s="473"/>
+      <c r="N40" s="474"/>
+      <c r="O40" s="472"/>
+      <c r="P40" s="473"/>
+      <c r="Q40" s="473"/>
+      <c r="R40" s="474"/>
     </row>
     <row r="41" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B41" s="521"/>
-      <c r="C41" s="522"/>
-      <c r="D41" s="522"/>
-      <c r="E41" s="522"/>
-      <c r="F41" s="523"/>
-      <c r="G41" s="508"/>
-      <c r="H41" s="509"/>
-      <c r="I41" s="509"/>
-      <c r="J41" s="510"/>
-      <c r="K41" s="508"/>
-      <c r="L41" s="509"/>
-      <c r="M41" s="509"/>
-      <c r="N41" s="510"/>
-      <c r="O41" s="508"/>
-      <c r="P41" s="509"/>
-      <c r="Q41" s="509"/>
-      <c r="R41" s="510"/>
+      <c r="B41" s="492"/>
+      <c r="C41" s="493"/>
+      <c r="D41" s="493"/>
+      <c r="E41" s="493"/>
+      <c r="F41" s="494"/>
+      <c r="G41" s="472"/>
+      <c r="H41" s="473"/>
+      <c r="I41" s="473"/>
+      <c r="J41" s="474"/>
+      <c r="K41" s="472"/>
+      <c r="L41" s="473"/>
+      <c r="M41" s="473"/>
+      <c r="N41" s="474"/>
+      <c r="O41" s="472"/>
+      <c r="P41" s="473"/>
+      <c r="Q41" s="473"/>
+      <c r="R41" s="474"/>
     </row>
     <row r="42" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B42" s="521"/>
-      <c r="C42" s="522"/>
-      <c r="D42" s="522"/>
-      <c r="E42" s="522"/>
-      <c r="F42" s="523"/>
-      <c r="G42" s="508"/>
-      <c r="H42" s="509"/>
-      <c r="I42" s="509"/>
-      <c r="J42" s="510"/>
-      <c r="K42" s="508"/>
-      <c r="L42" s="509"/>
-      <c r="M42" s="509"/>
-      <c r="N42" s="510"/>
-      <c r="O42" s="508"/>
-      <c r="P42" s="509"/>
-      <c r="Q42" s="509"/>
-      <c r="R42" s="510"/>
+      <c r="B42" s="492"/>
+      <c r="C42" s="493"/>
+      <c r="D42" s="493"/>
+      <c r="E42" s="493"/>
+      <c r="F42" s="494"/>
+      <c r="G42" s="472"/>
+      <c r="H42" s="473"/>
+      <c r="I42" s="473"/>
+      <c r="J42" s="474"/>
+      <c r="K42" s="472"/>
+      <c r="L42" s="473"/>
+      <c r="M42" s="473"/>
+      <c r="N42" s="474"/>
+      <c r="O42" s="472"/>
+      <c r="P42" s="473"/>
+      <c r="Q42" s="473"/>
+      <c r="R42" s="474"/>
     </row>
     <row r="43" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B43" s="521"/>
-      <c r="C43" s="522"/>
-      <c r="D43" s="522"/>
-      <c r="E43" s="522"/>
-      <c r="F43" s="523"/>
-      <c r="G43" s="508"/>
-      <c r="H43" s="509"/>
-      <c r="I43" s="509"/>
-      <c r="J43" s="510"/>
-      <c r="K43" s="508"/>
-      <c r="L43" s="509"/>
-      <c r="M43" s="509"/>
-      <c r="N43" s="510"/>
-      <c r="O43" s="508"/>
-      <c r="P43" s="509"/>
-      <c r="Q43" s="509"/>
-      <c r="R43" s="510"/>
+      <c r="B43" s="492"/>
+      <c r="C43" s="493"/>
+      <c r="D43" s="493"/>
+      <c r="E43" s="493"/>
+      <c r="F43" s="494"/>
+      <c r="G43" s="472"/>
+      <c r="H43" s="473"/>
+      <c r="I43" s="473"/>
+      <c r="J43" s="474"/>
+      <c r="K43" s="472"/>
+      <c r="L43" s="473"/>
+      <c r="M43" s="473"/>
+      <c r="N43" s="474"/>
+      <c r="O43" s="472"/>
+      <c r="P43" s="473"/>
+      <c r="Q43" s="473"/>
+      <c r="R43" s="474"/>
     </row>
     <row r="44" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B44" s="521"/>
-      <c r="C44" s="522"/>
-      <c r="D44" s="522"/>
-      <c r="E44" s="522"/>
-      <c r="F44" s="523"/>
-      <c r="G44" s="508"/>
-      <c r="H44" s="509"/>
-      <c r="I44" s="509"/>
-      <c r="J44" s="510"/>
-      <c r="K44" s="508"/>
-      <c r="L44" s="509"/>
-      <c r="M44" s="509"/>
-      <c r="N44" s="510"/>
-      <c r="O44" s="508"/>
-      <c r="P44" s="509"/>
-      <c r="Q44" s="509"/>
-      <c r="R44" s="510"/>
+      <c r="B44" s="492"/>
+      <c r="C44" s="493"/>
+      <c r="D44" s="493"/>
+      <c r="E44" s="493"/>
+      <c r="F44" s="494"/>
+      <c r="G44" s="472"/>
+      <c r="H44" s="473"/>
+      <c r="I44" s="473"/>
+      <c r="J44" s="474"/>
+      <c r="K44" s="472"/>
+      <c r="L44" s="473"/>
+      <c r="M44" s="473"/>
+      <c r="N44" s="474"/>
+      <c r="O44" s="472"/>
+      <c r="P44" s="473"/>
+      <c r="Q44" s="473"/>
+      <c r="R44" s="474"/>
     </row>
     <row r="45" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B45" s="521"/>
-      <c r="C45" s="522"/>
-      <c r="D45" s="522"/>
-      <c r="E45" s="522"/>
-      <c r="F45" s="523"/>
-      <c r="G45" s="508"/>
-      <c r="H45" s="509"/>
-      <c r="I45" s="509"/>
-      <c r="J45" s="510"/>
-      <c r="K45" s="508"/>
-      <c r="L45" s="509"/>
-      <c r="M45" s="509"/>
-      <c r="N45" s="510"/>
-      <c r="O45" s="508"/>
-      <c r="P45" s="509"/>
-      <c r="Q45" s="509"/>
-      <c r="R45" s="510"/>
+      <c r="B45" s="492"/>
+      <c r="C45" s="493"/>
+      <c r="D45" s="493"/>
+      <c r="E45" s="493"/>
+      <c r="F45" s="494"/>
+      <c r="G45" s="472"/>
+      <c r="H45" s="473"/>
+      <c r="I45" s="473"/>
+      <c r="J45" s="474"/>
+      <c r="K45" s="472"/>
+      <c r="L45" s="473"/>
+      <c r="M45" s="473"/>
+      <c r="N45" s="474"/>
+      <c r="O45" s="472"/>
+      <c r="P45" s="473"/>
+      <c r="Q45" s="473"/>
+      <c r="R45" s="474"/>
     </row>
     <row r="46" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B46" s="521"/>
-      <c r="C46" s="522"/>
-      <c r="D46" s="522"/>
-      <c r="E46" s="522"/>
-      <c r="F46" s="523"/>
-      <c r="G46" s="508"/>
-      <c r="H46" s="509"/>
-      <c r="I46" s="509"/>
-      <c r="J46" s="510"/>
-      <c r="K46" s="508"/>
-      <c r="L46" s="509"/>
-      <c r="M46" s="509"/>
-      <c r="N46" s="510"/>
-      <c r="O46" s="508"/>
-      <c r="P46" s="509"/>
-      <c r="Q46" s="509"/>
-      <c r="R46" s="510"/>
+      <c r="B46" s="492"/>
+      <c r="C46" s="493"/>
+      <c r="D46" s="493"/>
+      <c r="E46" s="493"/>
+      <c r="F46" s="494"/>
+      <c r="G46" s="472"/>
+      <c r="H46" s="473"/>
+      <c r="I46" s="473"/>
+      <c r="J46" s="474"/>
+      <c r="K46" s="472"/>
+      <c r="L46" s="473"/>
+      <c r="M46" s="473"/>
+      <c r="N46" s="474"/>
+      <c r="O46" s="472"/>
+      <c r="P46" s="473"/>
+      <c r="Q46" s="473"/>
+      <c r="R46" s="474"/>
     </row>
     <row r="47" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B47" s="521"/>
-      <c r="C47" s="522"/>
-      <c r="D47" s="522"/>
-      <c r="E47" s="522"/>
-      <c r="F47" s="523"/>
-      <c r="G47" s="508"/>
-      <c r="H47" s="509"/>
-      <c r="I47" s="509"/>
-      <c r="J47" s="510"/>
-      <c r="K47" s="508"/>
-      <c r="L47" s="509"/>
-      <c r="M47" s="509"/>
-      <c r="N47" s="510"/>
-      <c r="O47" s="508"/>
-      <c r="P47" s="509"/>
-      <c r="Q47" s="509"/>
-      <c r="R47" s="510"/>
+      <c r="B47" s="492"/>
+      <c r="C47" s="493"/>
+      <c r="D47" s="493"/>
+      <c r="E47" s="493"/>
+      <c r="F47" s="494"/>
+      <c r="G47" s="472"/>
+      <c r="H47" s="473"/>
+      <c r="I47" s="473"/>
+      <c r="J47" s="474"/>
+      <c r="K47" s="472"/>
+      <c r="L47" s="473"/>
+      <c r="M47" s="473"/>
+      <c r="N47" s="474"/>
+      <c r="O47" s="472"/>
+      <c r="P47" s="473"/>
+      <c r="Q47" s="473"/>
+      <c r="R47" s="474"/>
     </row>
     <row r="48" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B48" s="521"/>
-      <c r="C48" s="522"/>
-      <c r="D48" s="522"/>
-      <c r="E48" s="522"/>
-      <c r="F48" s="523"/>
-      <c r="G48" s="508"/>
-      <c r="H48" s="509"/>
-      <c r="I48" s="509"/>
-      <c r="J48" s="510"/>
-      <c r="K48" s="508"/>
-      <c r="L48" s="509"/>
-      <c r="M48" s="509"/>
-      <c r="N48" s="510"/>
-      <c r="O48" s="508"/>
-      <c r="P48" s="509"/>
-      <c r="Q48" s="509"/>
-      <c r="R48" s="510"/>
+      <c r="B48" s="492"/>
+      <c r="C48" s="493"/>
+      <c r="D48" s="493"/>
+      <c r="E48" s="493"/>
+      <c r="F48" s="494"/>
+      <c r="G48" s="472"/>
+      <c r="H48" s="473"/>
+      <c r="I48" s="473"/>
+      <c r="J48" s="474"/>
+      <c r="K48" s="472"/>
+      <c r="L48" s="473"/>
+      <c r="M48" s="473"/>
+      <c r="N48" s="474"/>
+      <c r="O48" s="472"/>
+      <c r="P48" s="473"/>
+      <c r="Q48" s="473"/>
+      <c r="R48" s="474"/>
     </row>
     <row r="49" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B49" s="521"/>
-      <c r="C49" s="522"/>
-      <c r="D49" s="522"/>
-      <c r="E49" s="522"/>
-      <c r="F49" s="523"/>
-      <c r="G49" s="508"/>
-      <c r="H49" s="509"/>
-      <c r="I49" s="509"/>
-      <c r="J49" s="510"/>
-      <c r="K49" s="508"/>
-      <c r="L49" s="509"/>
-      <c r="M49" s="509"/>
-      <c r="N49" s="510"/>
-      <c r="O49" s="508"/>
-      <c r="P49" s="509"/>
-      <c r="Q49" s="509"/>
-      <c r="R49" s="510"/>
+      <c r="B49" s="492"/>
+      <c r="C49" s="493"/>
+      <c r="D49" s="493"/>
+      <c r="E49" s="493"/>
+      <c r="F49" s="494"/>
+      <c r="G49" s="472"/>
+      <c r="H49" s="473"/>
+      <c r="I49" s="473"/>
+      <c r="J49" s="474"/>
+      <c r="K49" s="472"/>
+      <c r="L49" s="473"/>
+      <c r="M49" s="473"/>
+      <c r="N49" s="474"/>
+      <c r="O49" s="472"/>
+      <c r="P49" s="473"/>
+      <c r="Q49" s="473"/>
+      <c r="R49" s="474"/>
     </row>
     <row r="50" spans="2:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B50" s="524"/>
-      <c r="C50" s="525"/>
-      <c r="D50" s="525"/>
-      <c r="E50" s="525"/>
-      <c r="F50" s="526"/>
-      <c r="G50" s="511"/>
-      <c r="H50" s="512"/>
-      <c r="I50" s="512"/>
-      <c r="J50" s="513"/>
-      <c r="K50" s="511"/>
-      <c r="L50" s="512"/>
-      <c r="M50" s="512"/>
-      <c r="N50" s="513"/>
-      <c r="O50" s="511"/>
-      <c r="P50" s="512"/>
-      <c r="Q50" s="512"/>
-      <c r="R50" s="513"/>
+      <c r="B50" s="495"/>
+      <c r="C50" s="496"/>
+      <c r="D50" s="496"/>
+      <c r="E50" s="496"/>
+      <c r="F50" s="497"/>
+      <c r="G50" s="475"/>
+      <c r="H50" s="476"/>
+      <c r="I50" s="476"/>
+      <c r="J50" s="477"/>
+      <c r="K50" s="475"/>
+      <c r="L50" s="476"/>
+      <c r="M50" s="476"/>
+      <c r="N50" s="477"/>
+      <c r="O50" s="475"/>
+      <c r="P50" s="476"/>
+      <c r="Q50" s="476"/>
+      <c r="R50" s="477"/>
     </row>
   </sheetData>
   <mergeCells count="29">
-    <mergeCell ref="K33:N33"/>
-    <mergeCell ref="O33:R33"/>
-    <mergeCell ref="G34:J50"/>
-    <mergeCell ref="K34:N50"/>
-    <mergeCell ref="O34:R50"/>
-    <mergeCell ref="B30:F30"/>
-    <mergeCell ref="B31:F31"/>
-    <mergeCell ref="B32:F32"/>
-    <mergeCell ref="K30:N30"/>
-    <mergeCell ref="O30:R30"/>
-    <mergeCell ref="G31:J31"/>
-    <mergeCell ref="K31:N31"/>
-    <mergeCell ref="O31:R31"/>
     <mergeCell ref="O7:R7"/>
     <mergeCell ref="K7:N7"/>
     <mergeCell ref="G7:J7"/>
@@ -34472,6 +34459,19 @@
     <mergeCell ref="G32:J32"/>
     <mergeCell ref="K32:N32"/>
     <mergeCell ref="O32:R32"/>
+    <mergeCell ref="B30:F30"/>
+    <mergeCell ref="B31:F31"/>
+    <mergeCell ref="B32:F32"/>
+    <mergeCell ref="K30:N30"/>
+    <mergeCell ref="O30:R30"/>
+    <mergeCell ref="G31:J31"/>
+    <mergeCell ref="K31:N31"/>
+    <mergeCell ref="O31:R31"/>
+    <mergeCell ref="K33:N33"/>
+    <mergeCell ref="O33:R33"/>
+    <mergeCell ref="G34:J50"/>
+    <mergeCell ref="K34:N50"/>
+    <mergeCell ref="O34:R50"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -39333,21 +39333,21 @@
         <v>400</v>
       </c>
       <c r="E136" s="239">
-        <v>46184</v>
+        <v>46186</v>
       </c>
       <c r="F136" s="188">
-        <v>46188.739583333336</v>
+        <v>46190.197916666664</v>
       </c>
       <c r="G136" s="188">
         <f t="shared" si="13"/>
-        <v>46190.239583333336</v>
+        <v>46191.697916666664</v>
       </c>
       <c r="H136" s="189">
         <v>36</v>
       </c>
       <c r="I136" s="188">
         <f t="shared" si="8"/>
-        <v>46190.90625</v>
+        <v>46192.364583333328</v>
       </c>
       <c r="J136" s="190">
         <v>16</v>
@@ -39367,21 +39367,21 @@
         <v>401</v>
       </c>
       <c r="E137" s="54">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="F137" s="180">
-        <v>46189.34375</v>
+        <v>46190.802083333336</v>
       </c>
       <c r="G137" s="180">
         <f t="shared" si="13"/>
-        <v>46190.34375</v>
+        <v>46191.802083333336</v>
       </c>
       <c r="H137" s="32">
         <v>24</v>
       </c>
       <c r="I137" s="180">
         <f t="shared" si="8"/>
-        <v>46191.010416666664</v>
+        <v>46192.46875</v>
       </c>
       <c r="J137" s="126">
         <v>16</v>
@@ -39401,21 +39401,21 @@
         <v>402</v>
       </c>
       <c r="E138" s="393">
-        <v>46190</v>
+        <v>46192</v>
       </c>
       <c r="F138" s="394">
-        <v>46192.697916666664</v>
+        <v>46194.15625</v>
       </c>
       <c r="G138" s="394">
         <f t="shared" si="13"/>
-        <v>46194.197916666664</v>
+        <v>46195.65625</v>
       </c>
       <c r="H138" s="391">
         <v>36</v>
       </c>
       <c r="I138" s="394">
         <f t="shared" si="8"/>
-        <v>46194.864583333328</v>
+        <v>46196.322916666664</v>
       </c>
       <c r="J138" s="126">
         <v>16</v>
@@ -39435,21 +39435,21 @@
         <v>403</v>
       </c>
       <c r="E139" s="54">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="F139" s="180">
-        <v>46194.09375</v>
+        <v>46195.552083333336</v>
       </c>
       <c r="G139" s="180">
         <f t="shared" si="13"/>
-        <v>46196.09375</v>
+        <v>46197.552083333336</v>
       </c>
       <c r="H139" s="32">
         <v>48</v>
       </c>
       <c r="I139" s="180">
         <f t="shared" si="8"/>
-        <v>46196.760416666664</v>
+        <v>46198.21875</v>
       </c>
       <c r="J139" s="126">
         <v>16</v>
@@ -39469,21 +39469,21 @@
         <v>404</v>
       </c>
       <c r="E140" s="54">
-        <v>46196</v>
+        <v>46197</v>
       </c>
       <c r="F140" s="180">
-        <v>46198.40625</v>
+        <v>46199.864583333336</v>
       </c>
       <c r="G140" s="180">
         <f t="shared" si="13"/>
-        <v>46199.40625</v>
+        <v>46200.864583333336</v>
       </c>
       <c r="H140" s="32">
         <v>24</v>
       </c>
       <c r="I140" s="180">
         <f t="shared" si="8"/>
-        <v>46200.072916666664</v>
+        <v>46201.53125</v>
       </c>
       <c r="J140" s="126">
         <v>16</v>
@@ -39503,21 +39503,21 @@
         <v>405</v>
       </c>
       <c r="E141" s="54">
-        <v>46207</v>
+        <v>46208</v>
       </c>
       <c r="F141" s="180">
-        <v>46209.036111111112</v>
+        <v>46210.494444444441</v>
       </c>
       <c r="G141" s="180">
         <f t="shared" si="13"/>
-        <v>46210.036111111112</v>
+        <v>46211.494444444441</v>
       </c>
       <c r="H141" s="32">
         <v>24</v>
       </c>
       <c r="I141" s="180">
         <f t="shared" si="8"/>
-        <v>46210.702777777777</v>
+        <v>46212.161111111105</v>
       </c>
       <c r="J141" s="126">
         <v>16</v>
@@ -39537,21 +39537,21 @@
         <v>406</v>
       </c>
       <c r="E142" s="54">
-        <v>46209</v>
+        <v>46210</v>
       </c>
       <c r="F142" s="180">
-        <v>46211.036111111112</v>
+        <v>46212.494444444441</v>
       </c>
       <c r="G142" s="245">
         <f>F142+(H142/24)</f>
-        <v>46212.036111111112</v>
+        <v>46213.494444444441</v>
       </c>
       <c r="H142" s="32">
         <v>24</v>
       </c>
       <c r="I142" s="245">
         <f>G142+(J142/24)</f>
-        <v>46212.702777777777</v>
+        <v>46214.161111111105</v>
       </c>
       <c r="J142" s="126">
         <v>16</v>
@@ -39571,21 +39571,21 @@
         <v>407</v>
       </c>
       <c r="E143" s="240">
-        <v>46217</v>
+        <v>46219</v>
       </c>
       <c r="F143" s="183">
-        <v>46219.691666666666</v>
+        <v>46221.15</v>
       </c>
       <c r="G143" s="205">
         <f>F143+(H143/24)</f>
-        <v>46220.691666666666</v>
+        <v>46222.15</v>
       </c>
       <c r="H143" s="184">
         <v>24</v>
       </c>
       <c r="I143" s="205">
         <f>G143+(J143/24)</f>
-        <v>46221.35833333333</v>
+        <v>46222.816666666666</v>
       </c>
       <c r="J143" s="127">
         <v>16</v>
@@ -41091,12 +41091,27 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="91455a6e-8899-4f67-a6e4-e187ec74b863">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="b2778aaa-fd83-416e-8091-738aa96f6cd3">
+      <Value>1</Value>
+    </TaxCatchAll>
+    <ShortDescription xmlns="91455a6e-8899-4f67-a6e4-e187ec74b863" xsi:nil="true"/>
+    <Sub_x002d_category xmlns="91455a6e-8899-4f67-a6e4-e187ec74b863" xsi:nil="true"/>
+    <SAEFSecurityClassificationTaxHTField0 xmlns="http://schemas.microsoft.com/sharepoint/v3">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+        <TermInfo xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+          <TermName xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">Confidential</TermName>
+          <TermId xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">e4bc29b2-6e76-48cc-b090-8b544c0802ae</TermId>
+        </TermInfo>
+      </Terms>
+    </SAEFSecurityClassificationTaxHTField0>
+    <FocusArea xmlns="91455a6e-8899-4f67-a6e4-e187ec74b863" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -41421,33 +41436,22 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="91455a6e-8899-4f67-a6e4-e187ec74b863">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="b2778aaa-fd83-416e-8091-738aa96f6cd3">
-      <Value>1</Value>
-    </TaxCatchAll>
-    <ShortDescription xmlns="91455a6e-8899-4f67-a6e4-e187ec74b863" xsi:nil="true"/>
-    <Sub_x002d_category xmlns="91455a6e-8899-4f67-a6e4-e187ec74b863" xsi:nil="true"/>
-    <SAEFSecurityClassificationTaxHTField0 xmlns="http://schemas.microsoft.com/sharepoint/v3">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-        <TermInfo xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-          <TermName xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">Confidential</TermName>
-          <TermId xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">e4bc29b2-6e76-48cc-b090-8b544c0802ae</TermId>
-        </TermInfo>
-      </Terms>
-    </SAEFSecurityClassificationTaxHTField0>
-    <FocusArea xmlns="91455a6e-8899-4f67-a6e4-e187ec74b863" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8C73227B-6E13-4F91-A067-CFE89F5B7659}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FE8C99E3-3621-4A94-B7E8-DFCD24F34FA6}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="91455a6e-8899-4f67-a6e4-e187ec74b863"/>
+    <ds:schemaRef ds:uri="b2778aaa-fd83-416e-8091-738aa96f6cd3"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -41473,13 +41477,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FE8C99E3-3621-4A94-B7E8-DFCD24F34FA6}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8C73227B-6E13-4F91-A067-CFE89F5B7659}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="91455a6e-8899-4f67-a6e4-e187ec74b863"/>
-    <ds:schemaRef ds:uri="b2778aaa-fd83-416e-8091-738aa96f6cd3"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Update task and spot-hire data
</commit_message>
<xml_diff>
--- a/uploads/Asset_Activity_Tracker_MASTER.xlsx
+++ b/uploads/Asset_Activity_Tracker_MASTER.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eu001-sp.shell.com/sites/UGPTDWGOMSupplyChain/Shared Documents/SC Delivery/Logistics New Ways of Working/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9322" documentId="8_{8BED3E6F-E7C2-45EA-AB2B-C6B0456C2E64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B3ED4D5B-26F2-4487-BBC7-10DC5A2CCC9F}"/>
+  <xr:revisionPtr revIDLastSave="9406" documentId="8_{8BED3E6F-E7C2-45EA-AB2B-C6B0456C2E64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7BCAF647-7368-47B7-858C-288D29875442}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="11_17_2025 Spot Hire Update" sheetId="2" r:id="rId1"/>
@@ -114,7 +114,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1243" uniqueCount="489">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1242" uniqueCount="488">
   <si>
     <t xml:space="preserve">Top Hole </t>
   </si>
@@ -1956,9 +1956,6 @@
     <t>GL 02 OSV / Drill 12 1/4''x 14 3/4'' section</t>
   </si>
   <si>
-    <t>7/54/2026</t>
-  </si>
-  <si>
     <t>GL 02 OSV-24 Hours- Whipstock BHA / SLB 12-1/4" BHA</t>
   </si>
   <si>
@@ -1975,10 +1972,10 @@
   </si>
   <si>
     <t xml:space="preserve">	
-GL 06 OSV / 48 hrs / 15,000 bbl of 16 ppg WBM</t>
-  </si>
-  <si>
-    <t>GL 12 OSV / 24 hrs / 12-1/4" &amp; 11.97" Casing, Casing Rack Back Tools, 12-1/4" Hanger</t>
+GL 05 OSV / 48 hrs / 15,000 bbl of 16 ppg WBM</t>
+  </si>
+  <si>
+    <t>GL 11 OSV / 24 hrs / 12-1/4" &amp; 11.97" Casing, Casing Rack Back Tools, 12-1/4" Hanger</t>
   </si>
 </sst>
 </file>
@@ -36108,21 +36105,21 @@
         <v>279</v>
       </c>
       <c r="E39" s="425">
-        <v>46199</v>
+        <v>46200</v>
       </c>
       <c r="F39" s="426">
-        <v>46201.3125</v>
+        <v>46202.46875</v>
       </c>
       <c r="G39" s="426">
         <f>F39+(H39/24)</f>
-        <v>46203.3125</v>
+        <v>46204.46875</v>
       </c>
       <c r="H39" s="424">
         <v>48</v>
       </c>
       <c r="I39" s="426">
         <f>G39+(J39/24)</f>
-        <v>46205.3125</v>
+        <v>46206.46875</v>
       </c>
       <c r="J39" s="427">
         <v>48</v>
@@ -36210,21 +36207,21 @@
         <v>281</v>
       </c>
       <c r="E42" s="241">
-        <v>46194</v>
+        <v>46195</v>
       </c>
       <c r="F42" s="213">
-        <v>46198.333333333336</v>
+        <v>46198.96875</v>
       </c>
       <c r="G42" s="180">
         <f>F42+(H42/24)</f>
-        <v>46200.333333333336</v>
+        <v>46200.96875</v>
       </c>
       <c r="H42" s="214">
         <v>48</v>
       </c>
       <c r="I42" s="180">
         <f>G42+(J42/24)</f>
-        <v>46202.333333333336</v>
+        <v>46202.96875</v>
       </c>
       <c r="J42" s="215">
         <v>48</v>
@@ -36278,21 +36275,21 @@
         <v>284</v>
       </c>
       <c r="E44" s="242">
-        <v>46209</v>
+        <v>46210</v>
       </c>
       <c r="F44" s="181">
-        <v>46212.5</v>
+        <v>46213.65625</v>
       </c>
       <c r="G44" s="181">
         <f t="shared" si="2"/>
-        <v>46215.5</v>
+        <v>46216.65625</v>
       </c>
       <c r="H44" s="170">
         <v>72</v>
       </c>
       <c r="I44" s="181">
         <f t="shared" si="3"/>
-        <v>46217.5</v>
+        <v>46218.65625</v>
       </c>
       <c r="J44" s="191">
         <v>48</v>
@@ -36312,21 +36309,21 @@
         <v>285</v>
       </c>
       <c r="E45" s="54">
-        <v>46212</v>
+        <v>46213</v>
       </c>
       <c r="F45" s="180">
-        <v>46215.135416666664</v>
+        <v>46216.291666666664</v>
       </c>
       <c r="G45" s="180">
         <f t="shared" si="2"/>
-        <v>46217.135416666664</v>
+        <v>46218.291666666664</v>
       </c>
       <c r="H45" s="32">
         <v>48</v>
       </c>
       <c r="I45" s="180">
         <f t="shared" si="3"/>
-        <v>46219.135416666664</v>
+        <v>46220.291666666664</v>
       </c>
       <c r="J45" s="126">
         <v>48</v>
@@ -36346,21 +36343,21 @@
         <v>286</v>
       </c>
       <c r="E46" s="54">
-        <v>46218</v>
+        <v>46219</v>
       </c>
       <c r="F46" s="180">
-        <v>46221.760416666664</v>
+        <v>46222.916666666664</v>
       </c>
       <c r="G46" s="180">
         <f t="shared" si="2"/>
-        <v>46224.760416666664</v>
+        <v>46225.916666666664</v>
       </c>
       <c r="H46" s="32">
         <v>72</v>
       </c>
       <c r="I46" s="180">
         <f t="shared" si="3"/>
-        <v>46226.760416666664</v>
+        <v>46227.916666666664</v>
       </c>
       <c r="J46" s="126">
         <v>48</v>
@@ -36380,21 +36377,21 @@
         <v>287</v>
       </c>
       <c r="E47" s="54">
-        <v>46222</v>
+        <v>46224</v>
       </c>
       <c r="F47" s="180">
-        <v>46226.416666666664</v>
+        <v>46227.572916666664</v>
       </c>
       <c r="G47" s="180">
         <f t="shared" si="2"/>
-        <v>46227.416666666664</v>
+        <v>46228.572916666664</v>
       </c>
       <c r="H47" s="32">
         <v>24</v>
       </c>
       <c r="I47" s="180">
         <f t="shared" si="3"/>
-        <v>46229.416666666664</v>
+        <v>46230.572916666664</v>
       </c>
       <c r="J47" s="126">
         <v>48</v>
@@ -36413,22 +36410,22 @@
       <c r="D48" s="7" t="s">
         <v>288</v>
       </c>
-      <c r="E48" s="54" t="s">
-        <v>481</v>
+      <c r="E48" s="54">
+        <v>46229</v>
       </c>
       <c r="F48" s="180">
-        <v>46231.114583333336</v>
+        <v>46232.270833333336</v>
       </c>
       <c r="G48" s="180">
         <f t="shared" si="2"/>
-        <v>46236.114583333336</v>
+        <v>46237.270833333336</v>
       </c>
       <c r="H48" s="32">
         <v>120</v>
       </c>
       <c r="I48" s="180">
         <f t="shared" si="3"/>
-        <v>46238.114583333336</v>
+        <v>46239.270833333336</v>
       </c>
       <c r="J48" s="126">
         <v>48</v>
@@ -36448,21 +36445,21 @@
         <v>289</v>
       </c>
       <c r="E49" s="54">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="F49" s="180">
-        <v>46234.114583333336</v>
+        <v>46235.270833333336</v>
       </c>
       <c r="G49" s="180">
         <f t="shared" si="2"/>
-        <v>46236.114583333336</v>
+        <v>46237.270833333336</v>
       </c>
       <c r="H49" s="32">
         <v>48</v>
       </c>
       <c r="I49" s="180">
         <f t="shared" si="3"/>
-        <v>46238.114583333336</v>
+        <v>46239.270833333336</v>
       </c>
       <c r="J49" s="126">
         <v>48</v>
@@ -36482,21 +36479,21 @@
         <v>290</v>
       </c>
       <c r="E50" s="240">
-        <v>46235</v>
+        <v>46236</v>
       </c>
       <c r="F50" s="183">
-        <v>46238.114583333336</v>
+        <v>46239.270833333336</v>
       </c>
       <c r="G50" s="183">
         <f t="shared" si="2"/>
-        <v>46240.114583333336</v>
+        <v>46241.270833333336</v>
       </c>
       <c r="H50" s="184">
         <v>48</v>
       </c>
       <c r="I50" s="183">
         <f t="shared" si="3"/>
-        <v>46242.114583333336</v>
+        <v>46243.270833333336</v>
       </c>
       <c r="J50" s="127">
         <v>48</v>
@@ -38170,7 +38167,7 @@
     </row>
     <row r="100" spans="1:10" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A100" s="246" t="s">
-        <v>278</v>
+        <v>231</v>
       </c>
       <c r="B100" s="32" t="s">
         <v>311</v>
@@ -38247,24 +38244,24 @@
         <v>348</v>
       </c>
       <c r="D102" s="187" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="E102" s="242">
         <v>46198</v>
       </c>
       <c r="F102" s="181">
-        <v>46200.291666666664</v>
+        <v>46199.75</v>
       </c>
       <c r="G102" s="188">
         <f t="shared" si="4"/>
-        <v>46201.291666666664</v>
+        <v>46200.75</v>
       </c>
       <c r="H102" s="170">
         <v>24</v>
       </c>
       <c r="I102" s="188">
         <f t="shared" si="5"/>
-        <v>46202.083333333328</v>
+        <v>46201.541666666664</v>
       </c>
       <c r="J102" s="191">
         <v>19</v>
@@ -38284,21 +38281,21 @@
         <v>350</v>
       </c>
       <c r="E103" s="54">
-        <v>46202</v>
+        <v>46201</v>
       </c>
       <c r="F103" s="180">
-        <v>46204.53125</v>
+        <v>46204.239583333336</v>
       </c>
       <c r="G103" s="180">
         <f t="shared" si="4"/>
-        <v>46207.03125</v>
+        <v>46206.739583333336</v>
       </c>
       <c r="H103" s="32">
         <v>60</v>
       </c>
       <c r="I103" s="180">
         <f t="shared" si="5"/>
-        <v>46207.822916666664</v>
+        <v>46207.53125</v>
       </c>
       <c r="J103" s="126">
         <v>19</v>
@@ -38315,24 +38312,24 @@
         <v>348</v>
       </c>
       <c r="D104" s="7" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="E104" s="54">
-        <v>46207</v>
+        <v>46206</v>
       </c>
       <c r="F104" s="180">
-        <v>46210.114583333336</v>
+        <v>46209.822916666664</v>
       </c>
       <c r="G104" s="180">
         <f t="shared" ref="G104:G133" si="6">F104+(H104/24)</f>
-        <v>46212.114583333336</v>
+        <v>46211.822916666664</v>
       </c>
       <c r="H104" s="32">
         <v>48</v>
       </c>
       <c r="I104" s="180">
         <f t="shared" ref="I104:I125" si="7">G104+(J104/24)</f>
-        <v>46212.90625</v>
+        <v>46212.614583333328</v>
       </c>
       <c r="J104" s="126">
         <v>19</v>
@@ -38349,24 +38346,24 @@
         <v>348</v>
       </c>
       <c r="D105" s="7" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="E105" s="54">
-        <v>46213</v>
+        <v>46212</v>
       </c>
       <c r="F105" s="213">
-        <v>46214.114583333336</v>
+        <v>46213.822916666664</v>
       </c>
       <c r="G105" s="180">
         <f t="shared" si="6"/>
-        <v>46215.364583333336</v>
+        <v>46215.072916666664</v>
       </c>
       <c r="H105" s="214">
         <v>30</v>
       </c>
       <c r="I105" s="180">
         <f t="shared" si="7"/>
-        <v>46216.15625</v>
+        <v>46215.864583333328</v>
       </c>
       <c r="J105" s="215">
         <v>19</v>
@@ -38389,18 +38386,18 @@
         <v>46219</v>
       </c>
       <c r="F106" s="183">
-        <v>46221.927083333336</v>
+        <v>46221.635416666664</v>
       </c>
       <c r="G106" s="183">
         <f t="shared" si="6"/>
-        <v>46223.427083333336</v>
+        <v>46223.135416666664</v>
       </c>
       <c r="H106" s="184">
         <v>36</v>
       </c>
       <c r="I106" s="183">
         <f t="shared" si="7"/>
-        <v>46224.21875</v>
+        <v>46223.927083333328</v>
       </c>
       <c r="J106" s="127">
         <v>19</v>
@@ -38655,7 +38652,7 @@
         <v>364</v>
       </c>
       <c r="D114" s="386" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="E114" s="387">
         <v>46229</v>
@@ -38689,7 +38686,7 @@
         <v>364</v>
       </c>
       <c r="D115" s="439" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="E115" s="387">
         <v>46231</v>
@@ -39512,21 +39509,21 @@
         <v>398</v>
       </c>
       <c r="E139" s="54">
-        <v>46191</v>
+        <v>46190</v>
       </c>
       <c r="F139" s="180">
-        <v>46194.5625</v>
+        <v>46193.291666666664</v>
       </c>
       <c r="G139" s="180">
         <f t="shared" si="13"/>
-        <v>46195.5625</v>
+        <v>46194.291666666664</v>
       </c>
       <c r="H139" s="32">
         <v>24</v>
       </c>
       <c r="I139" s="180">
         <f t="shared" si="8"/>
-        <v>46196.229166666664</v>
+        <v>46194.958333333328</v>
       </c>
       <c r="J139" s="126">
         <v>16</v>
@@ -39546,21 +39543,21 @@
         <v>399</v>
       </c>
       <c r="E140" s="393">
-        <v>46195</v>
+        <v>46193</v>
       </c>
       <c r="F140" s="394">
-        <v>46197.020833333336</v>
+        <v>46195.729166666664</v>
       </c>
       <c r="G140" s="394">
         <f t="shared" si="13"/>
-        <v>46198.520833333336</v>
+        <v>46197.229166666664</v>
       </c>
       <c r="H140" s="391">
         <v>36</v>
       </c>
       <c r="I140" s="394">
         <f t="shared" si="8"/>
-        <v>46199.1875</v>
+        <v>46197.895833333328</v>
       </c>
       <c r="J140" s="126">
         <v>16</v>
@@ -39577,24 +39574,24 @@
         <v>396</v>
       </c>
       <c r="D141" s="438" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="E141" s="54">
-        <v>46195</v>
+        <v>46194</v>
       </c>
       <c r="F141" s="180">
-        <v>46198.416666666664</v>
+        <v>46197.125</v>
       </c>
       <c r="G141" s="180">
         <f t="shared" si="13"/>
-        <v>46200.416666666664</v>
+        <v>46199.125</v>
       </c>
       <c r="H141" s="32">
         <v>48</v>
       </c>
       <c r="I141" s="180">
         <f t="shared" si="8"/>
-        <v>46201.083333333328</v>
+        <v>46199.791666666664</v>
       </c>
       <c r="J141" s="126">
         <v>16</v>
@@ -39614,21 +39611,21 @@
         <v>400</v>
       </c>
       <c r="E142" s="54">
-        <v>46200</v>
+        <v>46199</v>
       </c>
       <c r="F142" s="180">
-        <v>46202.729166666664</v>
+        <v>46201.4375</v>
       </c>
       <c r="G142" s="180">
         <f t="shared" si="13"/>
-        <v>46203.729166666664</v>
+        <v>46202.4375</v>
       </c>
       <c r="H142" s="32">
         <v>24</v>
       </c>
       <c r="I142" s="180">
         <f t="shared" si="8"/>
-        <v>46204.395833333328</v>
+        <v>46203.104166666664</v>
       </c>
       <c r="J142" s="126">
         <v>16</v>
@@ -39645,24 +39642,24 @@
         <v>396</v>
       </c>
       <c r="D143" s="397" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="E143" s="54">
-        <v>46211</v>
+        <v>46210</v>
       </c>
       <c r="F143" s="180">
-        <v>46213.359027777777</v>
+        <v>46212.067361111112</v>
       </c>
       <c r="G143" s="180">
         <f t="shared" si="13"/>
-        <v>46214.359027777777</v>
+        <v>46213.067361111112</v>
       </c>
       <c r="H143" s="32">
         <v>24</v>
       </c>
       <c r="I143" s="180">
         <f t="shared" si="8"/>
-        <v>46215.025694444441</v>
+        <v>46213.734027777777</v>
       </c>
       <c r="J143" s="126">
         <v>16</v>
@@ -39682,21 +39679,21 @@
         <v>401</v>
       </c>
       <c r="E144" s="54">
-        <v>46213</v>
+        <v>46212</v>
       </c>
       <c r="F144" s="180">
-        <v>46215.359027777777</v>
+        <v>46214.067361111112</v>
       </c>
       <c r="G144" s="245">
         <f t="shared" ref="G144:G153" si="14">F144+(H144/24)</f>
-        <v>46216.359027777777</v>
+        <v>46215.067361111112</v>
       </c>
       <c r="H144" s="32">
         <v>24</v>
       </c>
       <c r="I144" s="245">
         <f>G144+(J144/24)</f>
-        <v>46217.025694444441</v>
+        <v>46215.734027777777</v>
       </c>
       <c r="J144" s="126">
         <v>16</v>
@@ -39716,21 +39713,21 @@
         <v>402</v>
       </c>
       <c r="E145" s="240">
-        <v>46222</v>
+        <v>46220</v>
       </c>
       <c r="F145" s="183">
-        <v>46224.01458333333</v>
+        <v>46222.722916666666</v>
       </c>
       <c r="G145" s="205">
         <f t="shared" si="14"/>
-        <v>46225.01458333333</v>
+        <v>46223.722916666666</v>
       </c>
       <c r="H145" s="184">
         <v>24</v>
       </c>
       <c r="I145" s="205">
         <f>G145+(J145/24)</f>
-        <v>46225.681249999994</v>
+        <v>46224.38958333333</v>
       </c>
       <c r="J145" s="127">
         <v>16</v>

</xml_diff>

<commit_message>
Update OSV Demand Scheduler and Spot Hire Planner links - July 2, 2026 - Update links markdown with GitHub Pages URLs - Update local URL shortcuts to v20260702 - Add team distribution ZIP with START_SCHEDULER.bat - Import latest task data
</commit_message>
<xml_diff>
--- a/uploads/Asset_Activity_Tracker_MASTER.xlsx
+++ b/uploads/Asset_Activity_Tracker_MASTER.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eu001-sp.shell.com/sites/UGPTDWGOMSupplyChain/Shared Documents/SC Delivery/Logistics New Ways of Working/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10057" documentId="8_{8BED3E6F-E7C2-45EA-AB2B-C6B0456C2E64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{082D1287-C561-42F5-9975-C140488B7A1E}"/>
+  <xr:revisionPtr revIDLastSave="10112" documentId="8_{8BED3E6F-E7C2-45EA-AB2B-C6B0456C2E64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{63627695-D43C-41C6-9D6E-3780F162F986}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
     <sheet name="Vessel Schedule" sheetId="5" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'OSV Demand Tracker'!$A$1:$J$214</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'OSV Demand Tracker'!$A$1:$J$213</definedName>
     <definedName name="Actual">(PeriodInActual*(#REF!&gt;0))*PeriodInPlan</definedName>
     <definedName name="ActualBeyond">PeriodInActual*(#REF!&gt;0)</definedName>
     <definedName name="PercentComplete">PercentCompleteBeyond*PeriodInPlan</definedName>
@@ -114,7 +114,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1324" uniqueCount="508">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1320" uniqueCount="507">
   <si>
     <t xml:space="preserve">Top Hole </t>
   </si>
@@ -1757,10 +1757,6 @@
     <t>GL 08 OSV / 36 hrs / 9,000 bbl of 11.3 ppg SBM, SBM Chemicals, 18-1/8" x 21" BHA, 18" Casing, 18" Liner Hanger</t>
   </si>
   <si>
-    <t xml:space="preserve">	
-GL 11 OSV / 24 hrs / Weekly Groceries &amp; Rig Supplies, MI 9,000 bbls 13.2, 3,000 bbls 16.0 &amp; 1,500 bbls Unweighted</t>
-  </si>
-  <si>
     <t>GL 13 OSV / 24 hrs / 12-1/4" &amp; 11.97" Casing, Casing Rack Back Tools, 12-1/4" Hanger</t>
   </si>
   <si>
@@ -2026,10 +2022,6 @@
     <t>GL 10 OSV / 24 hrs / 18" Casing Tools, Cement Head, 3,7000 Sacks of Cement, Cement Chemicals, SBM Chemicals</t>
   </si>
   <si>
-    <t xml:space="preserve">	
-GL 12 OSV / 36 hrs / 16-1/2" x 19" BHA, 3,000 bbl 16 ppg &amp; 1,500 bbl Unweighted SBM, TOI 5-7/8 DP &amp; HWDP</t>
-  </si>
-  <si>
     <t>Vito VA-10 Drift / CTCO</t>
   </si>
   <si>
@@ -2049,6 +2041,9 @@
   </si>
   <si>
     <t>GL 06 OSV- 60 Hours- Demob</t>
+  </si>
+  <si>
+    <t>GL 12 OSV / 36 hrs / 16-1/2" x 19" BHA, 3,000 bbl 16 ppg &amp; 1,500 bbl Unweighted SBM, TOI 5-7/8 DP &amp; HWDP</t>
   </si>
 </sst>
 </file>
@@ -34285,7 +34280,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E64F7A7C-F00C-4BD1-AABC-21B710242BB1}">
   <sheetPr codeName="Sheet1" filterMode="1"/>
-  <dimension ref="A1:Y214"/>
+  <dimension ref="A1:Y213"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.109375" style="6" bestFit="1" customWidth="1"/>
@@ -37821,18 +37816,18 @@
         <v>46209</v>
       </c>
       <c r="F104" s="177">
-        <v>46212.125</v>
+        <v>46212.083333333336</v>
       </c>
       <c r="G104" s="177">
         <f t="shared" si="6"/>
-        <v>46214.625</v>
+        <v>46214.583333333336</v>
       </c>
       <c r="H104" s="32">
         <v>60</v>
       </c>
       <c r="I104" s="177">
         <f t="shared" si="7"/>
-        <v>46215.375</v>
+        <v>46215.333333333336</v>
       </c>
       <c r="J104" s="211">
         <v>18</v>
@@ -37855,18 +37850,18 @@
         <v>46214</v>
       </c>
       <c r="F105" s="177">
-        <v>46217.21875</v>
+        <v>46217.114583333336</v>
       </c>
       <c r="G105" s="177">
         <f t="shared" ref="G105:G138" si="8">F105+(H105/24)</f>
-        <v>46219.21875</v>
+        <v>46219.114583333336</v>
       </c>
       <c r="H105" s="32">
         <v>48</v>
       </c>
       <c r="I105" s="177">
         <f t="shared" ref="I105:I126" si="9">G105+(J105/24)</f>
-        <v>46219.96875</v>
+        <v>46219.864583333336</v>
       </c>
       <c r="J105" s="211">
         <v>18</v>
@@ -37889,18 +37884,18 @@
         <v>46218</v>
       </c>
       <c r="F106" s="177">
-        <v>46219.118750000001</v>
+        <v>46219.01458333333</v>
       </c>
       <c r="G106" s="177">
         <f t="shared" si="8"/>
-        <v>46220.368750000001</v>
+        <v>46220.26458333333</v>
       </c>
       <c r="H106" s="32">
         <v>30</v>
       </c>
       <c r="I106" s="177">
         <f t="shared" si="9"/>
-        <v>46221.118750000001</v>
+        <v>46221.01458333333</v>
       </c>
       <c r="J106" s="211">
         <v>18</v>
@@ -37923,18 +37918,18 @@
         <v>46226</v>
       </c>
       <c r="F107" s="177">
-        <v>46228.03125</v>
+        <v>46227.927083333336</v>
       </c>
       <c r="G107" s="177">
         <f t="shared" si="8"/>
-        <v>46229.53125</v>
+        <v>46229.427083333336</v>
       </c>
       <c r="H107" s="32">
         <v>36</v>
       </c>
       <c r="I107" s="177">
         <f t="shared" si="9"/>
-        <v>46230.28125</v>
+        <v>46230.177083333336</v>
       </c>
       <c r="J107" s="211">
         <v>18</v>
@@ -38229,18 +38224,18 @@
         <v>46231</v>
       </c>
       <c r="F116" s="177">
-        <v>46233</v>
+        <v>46233.041666666664</v>
       </c>
       <c r="G116" s="177">
         <f t="shared" si="8"/>
-        <v>46235</v>
+        <v>46235.041666666664</v>
       </c>
       <c r="H116" s="32">
         <v>48</v>
       </c>
       <c r="I116" s="177">
         <f t="shared" si="9"/>
-        <v>46235.5</v>
+        <v>46235.541666666664</v>
       </c>
       <c r="J116" s="32">
         <v>12</v>
@@ -38989,7 +38984,7 @@
         <v>10</v>
       </c>
       <c r="I138" s="177">
-        <f t="shared" ref="I138:I196" si="15">G138+(J138/24)</f>
+        <f t="shared" ref="I138:I195" si="15">G138+(J138/24)</f>
         <v>46164.833333333328</v>
       </c>
       <c r="J138" s="32">
@@ -39050,7 +39045,7 @@
         <v>46168</v>
       </c>
       <c r="G140" s="177">
-        <f t="shared" ref="G140:G196" si="16">F140+(H140/24)</f>
+        <f t="shared" ref="G140:G195" si="16">F140+(H140/24)</f>
         <v>46168.208333333336</v>
       </c>
       <c r="H140" s="32">
@@ -39381,24 +39376,24 @@
         <v>408</v>
       </c>
       <c r="D150" s="304" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="E150" s="54">
         <v>46207</v>
       </c>
       <c r="F150" s="177">
-        <v>46209.802083333336</v>
+        <v>46209.84375</v>
       </c>
       <c r="G150" s="177">
         <f>F150+(H150/24)</f>
-        <v>46210.802083333336</v>
+        <v>46210.84375</v>
       </c>
       <c r="H150" s="32">
         <v>24</v>
       </c>
       <c r="I150" s="177">
         <f>G150+(J150/24)</f>
-        <v>46211.34375</v>
+        <v>46211.385416666664</v>
       </c>
       <c r="J150" s="32">
         <v>13</v>
@@ -39415,24 +39410,24 @@
         <v>408</v>
       </c>
       <c r="D151" s="309" t="s">
-        <v>416</v>
+        <v>506</v>
       </c>
       <c r="E151" s="54">
-        <v>46210</v>
+        <v>46211</v>
       </c>
       <c r="F151" s="177">
-        <v>46212.25</v>
+        <v>46212.5</v>
       </c>
       <c r="G151" s="177">
         <f t="shared" si="16"/>
-        <v>46213.25</v>
+        <v>46213.5</v>
       </c>
       <c r="H151" s="32">
         <v>24</v>
       </c>
       <c r="I151" s="177">
         <f t="shared" si="15"/>
-        <v>46213.791666666664</v>
+        <v>46214.041666666664</v>
       </c>
       <c r="J151" s="32">
         <v>13</v>
@@ -39449,24 +39444,24 @@
         <v>408</v>
       </c>
       <c r="D152" s="309" t="s">
-        <v>501</v>
+        <v>416</v>
       </c>
       <c r="E152" s="54">
-        <v>46210</v>
+        <v>46214</v>
       </c>
       <c r="F152" s="177">
-        <v>46212.458333333336</v>
+        <v>46216.668749999997</v>
       </c>
       <c r="G152" s="177">
-        <f t="shared" si="16"/>
-        <v>46213.958333333336</v>
+        <f>F152+(H152/24)</f>
+        <v>46217.668749999997</v>
       </c>
       <c r="H152" s="32">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="I152" s="177">
-        <f t="shared" si="15"/>
-        <v>46214.5</v>
+        <f>G152+(J152/24)</f>
+        <v>46218.210416666661</v>
       </c>
       <c r="J152" s="32">
         <v>13</v>
@@ -39486,139 +39481,139 @@
         <v>417</v>
       </c>
       <c r="E153" s="54">
-        <v>46214</v>
+        <v>46216</v>
       </c>
       <c r="F153" s="177">
-        <v>46216.533333333333</v>
+        <v>46217.818749999999</v>
       </c>
       <c r="G153" s="177">
         <f>F153+(H153/24)</f>
-        <v>46217.533333333333</v>
+        <v>46218.818749999999</v>
       </c>
       <c r="H153" s="32">
         <v>24</v>
       </c>
       <c r="I153" s="177">
         <f>G153+(J153/24)</f>
-        <v>46218.074999999997</v>
+        <v>46219.360416666663</v>
       </c>
       <c r="J153" s="32">
         <v>13</v>
       </c>
     </row>
     <row r="154" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A154" s="7" t="s">
+      <c r="A154" s="212" t="s">
         <v>282</v>
       </c>
-      <c r="B154" s="32" t="s">
+      <c r="B154" s="211" t="s">
         <v>232</v>
       </c>
-      <c r="C154" s="7" t="s">
+      <c r="C154" s="212" t="s">
         <v>408</v>
       </c>
       <c r="D154" s="309" t="s">
         <v>418</v>
       </c>
       <c r="E154" s="54">
-        <v>46216</v>
+        <v>46225</v>
       </c>
       <c r="F154" s="177">
-        <v>46217.777083333334</v>
-      </c>
-      <c r="G154" s="177">
-        <f>F154+(H154/24)</f>
-        <v>46218.777083333334</v>
+        <v>46227.323611111111</v>
+      </c>
+      <c r="G154" s="213">
+        <f t="shared" ref="G154:G165" si="17">F154+(H154/24)</f>
+        <v>46228.323611111111</v>
       </c>
       <c r="H154" s="32">
         <v>24</v>
       </c>
-      <c r="I154" s="177">
+      <c r="I154" s="213">
         <f>G154+(J154/24)</f>
-        <v>46219.318749999999</v>
+        <v>46228.865277777775</v>
       </c>
       <c r="J154" s="32">
         <v>13</v>
       </c>
     </row>
-    <row r="155" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A155" s="212" t="s">
-        <v>282</v>
-      </c>
-      <c r="B155" s="211" t="s">
-        <v>232</v>
-      </c>
-      <c r="C155" s="212" t="s">
-        <v>408</v>
-      </c>
-      <c r="D155" s="309" t="s">
+    <row r="155" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A155" s="7" t="s">
+        <v>231</v>
+      </c>
+      <c r="B155" s="32" t="s">
+        <v>64</v>
+      </c>
+      <c r="C155" s="7" t="s">
         <v>419</v>
       </c>
+      <c r="D155" s="304" t="s">
+        <v>420</v>
+      </c>
       <c r="E155" s="54">
-        <v>46225</v>
+        <v>46193</v>
       </c>
       <c r="F155" s="177">
-        <v>46227.281944444447</v>
-      </c>
-      <c r="G155" s="213">
-        <f t="shared" ref="G155:G166" si="17">F155+(H155/24)</f>
-        <v>46228.281944444447</v>
-      </c>
-      <c r="H155" s="32">
-        <v>24</v>
-      </c>
-      <c r="I155" s="213">
+        <v>46195.25</v>
+      </c>
+      <c r="G155" s="177">
+        <f t="shared" si="17"/>
+        <v>46197.25</v>
+      </c>
+      <c r="H155" s="303">
+        <v>48</v>
+      </c>
+      <c r="I155" s="177">
         <f>G155+(J155/24)</f>
-        <v>46228.823611111111</v>
-      </c>
-      <c r="J155" s="32">
-        <v>13</v>
+        <v>46197.5</v>
+      </c>
+      <c r="J155" s="303">
+        <v>6</v>
       </c>
     </row>
     <row r="156" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A156" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="B156" s="32" t="s">
-        <v>64</v>
-      </c>
-      <c r="C156" s="7" t="s">
-        <v>420</v>
-      </c>
-      <c r="D156" s="304" t="s">
+      <c r="A156" s="7"/>
+      <c r="B156" s="32"/>
+      <c r="C156" s="7"/>
+      <c r="D156" s="304"/>
+      <c r="E156" s="54"/>
+      <c r="F156" s="177"/>
+      <c r="G156" s="177"/>
+      <c r="H156" s="32"/>
+      <c r="I156" s="177"/>
+      <c r="J156" s="32"/>
+    </row>
+    <row r="157" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A157" s="7" t="s">
+        <v>282</v>
+      </c>
+      <c r="B157" s="32" t="s">
+        <v>20</v>
+      </c>
+      <c r="C157" s="7" t="s">
         <v>421</v>
       </c>
-      <c r="E156" s="54">
-        <v>46193</v>
-      </c>
-      <c r="F156" s="177">
-        <v>46195.25</v>
-      </c>
-      <c r="G156" s="177">
+      <c r="D157" s="304" t="s">
+        <v>422</v>
+      </c>
+      <c r="E157" s="54">
+        <v>46211</v>
+      </c>
+      <c r="F157" s="177">
+        <v>46213.041666666664</v>
+      </c>
+      <c r="G157" s="177">
         <f t="shared" si="17"/>
-        <v>46197.25</v>
-      </c>
-      <c r="H156" s="303">
-        <v>48</v>
-      </c>
-      <c r="I156" s="177">
-        <f>G156+(J156/24)</f>
-        <v>46197.5</v>
-      </c>
-      <c r="J156" s="303">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="157" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A157" s="7"/>
-      <c r="B157" s="32"/>
-      <c r="C157" s="7"/>
-      <c r="D157" s="304"/>
-      <c r="E157" s="54"/>
-      <c r="F157" s="177"/>
-      <c r="G157" s="177"/>
-      <c r="H157" s="32"/>
-      <c r="I157" s="177"/>
-      <c r="J157" s="32"/>
+        <v>46216.041666666664</v>
+      </c>
+      <c r="H157" s="32">
+        <v>72</v>
+      </c>
+      <c r="I157" s="177">
+        <f t="shared" ref="I157:I159" si="18">G157+(J157/24)</f>
+        <v>46217.541666666664</v>
+      </c>
+      <c r="J157" s="32">
+        <v>36</v>
+      </c>
     </row>
     <row r="158" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A158" s="7" t="s">
@@ -39628,27 +39623,27 @@
         <v>20</v>
       </c>
       <c r="C158" s="7" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="D158" s="304" t="s">
         <v>423</v>
       </c>
       <c r="E158" s="54">
-        <v>46210</v>
+        <v>46216</v>
       </c>
       <c r="F158" s="177">
-        <v>46212.479166666664</v>
+        <v>46218.4375</v>
       </c>
       <c r="G158" s="177">
         <f t="shared" si="17"/>
-        <v>46215.479166666664</v>
-      </c>
-      <c r="H158" s="32">
+        <v>46221.4375</v>
+      </c>
+      <c r="H158" s="303">
         <v>72</v>
       </c>
       <c r="I158" s="177">
-        <f t="shared" ref="I158:I160" si="18">G158+(J158/24)</f>
-        <v>46216.979166666664</v>
+        <f t="shared" si="18"/>
+        <v>46222.9375</v>
       </c>
       <c r="J158" s="32">
         <v>36</v>
@@ -39662,27 +39657,27 @@
         <v>20</v>
       </c>
       <c r="C159" s="7" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="D159" s="304" t="s">
         <v>424</v>
       </c>
       <c r="E159" s="54">
-        <v>46215</v>
+        <v>46218</v>
       </c>
       <c r="F159" s="177">
-        <v>46217.875</v>
+        <v>46220.770833333336</v>
       </c>
       <c r="G159" s="177">
         <f t="shared" si="17"/>
-        <v>46220.875</v>
+        <v>46223.770833333336</v>
       </c>
       <c r="H159" s="303">
         <v>72</v>
       </c>
       <c r="I159" s="177">
         <f t="shared" si="18"/>
-        <v>46222.375</v>
+        <v>46225.270833333336</v>
       </c>
       <c r="J159" s="32">
         <v>36</v>
@@ -39696,27 +39691,27 @@
         <v>20</v>
       </c>
       <c r="C160" s="7" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="D160" s="304" t="s">
         <v>425</v>
       </c>
       <c r="E160" s="54">
-        <v>46218</v>
+        <v>46222</v>
       </c>
       <c r="F160" s="177">
-        <v>46220.208333333336</v>
+        <v>46224.6875</v>
       </c>
       <c r="G160" s="177">
         <f t="shared" si="17"/>
-        <v>46223.208333333336</v>
+        <v>46227.6875</v>
       </c>
       <c r="H160" s="303">
         <v>72</v>
       </c>
       <c r="I160" s="177">
-        <f t="shared" si="18"/>
-        <v>46224.708333333336</v>
+        <f t="shared" ref="I160:I165" si="19">G160+(J160/24)</f>
+        <v>46229.1875</v>
       </c>
       <c r="J160" s="32">
         <v>36</v>
@@ -39730,27 +39725,27 @@
         <v>20</v>
       </c>
       <c r="C161" s="7" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="D161" s="304" t="s">
         <v>426</v>
       </c>
       <c r="E161" s="54">
-        <v>46222</v>
+        <v>46225</v>
       </c>
       <c r="F161" s="177">
-        <v>46224.125</v>
+        <v>46227.541666666664</v>
       </c>
       <c r="G161" s="177">
         <f t="shared" si="17"/>
-        <v>46227.125</v>
+        <v>46230.541666666664</v>
       </c>
       <c r="H161" s="303">
         <v>72</v>
       </c>
       <c r="I161" s="177">
-        <f t="shared" ref="I161:I166" si="19">G161+(J161/24)</f>
-        <v>46228.625</v>
+        <f t="shared" si="19"/>
+        <v>46232.041666666664</v>
       </c>
       <c r="J161" s="32">
         <v>36</v>
@@ -39764,27 +39759,27 @@
         <v>20</v>
       </c>
       <c r="C162" s="7" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="D162" s="304" t="s">
         <v>427</v>
       </c>
       <c r="E162" s="54">
-        <v>46224</v>
+        <v>46235</v>
       </c>
       <c r="F162" s="177">
-        <v>46226.979166666664</v>
+        <v>46237.125</v>
       </c>
       <c r="G162" s="177">
         <f t="shared" si="17"/>
-        <v>46229.979166666664</v>
+        <v>46240.125</v>
       </c>
       <c r="H162" s="303">
         <v>72</v>
       </c>
       <c r="I162" s="177">
         <f t="shared" si="19"/>
-        <v>46231.479166666664</v>
+        <v>46241.625</v>
       </c>
       <c r="J162" s="32">
         <v>36</v>
@@ -39798,27 +39793,27 @@
         <v>20</v>
       </c>
       <c r="C163" s="7" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="D163" s="304" t="s">
         <v>428</v>
       </c>
       <c r="E163" s="54">
-        <v>46234</v>
+        <v>46240</v>
       </c>
       <c r="F163" s="177">
-        <v>46236.5625</v>
+        <v>46242.25</v>
       </c>
       <c r="G163" s="177">
         <f t="shared" si="17"/>
-        <v>46239.5625</v>
+        <v>46245.25</v>
       </c>
       <c r="H163" s="303">
         <v>72</v>
       </c>
       <c r="I163" s="177">
         <f t="shared" si="19"/>
-        <v>46241.0625</v>
+        <v>46246.75</v>
       </c>
       <c r="J163" s="32">
         <v>36</v>
@@ -39832,27 +39827,27 @@
         <v>20</v>
       </c>
       <c r="C164" s="7" t="s">
-        <v>422</v>
-      </c>
-      <c r="D164" s="304" t="s">
+        <v>421</v>
+      </c>
+      <c r="D164" s="6" t="s">
         <v>429</v>
       </c>
       <c r="E164" s="54">
-        <v>46239</v>
+        <v>46241</v>
       </c>
       <c r="F164" s="177">
-        <v>46241.6875</v>
+        <v>46243.3125</v>
       </c>
       <c r="G164" s="177">
         <f t="shared" si="17"/>
-        <v>46244.6875</v>
+        <v>46246.3125</v>
       </c>
       <c r="H164" s="303">
         <v>72</v>
       </c>
       <c r="I164" s="177">
         <f t="shared" si="19"/>
-        <v>46246.1875</v>
+        <v>46247.8125</v>
       </c>
       <c r="J164" s="32">
         <v>36</v>
@@ -39866,65 +39861,43 @@
         <v>20</v>
       </c>
       <c r="C165" s="7" t="s">
-        <v>422</v>
-      </c>
-      <c r="D165" s="6" t="s">
+        <v>421</v>
+      </c>
+      <c r="D165" s="304" t="s">
         <v>430</v>
       </c>
       <c r="E165" s="54">
-        <v>46240</v>
+        <v>46357</v>
       </c>
       <c r="F165" s="177">
-        <v>46242.75</v>
+        <v>46361</v>
       </c>
       <c r="G165" s="177">
         <f t="shared" si="17"/>
-        <v>46245.75</v>
+        <v>46364</v>
       </c>
       <c r="H165" s="303">
         <v>72</v>
       </c>
       <c r="I165" s="177">
         <f t="shared" si="19"/>
-        <v>46247.25</v>
+        <v>46365.5</v>
       </c>
       <c r="J165" s="32">
         <v>36</v>
       </c>
     </row>
-    <row r="166" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A166" s="7" t="s">
-        <v>282</v>
-      </c>
-      <c r="B166" s="32" t="s">
-        <v>20</v>
-      </c>
-      <c r="C166" s="7" t="s">
-        <v>422</v>
-      </c>
-      <c r="D166" s="304" t="s">
-        <v>431</v>
-      </c>
-      <c r="E166" s="54">
-        <v>46357</v>
-      </c>
-      <c r="F166" s="177">
-        <v>46361</v>
-      </c>
-      <c r="G166" s="177">
-        <f t="shared" si="17"/>
-        <v>46364</v>
-      </c>
-      <c r="H166" s="303">
-        <v>72</v>
-      </c>
-      <c r="I166" s="177">
-        <f t="shared" si="19"/>
-        <v>46365.5</v>
-      </c>
-      <c r="J166" s="32">
-        <v>36</v>
-      </c>
+    <row r="166" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A166" s="7"/>
+      <c r="B166" s="32"/>
+      <c r="C166" s="7"/>
+      <c r="D166" s="304"/>
+      <c r="E166" s="54"/>
+      <c r="F166" s="177"/>
+      <c r="G166" s="177"/>
+      <c r="H166" s="303"/>
+      <c r="I166" s="177"/>
+      <c r="J166" s="32"/>
     </row>
     <row r="167" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A167" s="7"/>
@@ -40076,23 +40049,60 @@
       <c r="C179" s="7"/>
       <c r="D179" s="304"/>
       <c r="E179" s="54"/>
-      <c r="F179" s="177"/>
+      <c r="F179" s="213"/>
       <c r="G179" s="177"/>
-      <c r="H179" s="303"/>
+      <c r="H179" s="32"/>
       <c r="I179" s="177"/>
       <c r="J179" s="32"/>
     </row>
-    <row r="180" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A180" s="7"/>
-      <c r="B180" s="32"/>
-      <c r="C180" s="7"/>
-      <c r="D180" s="304"/>
-      <c r="E180" s="54"/>
-      <c r="F180" s="213"/>
-      <c r="G180" s="177"/>
-      <c r="H180" s="32"/>
-      <c r="I180" s="177"/>
-      <c r="J180" s="32"/>
+    <row r="180" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A180" s="212" t="s">
+        <v>282</v>
+      </c>
+      <c r="B180" s="211" t="s">
+        <v>20</v>
+      </c>
+      <c r="C180" s="212" t="s">
+        <v>431</v>
+      </c>
+      <c r="D180" s="310" t="s">
+        <v>432</v>
+      </c>
+      <c r="E180" s="311">
+        <v>46327</v>
+      </c>
+      <c r="F180" s="213">
+        <v>46330.25</v>
+      </c>
+      <c r="G180" s="213">
+        <f t="shared" si="16"/>
+        <v>46334.25</v>
+      </c>
+      <c r="H180" s="211">
+        <v>96</v>
+      </c>
+      <c r="I180" s="213">
+        <f t="shared" si="15"/>
+        <v>46335.75</v>
+      </c>
+      <c r="J180" s="211">
+        <v>36</v>
+      </c>
+      <c r="K180" s="312"/>
+      <c r="L180" s="312"/>
+      <c r="M180" s="312"/>
+      <c r="N180" s="312"/>
+      <c r="O180" s="312"/>
+      <c r="P180" s="312"/>
+      <c r="Q180" s="312"/>
+      <c r="R180" s="312"/>
+      <c r="S180" s="312"/>
+      <c r="T180" s="312"/>
+      <c r="U180" s="312"/>
+      <c r="V180" s="312"/>
+      <c r="W180" s="312"/>
+      <c r="X180" s="312"/>
+      <c r="Y180" s="312"/>
     </row>
     <row r="181" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A181" s="212" t="s">
@@ -40102,27 +40112,27 @@
         <v>20</v>
       </c>
       <c r="C181" s="212" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="D181" s="310" t="s">
         <v>433</v>
       </c>
       <c r="E181" s="311">
-        <v>46327</v>
+        <v>46334</v>
       </c>
       <c r="F181" s="213">
-        <v>46330.25</v>
+        <v>46334.25</v>
       </c>
       <c r="G181" s="213">
         <f t="shared" si="16"/>
-        <v>46334.25</v>
+        <v>46338.25</v>
       </c>
       <c r="H181" s="211">
         <v>96</v>
       </c>
       <c r="I181" s="213">
         <f t="shared" si="15"/>
-        <v>46335.75</v>
+        <v>46339.75</v>
       </c>
       <c r="J181" s="211">
         <v>36</v>
@@ -40151,27 +40161,27 @@
         <v>20</v>
       </c>
       <c r="C182" s="212" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="D182" s="310" t="s">
         <v>434</v>
       </c>
       <c r="E182" s="311">
-        <v>46334</v>
+        <v>46341</v>
       </c>
       <c r="F182" s="213">
-        <v>46334.25</v>
+        <v>46344.25</v>
       </c>
       <c r="G182" s="213">
         <f t="shared" si="16"/>
-        <v>46338.25</v>
+        <v>46348.25</v>
       </c>
       <c r="H182" s="211">
         <v>96</v>
       </c>
       <c r="I182" s="213">
         <f t="shared" si="15"/>
-        <v>46339.75</v>
+        <v>46349.75</v>
       </c>
       <c r="J182" s="211">
         <v>36</v>
@@ -40200,27 +40210,27 @@
         <v>20</v>
       </c>
       <c r="C183" s="212" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="D183" s="310" t="s">
         <v>435</v>
       </c>
       <c r="E183" s="311">
-        <v>46341</v>
+        <v>46348</v>
       </c>
       <c r="F183" s="213">
-        <v>46344.25</v>
+        <v>46351.25</v>
       </c>
       <c r="G183" s="213">
         <f t="shared" si="16"/>
-        <v>46348.25</v>
+        <v>46355.25</v>
       </c>
       <c r="H183" s="211">
         <v>96</v>
       </c>
       <c r="I183" s="213">
         <f t="shared" si="15"/>
-        <v>46349.75</v>
+        <v>46356.75</v>
       </c>
       <c r="J183" s="211">
         <v>36</v>
@@ -40249,27 +40259,27 @@
         <v>20</v>
       </c>
       <c r="C184" s="212" t="s">
-        <v>432</v>
-      </c>
-      <c r="D184" s="310" t="s">
+        <v>431</v>
+      </c>
+      <c r="D184" s="302" t="s">
         <v>436</v>
       </c>
       <c r="E184" s="311">
-        <v>46348</v>
+        <v>46355</v>
       </c>
       <c r="F184" s="213">
-        <v>46351.25</v>
+        <v>46358.25</v>
       </c>
       <c r="G184" s="213">
         <f t="shared" si="16"/>
-        <v>46355.25</v>
+        <v>46362.25</v>
       </c>
       <c r="H184" s="211">
         <v>96</v>
       </c>
       <c r="I184" s="213">
         <f t="shared" si="15"/>
-        <v>46356.75</v>
+        <v>46363.75</v>
       </c>
       <c r="J184" s="211">
         <v>36</v>
@@ -40297,28 +40307,28 @@
       <c r="B185" s="211" t="s">
         <v>20</v>
       </c>
-      <c r="C185" s="212" t="s">
-        <v>432</v>
+      <c r="C185" s="7" t="s">
+        <v>437</v>
       </c>
       <c r="D185" s="302" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="E185" s="311">
-        <v>46355</v>
+        <v>46235</v>
       </c>
       <c r="F185" s="213">
-        <v>46358.25</v>
+        <v>46237.25</v>
       </c>
       <c r="G185" s="213">
         <f t="shared" si="16"/>
-        <v>46362.25</v>
+        <v>46282.25</v>
       </c>
       <c r="H185" s="211">
-        <v>96</v>
+        <v>1080</v>
       </c>
       <c r="I185" s="213">
         <f t="shared" si="15"/>
-        <v>46363.75</v>
+        <v>46283.75</v>
       </c>
       <c r="J185" s="211">
         <v>36</v>
@@ -40347,10 +40357,10 @@
         <v>20</v>
       </c>
       <c r="C186" s="7" t="s">
+        <v>437</v>
+      </c>
+      <c r="D186" s="302" t="s">
         <v>438</v>
-      </c>
-      <c r="D186" s="302" t="s">
-        <v>439</v>
       </c>
       <c r="E186" s="311">
         <v>46235</v>
@@ -40388,167 +40398,152 @@
       <c r="X186" s="312"/>
       <c r="Y186" s="312"/>
     </row>
-    <row r="187" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="A187" s="212" t="s">
+    <row r="187" spans="1:25" s="9" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A187" s="314" t="s">
+        <v>231</v>
+      </c>
+      <c r="B187" s="313" t="s">
+        <v>122</v>
+      </c>
+      <c r="C187" s="314" t="s">
+        <v>439</v>
+      </c>
+      <c r="D187" s="315" t="s">
+        <v>440</v>
+      </c>
+      <c r="E187" s="318">
+        <v>46193</v>
+      </c>
+      <c r="F187" s="319">
+        <v>46196.25</v>
+      </c>
+      <c r="G187" s="319">
+        <f t="shared" si="16"/>
+        <v>46197.75</v>
+      </c>
+      <c r="H187" s="313">
+        <v>36</v>
+      </c>
+      <c r="I187" s="319">
+        <f t="shared" si="15"/>
+        <v>46198.25</v>
+      </c>
+      <c r="J187" s="313">
+        <v>12</v>
+      </c>
+      <c r="K187" s="320"/>
+      <c r="L187" s="320"/>
+      <c r="M187" s="320"/>
+      <c r="N187" s="320"/>
+      <c r="O187" s="320"/>
+      <c r="P187" s="320"/>
+      <c r="Q187" s="320"/>
+      <c r="R187" s="320"/>
+      <c r="S187" s="320"/>
+      <c r="T187" s="320"/>
+      <c r="U187" s="320"/>
+      <c r="V187" s="320"/>
+      <c r="W187" s="320"/>
+      <c r="X187" s="320"/>
+      <c r="Y187" s="320"/>
+    </row>
+    <row r="188" spans="1:25" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A188" s="314" t="s">
         <v>282</v>
-      </c>
-      <c r="B187" s="211" t="s">
-        <v>20</v>
-      </c>
-      <c r="C187" s="7" t="s">
-        <v>438</v>
-      </c>
-      <c r="D187" s="302" t="s">
-        <v>439</v>
-      </c>
-      <c r="E187" s="311">
-        <v>46235</v>
-      </c>
-      <c r="F187" s="213">
-        <v>46237.25</v>
-      </c>
-      <c r="G187" s="213">
-        <f t="shared" si="16"/>
-        <v>46282.25</v>
-      </c>
-      <c r="H187" s="211">
-        <v>1080</v>
-      </c>
-      <c r="I187" s="213">
-        <f t="shared" si="15"/>
-        <v>46283.75</v>
-      </c>
-      <c r="J187" s="211">
-        <v>36</v>
-      </c>
-      <c r="K187" s="312"/>
-      <c r="L187" s="312"/>
-      <c r="M187" s="312"/>
-      <c r="N187" s="312"/>
-      <c r="O187" s="312"/>
-      <c r="P187" s="312"/>
-      <c r="Q187" s="312"/>
-      <c r="R187" s="312"/>
-      <c r="S187" s="312"/>
-      <c r="T187" s="312"/>
-      <c r="U187" s="312"/>
-      <c r="V187" s="312"/>
-      <c r="W187" s="312"/>
-      <c r="X187" s="312"/>
-      <c r="Y187" s="312"/>
-    </row>
-    <row r="188" spans="1:25" s="9" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A188" s="314" t="s">
-        <v>231</v>
       </c>
       <c r="B188" s="313" t="s">
         <v>122</v>
       </c>
       <c r="C188" s="314" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="D188" s="315" t="s">
-        <v>441</v>
-      </c>
-      <c r="E188" s="318">
-        <v>46193</v>
-      </c>
-      <c r="F188" s="319">
-        <v>46196.25</v>
-      </c>
-      <c r="G188" s="319">
+        <v>442</v>
+      </c>
+      <c r="E188" s="316">
+        <v>46209</v>
+      </c>
+      <c r="F188" s="317">
+        <v>46211.375</v>
+      </c>
+      <c r="G188" s="317">
         <f t="shared" si="16"/>
-        <v>46197.75</v>
+        <v>46213.375</v>
       </c>
       <c r="H188" s="313">
-        <v>36</v>
-      </c>
-      <c r="I188" s="319">
+        <v>48</v>
+      </c>
+      <c r="I188" s="317">
         <f t="shared" si="15"/>
-        <v>46198.25</v>
+        <v>46213.875</v>
       </c>
       <c r="J188" s="313">
         <v>12</v>
       </c>
-      <c r="K188" s="320"/>
-      <c r="L188" s="320"/>
-      <c r="M188" s="320"/>
-      <c r="N188" s="320"/>
-      <c r="O188" s="320"/>
-      <c r="P188" s="320"/>
-      <c r="Q188" s="320"/>
-      <c r="R188" s="320"/>
-      <c r="S188" s="320"/>
-      <c r="T188" s="320"/>
-      <c r="U188" s="320"/>
-      <c r="V188" s="320"/>
-      <c r="W188" s="320"/>
-      <c r="X188" s="320"/>
-      <c r="Y188" s="320"/>
     </row>
-    <row r="189" spans="1:25" s="9" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A189" s="314" t="s">
+    <row r="189" spans="1:25" s="9" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A189" s="314"/>
+      <c r="B189" s="313"/>
+      <c r="C189" s="314"/>
+      <c r="D189" s="329" t="s">
+        <v>443</v>
+      </c>
+      <c r="E189" s="316">
+        <v>46222</v>
+      </c>
+      <c r="F189" s="317">
+        <v>46224.53125</v>
+      </c>
+      <c r="G189" s="317">
+        <f t="shared" ref="G189" si="20">F189+(H189/24)</f>
+        <v>46227.03125</v>
+      </c>
+      <c r="H189" s="313">
+        <v>60</v>
+      </c>
+      <c r="I189" s="317">
+        <f t="shared" ref="I189" si="21">G189+(J189/24)</f>
+        <v>46227.572916666664</v>
+      </c>
+      <c r="J189" s="313">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="190" spans="1:25" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A190" s="314" t="s">
         <v>282</v>
       </c>
-      <c r="B189" s="313" t="s">
+      <c r="B190" s="313" t="s">
         <v>122</v>
       </c>
-      <c r="C189" s="314" t="s">
-        <v>442</v>
-      </c>
-      <c r="D189" s="315" t="s">
-        <v>443</v>
-      </c>
-      <c r="E189" s="316">
-        <v>46209</v>
-      </c>
-      <c r="F189" s="317">
-        <v>46211.375</v>
-      </c>
-      <c r="G189" s="317">
+      <c r="C190" s="314" t="s">
+        <v>441</v>
+      </c>
+      <c r="D190" s="315" t="s">
+        <v>444</v>
+      </c>
+      <c r="E190" s="316">
+        <v>46228</v>
+      </c>
+      <c r="F190" s="317">
+        <v>46230.1875</v>
+      </c>
+      <c r="G190" s="317">
         <f t="shared" si="16"/>
-        <v>46213.375</v>
-      </c>
-      <c r="H189" s="313">
+        <v>46232.1875</v>
+      </c>
+      <c r="H190" s="313">
         <v>48</v>
       </c>
-      <c r="I189" s="317">
+      <c r="I190" s="317">
         <f t="shared" si="15"/>
-        <v>46213.875</v>
-      </c>
-      <c r="J189" s="313">
+        <v>46232.6875</v>
+      </c>
+      <c r="J190" s="313">
         <v>12</v>
       </c>
     </row>
-    <row r="190" spans="1:25" s="9" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A190" s="314"/>
-      <c r="B190" s="313"/>
-      <c r="C190" s="314"/>
-      <c r="D190" s="329" t="s">
-        <v>444</v>
-      </c>
-      <c r="E190" s="316">
-        <v>46222</v>
-      </c>
-      <c r="F190" s="317">
-        <v>46224.53125</v>
-      </c>
-      <c r="G190" s="317">
-        <f t="shared" ref="G190" si="20">F190+(H190/24)</f>
-        <v>46227.03125</v>
-      </c>
-      <c r="H190" s="313">
-        <v>60</v>
-      </c>
-      <c r="I190" s="317">
-        <f t="shared" ref="I190" si="21">G190+(J190/24)</f>
-        <v>46227.572916666664</v>
-      </c>
-      <c r="J190" s="313">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="191" spans="1:25" s="9" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:25" s="9" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A191" s="314" t="s">
         <v>282</v>
       </c>
@@ -40556,33 +40551,33 @@
         <v>122</v>
       </c>
       <c r="C191" s="314" t="s">
-        <v>442</v>
-      </c>
-      <c r="D191" s="315" t="s">
+        <v>441</v>
+      </c>
+      <c r="D191" s="328" t="s">
         <v>445</v>
       </c>
       <c r="E191" s="316">
-        <v>46228</v>
+        <v>46233</v>
       </c>
       <c r="F191" s="317">
-        <v>46230.1875</v>
+        <v>46235.729166666664</v>
       </c>
       <c r="G191" s="317">
         <f t="shared" si="16"/>
-        <v>46232.1875</v>
+        <v>46238.729166666664</v>
       </c>
       <c r="H191" s="313">
-        <v>48</v>
+        <v>72</v>
       </c>
       <c r="I191" s="317">
         <f t="shared" si="15"/>
-        <v>46232.6875</v>
+        <v>46239.229166666664</v>
       </c>
       <c r="J191" s="313">
         <v>12</v>
       </c>
     </row>
-    <row r="192" spans="1:25" s="9" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:25" s="9" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A192" s="314" t="s">
         <v>282</v>
       </c>
@@ -40590,33 +40585,33 @@
         <v>122</v>
       </c>
       <c r="C192" s="314" t="s">
-        <v>442</v>
-      </c>
-      <c r="D192" s="328" t="s">
+        <v>441</v>
+      </c>
+      <c r="D192" s="315" t="s">
         <v>446</v>
       </c>
       <c r="E192" s="316">
-        <v>46233</v>
+        <v>46242</v>
       </c>
       <c r="F192" s="317">
-        <v>46235.729166666664</v>
+        <v>46244.645833333336</v>
       </c>
       <c r="G192" s="317">
         <f t="shared" si="16"/>
-        <v>46238.729166666664</v>
+        <v>46246.645833333336</v>
       </c>
       <c r="H192" s="313">
-        <v>72</v>
+        <v>48</v>
       </c>
       <c r="I192" s="317">
         <f t="shared" si="15"/>
-        <v>46239.229166666664</v>
+        <v>46247.145833333336</v>
       </c>
       <c r="J192" s="313">
         <v>12</v>
       </c>
     </row>
-    <row r="193" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:10" s="9" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A193" s="314" t="s">
         <v>282</v>
       </c>
@@ -40624,27 +40619,27 @@
         <v>122</v>
       </c>
       <c r="C193" s="314" t="s">
-        <v>442</v>
-      </c>
-      <c r="D193" s="315" t="s">
+        <v>441</v>
+      </c>
+      <c r="D193" s="328" t="s">
         <v>447</v>
       </c>
       <c r="E193" s="316">
-        <v>46242</v>
+        <v>46245</v>
       </c>
       <c r="F193" s="317">
-        <v>46244.645833333336</v>
+        <v>46247.833333333336</v>
       </c>
       <c r="G193" s="317">
         <f t="shared" si="16"/>
-        <v>46246.645833333336</v>
+        <v>46249.833333333336</v>
       </c>
       <c r="H193" s="313">
         <v>48</v>
       </c>
       <c r="I193" s="317">
         <f t="shared" si="15"/>
-        <v>46247.145833333336</v>
+        <v>46250.333333333336</v>
       </c>
       <c r="J193" s="313">
         <v>12</v>
@@ -40658,27 +40653,27 @@
         <v>122</v>
       </c>
       <c r="C194" s="314" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="D194" s="328" t="s">
         <v>448</v>
       </c>
       <c r="E194" s="316">
-        <v>46245</v>
+        <v>46248</v>
       </c>
       <c r="F194" s="317">
-        <v>46247.833333333336</v>
+        <v>46250.75</v>
       </c>
       <c r="G194" s="317">
         <f t="shared" si="16"/>
-        <v>46249.833333333336</v>
+        <v>46252.75</v>
       </c>
       <c r="H194" s="313">
         <v>48</v>
       </c>
       <c r="I194" s="317">
         <f t="shared" si="15"/>
-        <v>46250.333333333336</v>
+        <v>46253.25</v>
       </c>
       <c r="J194" s="313">
         <v>12</v>
@@ -40692,95 +40687,95 @@
         <v>122</v>
       </c>
       <c r="C195" s="314" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="D195" s="328" t="s">
         <v>449</v>
       </c>
       <c r="E195" s="316">
-        <v>46248</v>
+        <v>46250</v>
       </c>
       <c r="F195" s="317">
-        <v>46250.75</v>
+        <v>46252.479166666664</v>
       </c>
       <c r="G195" s="317">
         <f t="shared" si="16"/>
-        <v>46252.75</v>
+        <v>46254.979166666664</v>
       </c>
       <c r="H195" s="313">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="I195" s="317">
         <f t="shared" si="15"/>
-        <v>46253.25</v>
+        <v>46255.479166666664</v>
       </c>
       <c r="J195" s="313">
         <v>12</v>
       </c>
     </row>
-    <row r="196" spans="1:10" s="9" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A196" s="314" t="s">
+    <row r="196" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A196" s="212" t="s">
+        <v>231</v>
+      </c>
+      <c r="B196" s="32" t="s">
+        <v>64</v>
+      </c>
+      <c r="C196" s="212" t="s">
+        <v>450</v>
+      </c>
+      <c r="D196" s="310" t="s">
+        <v>451</v>
+      </c>
+      <c r="E196" s="54">
+        <v>46184</v>
+      </c>
+      <c r="F196" s="177">
+        <v>46185</v>
+      </c>
+      <c r="G196" s="177">
+        <f t="shared" ref="G196:G213" si="22">F196+(H196/24)</f>
+        <v>46187</v>
+      </c>
+      <c r="H196" s="303">
+        <v>48</v>
+      </c>
+      <c r="I196" s="177">
+        <f t="shared" ref="I196:I213" si="23">G196+(J196/24)</f>
+        <v>46187.25</v>
+      </c>
+      <c r="J196" s="211">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="197" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A197" s="212" t="s">
         <v>282</v>
-      </c>
-      <c r="B196" s="313" t="s">
-        <v>122</v>
-      </c>
-      <c r="C196" s="314" t="s">
-        <v>442</v>
-      </c>
-      <c r="D196" s="328" t="s">
-        <v>450</v>
-      </c>
-      <c r="E196" s="316">
-        <v>46250</v>
-      </c>
-      <c r="F196" s="317">
-        <v>46252.479166666664</v>
-      </c>
-      <c r="G196" s="317">
-        <f t="shared" si="16"/>
-        <v>46254.979166666664</v>
-      </c>
-      <c r="H196" s="313">
-        <v>60</v>
-      </c>
-      <c r="I196" s="317">
-        <f t="shared" si="15"/>
-        <v>46255.479166666664</v>
-      </c>
-      <c r="J196" s="313">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="197" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A197" s="212" t="s">
-        <v>231</v>
       </c>
       <c r="B197" s="32" t="s">
         <v>64</v>
       </c>
-      <c r="C197" s="212" t="s">
-        <v>451</v>
-      </c>
-      <c r="D197" s="310" t="s">
+      <c r="C197" s="7" t="s">
+        <v>500</v>
+      </c>
+      <c r="D197" s="212" t="s">
         <v>452</v>
       </c>
       <c r="E197" s="54">
-        <v>46184</v>
+        <v>46207</v>
       </c>
       <c r="F197" s="177">
-        <v>46185</v>
-      </c>
-      <c r="G197" s="177">
-        <f t="shared" ref="G197:G214" si="22">F197+(H197/24)</f>
-        <v>46187</v>
+        <v>46208.645833333336</v>
+      </c>
+      <c r="G197" s="213">
+        <f t="shared" si="22"/>
+        <v>46210.645833333336</v>
       </c>
       <c r="H197" s="303">
         <v>48</v>
       </c>
-      <c r="I197" s="177">
-        <f t="shared" ref="I197:I214" si="23">G197+(J197/24)</f>
-        <v>46187.25</v>
+      <c r="I197" s="213">
+        <f t="shared" si="23"/>
+        <v>46210.895833333336</v>
       </c>
       <c r="J197" s="211">
         <v>6</v>
@@ -40794,98 +40789,98 @@
         <v>64</v>
       </c>
       <c r="C198" s="7" t="s">
-        <v>502</v>
+        <v>500</v>
       </c>
       <c r="D198" s="212" t="s">
         <v>453</v>
       </c>
       <c r="E198" s="54">
-        <v>46207</v>
+        <v>46208</v>
       </c>
       <c r="F198" s="177">
-        <v>46208.645833333336</v>
+        <v>46210.375</v>
       </c>
       <c r="G198" s="213">
         <f t="shared" si="22"/>
-        <v>46210.645833333336</v>
+        <v>46212.375</v>
       </c>
       <c r="H198" s="303">
         <v>48</v>
       </c>
       <c r="I198" s="213">
         <f t="shared" si="23"/>
-        <v>46210.895833333336</v>
+        <v>46212.625</v>
       </c>
       <c r="J198" s="211">
         <v>6</v>
       </c>
     </row>
     <row r="199" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A199" s="212" t="s">
+      <c r="A199" s="7" t="s">
         <v>282</v>
       </c>
       <c r="B199" s="32" t="s">
         <v>64</v>
       </c>
       <c r="C199" s="7" t="s">
-        <v>502</v>
-      </c>
-      <c r="D199" s="212" t="s">
         <v>454</v>
+      </c>
+      <c r="D199" s="7" t="s">
+        <v>455</v>
       </c>
       <c r="E199" s="54">
         <v>46208</v>
       </c>
       <c r="F199" s="177">
-        <v>46210.375</v>
+        <v>46212.875</v>
       </c>
       <c r="G199" s="213">
         <f t="shared" si="22"/>
-        <v>46212.375</v>
-      </c>
-      <c r="H199" s="303">
+        <v>46214.875</v>
+      </c>
+      <c r="H199" s="327">
         <v>48</v>
       </c>
       <c r="I199" s="213">
         <f t="shared" si="23"/>
-        <v>46212.625</v>
+        <v>46215.125</v>
       </c>
       <c r="J199" s="211">
         <v>6</v>
       </c>
     </row>
     <row r="200" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A200" s="7" t="s">
+      <c r="A200" s="212" t="s">
         <v>282</v>
       </c>
-      <c r="B200" s="32" t="s">
-        <v>64</v>
-      </c>
-      <c r="C200" s="7" t="s">
-        <v>455</v>
-      </c>
-      <c r="D200" s="7" t="s">
+      <c r="B200" s="211" t="s">
+        <v>160</v>
+      </c>
+      <c r="C200" s="212" t="s">
         <v>456</v>
       </c>
+      <c r="D200" s="212" t="s">
+        <v>457</v>
+      </c>
       <c r="E200" s="54">
-        <v>46208</v>
+        <v>46237</v>
       </c>
       <c r="F200" s="177">
-        <v>46212.875</v>
+        <v>46240.916666666664</v>
       </c>
       <c r="G200" s="213">
         <f t="shared" si="22"/>
-        <v>46214.875</v>
-      </c>
-      <c r="H200" s="327">
-        <v>48</v>
+        <v>46243.916666666664</v>
+      </c>
+      <c r="H200" s="32">
+        <v>72</v>
       </c>
       <c r="I200" s="213">
         <f t="shared" si="23"/>
-        <v>46215.125</v>
-      </c>
-      <c r="J200" s="211">
-        <v>6</v>
+        <v>46245.416666666664</v>
+      </c>
+      <c r="J200" s="32">
+        <v>36</v>
       </c>
     </row>
     <row r="201" spans="1:10" x14ac:dyDescent="0.3">
@@ -40896,27 +40891,27 @@
         <v>160</v>
       </c>
       <c r="C201" s="212" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="D201" s="212" t="s">
         <v>458</v>
       </c>
       <c r="E201" s="54">
-        <v>46237</v>
+        <v>46239</v>
       </c>
       <c r="F201" s="177">
-        <v>46240.916666666664</v>
+        <v>46242.541666666664</v>
       </c>
       <c r="G201" s="213">
         <f t="shared" si="22"/>
-        <v>46243.916666666664</v>
+        <v>46245.541666666664</v>
       </c>
       <c r="H201" s="32">
         <v>72</v>
       </c>
       <c r="I201" s="213">
         <f t="shared" si="23"/>
-        <v>46245.416666666664</v>
+        <v>46247.041666666664</v>
       </c>
       <c r="J201" s="32">
         <v>36</v>
@@ -40930,27 +40925,27 @@
         <v>160</v>
       </c>
       <c r="C202" s="212" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="D202" s="212" t="s">
         <v>459</v>
       </c>
       <c r="E202" s="54">
-        <v>46239</v>
+        <v>46242</v>
       </c>
       <c r="F202" s="177">
-        <v>46242.541666666664</v>
+        <v>46245.59652777778</v>
       </c>
       <c r="G202" s="213">
         <f t="shared" si="22"/>
-        <v>46245.541666666664</v>
+        <v>46248.59652777778</v>
       </c>
       <c r="H202" s="32">
         <v>72</v>
       </c>
       <c r="I202" s="213">
         <f t="shared" si="23"/>
-        <v>46247.041666666664</v>
+        <v>46250.09652777778</v>
       </c>
       <c r="J202" s="32">
         <v>36</v>
@@ -40964,27 +40959,27 @@
         <v>160</v>
       </c>
       <c r="C203" s="212" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="D203" s="212" t="s">
         <v>460</v>
       </c>
       <c r="E203" s="54">
-        <v>46242</v>
+        <v>46245</v>
       </c>
       <c r="F203" s="177">
-        <v>46245.59652777778</v>
+        <v>46248.059027777781</v>
       </c>
       <c r="G203" s="213">
         <f t="shared" si="22"/>
-        <v>46248.59652777778</v>
+        <v>46251.059027777781</v>
       </c>
       <c r="H203" s="32">
         <v>72</v>
       </c>
       <c r="I203" s="213">
         <f t="shared" si="23"/>
-        <v>46250.09652777778</v>
+        <v>46252.559027777781</v>
       </c>
       <c r="J203" s="32">
         <v>36</v>
@@ -40998,27 +40993,27 @@
         <v>160</v>
       </c>
       <c r="C204" s="212" t="s">
-        <v>457</v>
+        <v>461</v>
       </c>
       <c r="D204" s="212" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="E204" s="54">
-        <v>46245</v>
+        <v>46247</v>
       </c>
       <c r="F204" s="177">
-        <v>46248.059027777781</v>
+        <v>46250.017361111109</v>
       </c>
       <c r="G204" s="213">
         <f t="shared" si="22"/>
-        <v>46251.059027777781</v>
+        <v>46253.017361111109</v>
       </c>
       <c r="H204" s="32">
         <v>72</v>
       </c>
       <c r="I204" s="213">
         <f t="shared" si="23"/>
-        <v>46252.559027777781</v>
+        <v>46254.517361111109</v>
       </c>
       <c r="J204" s="32">
         <v>36</v>
@@ -41032,27 +41027,27 @@
         <v>160</v>
       </c>
       <c r="C205" s="212" t="s">
-        <v>462</v>
-      </c>
-      <c r="D205" s="212" t="s">
-        <v>463</v>
+        <v>461</v>
+      </c>
+      <c r="D205" s="7" t="s">
+        <v>275</v>
       </c>
       <c r="E205" s="54">
-        <v>46247</v>
+        <v>46252</v>
       </c>
       <c r="F205" s="177">
-        <v>46250.017361111109</v>
+        <v>46255.892361111109</v>
       </c>
       <c r="G205" s="213">
         <f t="shared" si="22"/>
-        <v>46253.017361111109</v>
+        <v>46257.892361111109</v>
       </c>
       <c r="H205" s="32">
-        <v>72</v>
+        <v>48</v>
       </c>
       <c r="I205" s="213">
         <f t="shared" si="23"/>
-        <v>46254.517361111109</v>
+        <v>46259.392361111109</v>
       </c>
       <c r="J205" s="32">
         <v>36</v>
@@ -41066,27 +41061,27 @@
         <v>160</v>
       </c>
       <c r="C206" s="212" t="s">
-        <v>462</v>
-      </c>
-      <c r="D206" s="7" t="s">
-        <v>275</v>
+        <v>461</v>
+      </c>
+      <c r="D206" s="212" t="s">
+        <v>463</v>
       </c>
       <c r="E206" s="54">
-        <v>46252</v>
+        <v>46262</v>
       </c>
       <c r="F206" s="177">
-        <v>46255.892361111109</v>
+        <v>46265.704861111109</v>
       </c>
       <c r="G206" s="213">
         <f t="shared" si="22"/>
-        <v>46257.892361111109</v>
+        <v>46267.704861111109</v>
       </c>
       <c r="H206" s="32">
         <v>48</v>
       </c>
       <c r="I206" s="213">
         <f t="shared" si="23"/>
-        <v>46259.392361111109</v>
+        <v>46269.204861111109</v>
       </c>
       <c r="J206" s="32">
         <v>36</v>
@@ -41100,27 +41095,27 @@
         <v>160</v>
       </c>
       <c r="C207" s="212" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="D207" s="212" t="s">
-        <v>464</v>
+        <v>278</v>
       </c>
       <c r="E207" s="54">
-        <v>46262</v>
+        <v>46269</v>
       </c>
       <c r="F207" s="177">
-        <v>46265.704861111109</v>
+        <v>46272.079861111109</v>
       </c>
       <c r="G207" s="213">
         <f t="shared" si="22"/>
-        <v>46267.704861111109</v>
+        <v>46274.079861111109</v>
       </c>
       <c r="H207" s="32">
         <v>48</v>
       </c>
       <c r="I207" s="213">
         <f t="shared" si="23"/>
-        <v>46269.204861111109</v>
+        <v>46275.579861111109</v>
       </c>
       <c r="J207" s="32">
         <v>36</v>
@@ -41131,33 +41126,33 @@
         <v>282</v>
       </c>
       <c r="B208" s="211" t="s">
-        <v>160</v>
+        <v>312</v>
       </c>
       <c r="C208" s="212" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="D208" s="212" t="s">
-        <v>278</v>
+        <v>465</v>
       </c>
       <c r="E208" s="54">
-        <v>46269</v>
+        <v>46233</v>
       </c>
       <c r="F208" s="177">
-        <v>46272.079861111109</v>
+        <v>46236.072916666664</v>
       </c>
       <c r="G208" s="213">
         <f t="shared" si="22"/>
-        <v>46274.079861111109</v>
+        <v>46238.072916666664</v>
       </c>
       <c r="H208" s="32">
         <v>48</v>
       </c>
       <c r="I208" s="213">
         <f t="shared" si="23"/>
-        <v>46275.579861111109</v>
+        <v>46238.822916666664</v>
       </c>
       <c r="J208" s="32">
-        <v>36</v>
+        <v>18</v>
       </c>
     </row>
     <row r="209" spans="1:10" x14ac:dyDescent="0.3">
@@ -41168,27 +41163,27 @@
         <v>312</v>
       </c>
       <c r="C209" s="212" t="s">
-        <v>465</v>
-      </c>
-      <c r="D209" s="212" t="s">
-        <v>466</v>
+        <v>464</v>
+      </c>
+      <c r="D209" s="7" t="s">
+        <v>501</v>
       </c>
       <c r="E209" s="54">
-        <v>46233</v>
+        <v>46235</v>
       </c>
       <c r="F209" s="177">
-        <v>46236.114583333336</v>
+        <v>46237.822916666664</v>
       </c>
       <c r="G209" s="213">
         <f t="shared" si="22"/>
-        <v>46238.114583333336</v>
+        <v>46239.822916666664</v>
       </c>
       <c r="H209" s="32">
         <v>48</v>
       </c>
       <c r="I209" s="213">
         <f t="shared" si="23"/>
-        <v>46238.864583333336</v>
+        <v>46240.572916666664</v>
       </c>
       <c r="J209" s="32">
         <v>18</v>
@@ -41202,27 +41197,27 @@
         <v>312</v>
       </c>
       <c r="C210" s="212" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="D210" s="7" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="E210" s="54">
-        <v>46235</v>
+        <v>46242</v>
       </c>
       <c r="F210" s="177">
-        <v>46237.864583333336</v>
+        <v>46245.49722222222</v>
       </c>
       <c r="G210" s="213">
         <f t="shared" si="22"/>
-        <v>46239.864583333336</v>
+        <v>46247.49722222222</v>
       </c>
       <c r="H210" s="32">
         <v>48</v>
       </c>
       <c r="I210" s="213">
         <f t="shared" si="23"/>
-        <v>46240.614583333336</v>
+        <v>46248.24722222222</v>
       </c>
       <c r="J210" s="32">
         <v>18</v>
@@ -41236,27 +41231,27 @@
         <v>312</v>
       </c>
       <c r="C211" s="212" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="D211" s="7" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="E211" s="54">
-        <v>46242</v>
+        <v>46248</v>
       </c>
       <c r="F211" s="177">
-        <v>46245.538888888892</v>
+        <v>46251.027083333334</v>
       </c>
       <c r="G211" s="213">
         <f t="shared" si="22"/>
-        <v>46247.538888888892</v>
+        <v>46253.027083333334</v>
       </c>
       <c r="H211" s="32">
         <v>48</v>
       </c>
       <c r="I211" s="213">
         <f t="shared" si="23"/>
-        <v>46248.288888888892</v>
+        <v>46253.777083333334</v>
       </c>
       <c r="J211" s="32">
         <v>18</v>
@@ -41270,27 +41265,27 @@
         <v>312</v>
       </c>
       <c r="C212" s="212" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="D212" s="7" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="E212" s="54">
-        <v>46248</v>
+        <v>46256</v>
       </c>
       <c r="F212" s="177">
-        <v>46251.068749999999</v>
+        <v>46259.619444444441</v>
       </c>
       <c r="G212" s="213">
         <f t="shared" si="22"/>
-        <v>46253.068749999999</v>
+        <v>46261.119444444441</v>
       </c>
       <c r="H212" s="32">
-        <v>48</v>
+        <v>36</v>
       </c>
       <c r="I212" s="213">
         <f t="shared" si="23"/>
-        <v>46253.818749999999</v>
+        <v>46261.869444444441</v>
       </c>
       <c r="J212" s="32">
         <v>18</v>
@@ -41304,68 +41299,34 @@
         <v>312</v>
       </c>
       <c r="C213" s="212" t="s">
-        <v>465</v>
-      </c>
-      <c r="D213" s="7" t="s">
-        <v>506</v>
+        <v>464</v>
+      </c>
+      <c r="D213" s="308" t="s">
+        <v>505</v>
       </c>
       <c r="E213" s="54">
-        <v>46256</v>
+        <v>46262</v>
       </c>
       <c r="F213" s="177">
-        <v>46259.661111111112</v>
+        <v>46265.463194444441</v>
       </c>
       <c r="G213" s="213">
         <f t="shared" si="22"/>
-        <v>46261.161111111112</v>
+        <v>46267.963194444441</v>
       </c>
       <c r="H213" s="32">
-        <v>36</v>
+        <v>60</v>
       </c>
       <c r="I213" s="213">
         <f t="shared" si="23"/>
-        <v>46261.911111111112</v>
+        <v>46268.713194444441</v>
       </c>
       <c r="J213" s="32">
         <v>18</v>
       </c>
     </row>
-    <row r="214" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A214" s="212" t="s">
-        <v>282</v>
-      </c>
-      <c r="B214" s="211" t="s">
-        <v>312</v>
-      </c>
-      <c r="C214" s="212" t="s">
-        <v>465</v>
-      </c>
-      <c r="D214" s="308" t="s">
-        <v>507</v>
-      </c>
-      <c r="E214" s="54">
-        <v>46262</v>
-      </c>
-      <c r="F214" s="177">
-        <v>46265.504861111112</v>
-      </c>
-      <c r="G214" s="213">
-        <f t="shared" si="22"/>
-        <v>46268.004861111112</v>
-      </c>
-      <c r="H214" s="32">
-        <v>60</v>
-      </c>
-      <c r="I214" s="213">
-        <f t="shared" si="23"/>
-        <v>46268.754861111112</v>
-      </c>
-      <c r="J214" s="32">
-        <v>18</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:J214" xr:uid="{E64F7A7C-F00C-4BD1-AABC-21B710242BB1}">
+  <autoFilter ref="A1:J213" xr:uid="{E64F7A7C-F00C-4BD1-AABC-21B710242BB1}">
     <filterColumn colId="0">
       <filters>
         <filter val="Planned"/>
@@ -41374,14 +41335,14 @@
   </autoFilter>
   <phoneticPr fontId="15" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="D181" r:id="rId1" display="https://app01.kabal.com/mws/f?p=1720:320:3591087192783:ADDBACK:NO::P320_PORT_TASK_ID:60703:" xr:uid="{2CE69447-1583-4285-A3C6-E44253861F50}"/>
-    <hyperlink ref="D182" r:id="rId2" display="https://app01.kabal.com/mws/f?p=1720:320:3591087192783:ADDBACK:NO::P320_PORT_TASK_ID:60704:" xr:uid="{9B646115-87F0-4E9B-A26C-E8EDC2346D02}"/>
-    <hyperlink ref="D183" r:id="rId3" display="https://app01.kabal.com/mws/f?p=1720:320:3591087192783:ADDBACK:NO::P320_PORT_TASK_ID:60705:" xr:uid="{E88F1C80-86A4-402C-A7FA-01CE4B12C622}"/>
-    <hyperlink ref="D184" r:id="rId4" display="https://app01.kabal.com/mws/f?p=1720:320:3591087192783:ADDBACK:NO::P320_PORT_TASK_ID:60706:" xr:uid="{ED524307-DD66-4DB1-9398-118E3CD28160}"/>
-    <hyperlink ref="D185" r:id="rId5" display="https://app01.kabal.com/mws/f?p=1720:320:3591087192783:ADDBACK:NO::P320_PORT_TASK_ID:60707:" xr:uid="{2A3CDFC3-31C8-44B2-8428-4BB6443AB947}"/>
-    <hyperlink ref="C188" r:id="rId6" xr:uid="{4BF92AC9-6F81-47D3-BADE-793677667278}"/>
-    <hyperlink ref="D189" r:id="rId7" xr:uid="{E7B658C7-FFEB-4978-9A4E-D4E57D76FD92}"/>
-    <hyperlink ref="D191" r:id="rId8" xr:uid="{42CF593B-3B32-4FD3-BF01-D92D8C273D20}"/>
+    <hyperlink ref="D180" r:id="rId1" display="https://app01.kabal.com/mws/f?p=1720:320:3591087192783:ADDBACK:NO::P320_PORT_TASK_ID:60703:" xr:uid="{2CE69447-1583-4285-A3C6-E44253861F50}"/>
+    <hyperlink ref="D181" r:id="rId2" display="https://app01.kabal.com/mws/f?p=1720:320:3591087192783:ADDBACK:NO::P320_PORT_TASK_ID:60704:" xr:uid="{9B646115-87F0-4E9B-A26C-E8EDC2346D02}"/>
+    <hyperlink ref="D182" r:id="rId3" display="https://app01.kabal.com/mws/f?p=1720:320:3591087192783:ADDBACK:NO::P320_PORT_TASK_ID:60705:" xr:uid="{E88F1C80-86A4-402C-A7FA-01CE4B12C622}"/>
+    <hyperlink ref="D183" r:id="rId4" display="https://app01.kabal.com/mws/f?p=1720:320:3591087192783:ADDBACK:NO::P320_PORT_TASK_ID:60706:" xr:uid="{ED524307-DD66-4DB1-9398-118E3CD28160}"/>
+    <hyperlink ref="D184" r:id="rId5" display="https://app01.kabal.com/mws/f?p=1720:320:3591087192783:ADDBACK:NO::P320_PORT_TASK_ID:60707:" xr:uid="{2A3CDFC3-31C8-44B2-8428-4BB6443AB947}"/>
+    <hyperlink ref="C187" r:id="rId6" xr:uid="{4BF92AC9-6F81-47D3-BADE-793677667278}"/>
+    <hyperlink ref="D188" r:id="rId7" xr:uid="{E7B658C7-FFEB-4978-9A4E-D4E57D76FD92}"/>
+    <hyperlink ref="D190" r:id="rId8" xr:uid="{42CF593B-3B32-4FD3-BF01-D92D8C273D20}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId9"/>
@@ -41422,45 +41383,45 @@
     <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2" s="70"/>
       <c r="B2" s="71" t="s">
+        <v>466</v>
+      </c>
+      <c r="C2" s="72" t="s">
         <v>467</v>
       </c>
-      <c r="C2" s="72" t="s">
+      <c r="D2" s="72" t="s">
         <v>468</v>
       </c>
-      <c r="D2" s="72" t="s">
+      <c r="E2" s="73" t="s">
         <v>469</v>
       </c>
-      <c r="E2" s="73" t="s">
-        <v>470</v>
-      </c>
       <c r="F2" s="74" t="s">
+        <v>466</v>
+      </c>
+      <c r="G2" s="72" t="s">
         <v>467</v>
       </c>
-      <c r="G2" s="72" t="s">
+      <c r="H2" s="72" t="s">
         <v>468</v>
       </c>
-      <c r="H2" s="72" t="s">
+      <c r="I2" s="73" t="s">
         <v>469</v>
       </c>
-      <c r="I2" s="73" t="s">
-        <v>470</v>
-      </c>
       <c r="J2" s="74" t="s">
+        <v>466</v>
+      </c>
+      <c r="K2" s="72" t="s">
         <v>467</v>
       </c>
-      <c r="K2" s="72" t="s">
+      <c r="L2" s="72" t="s">
         <v>468</v>
       </c>
-      <c r="L2" s="72" t="s">
+      <c r="M2" s="73" t="s">
         <v>469</v>
-      </c>
-      <c r="M2" s="73" t="s">
-        <v>470</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3" s="75" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="B3" s="76"/>
       <c r="C3" s="76"/>
@@ -41468,7 +41429,7 @@
       <c r="E3" s="76"/>
       <c r="F3" s="76"/>
       <c r="G3" s="76" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="H3" s="76"/>
       <c r="I3" s="76"/>
@@ -41479,7 +41440,7 @@
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4" s="75" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="B4" s="76"/>
       <c r="C4" s="76"/>
@@ -41487,7 +41448,7 @@
       <c r="E4" s="76"/>
       <c r="F4" s="76"/>
       <c r="G4" s="76" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="H4" s="76"/>
       <c r="I4" s="76"/>
@@ -41498,7 +41459,7 @@
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5" s="75" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="B5" s="76"/>
       <c r="C5" s="76"/>
@@ -41506,7 +41467,7 @@
       <c r="E5" s="76"/>
       <c r="F5" s="76"/>
       <c r="G5" s="76" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="H5" s="76"/>
       <c r="I5" s="76"/>
@@ -41517,7 +41478,7 @@
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6" s="75" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="B6" s="77"/>
       <c r="C6" s="78"/>
@@ -41525,7 +41486,7 @@
       <c r="E6" s="79"/>
       <c r="F6" s="80"/>
       <c r="G6" s="81" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="H6" s="78"/>
       <c r="I6" s="79"/>
@@ -41536,7 +41497,7 @@
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7" s="75" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="B7" s="77"/>
       <c r="C7" s="78"/>
@@ -41544,7 +41505,7 @@
       <c r="E7" s="79"/>
       <c r="F7" s="80"/>
       <c r="G7" s="81" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="H7" s="78"/>
       <c r="I7" s="79"/>
@@ -41558,7 +41519,7 @@
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8" s="75" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="B8" s="77"/>
       <c r="C8" s="78"/>
@@ -41566,7 +41527,7 @@
       <c r="E8" s="79"/>
       <c r="F8" s="80"/>
       <c r="G8" s="81" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="H8" s="78"/>
       <c r="I8" s="79"/>
@@ -41577,7 +41538,7 @@
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9" s="75" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="B9" s="82"/>
       <c r="C9" s="83"/>
@@ -41585,7 +41546,7 @@
       <c r="E9" s="84"/>
       <c r="F9" s="85"/>
       <c r="G9" s="86" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="H9" s="83"/>
       <c r="I9" s="84"/>
@@ -41596,7 +41557,7 @@
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10" s="75" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="B10" s="87"/>
       <c r="C10" s="87"/>
@@ -41604,7 +41565,7 @@
       <c r="E10" s="87"/>
       <c r="F10" s="87"/>
       <c r="G10" s="87" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="H10" s="87"/>
       <c r="I10" s="87"/>
@@ -41615,7 +41576,7 @@
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11" s="75" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="B11" s="88"/>
       <c r="C11" s="89"/>
@@ -41623,7 +41584,7 @@
       <c r="E11" s="90"/>
       <c r="F11" s="91"/>
       <c r="G11" s="92" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="H11" s="89"/>
       <c r="I11" s="90"/>
@@ -41634,7 +41595,7 @@
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12" s="75" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="B12" s="93"/>
       <c r="C12" s="94"/>
@@ -41642,7 +41603,7 @@
       <c r="E12" s="95"/>
       <c r="F12" s="96"/>
       <c r="G12" s="97" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="H12" s="94"/>
       <c r="I12" s="95"/>
@@ -41653,7 +41614,7 @@
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13" s="75" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="B13" s="93"/>
       <c r="C13" s="94"/>
@@ -41666,17 +41627,17 @@
       <c r="H13" s="453"/>
       <c r="I13" s="454"/>
       <c r="J13" s="98" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="K13" s="86" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="L13" s="99"/>
       <c r="M13" s="100"/>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14" s="75" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="B14" s="101"/>
       <c r="C14" s="101" t="s">
@@ -41685,28 +41646,28 @@
       <c r="D14" s="101"/>
       <c r="E14" s="101"/>
       <c r="F14" s="86" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="G14" s="86" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="H14" s="86" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="I14" s="86" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="J14" s="98" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="K14" s="86" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="L14" s="86" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="M14" s="86" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="O14" s="69" t="s">
         <v>18</v>
@@ -41714,7 +41675,7 @@
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A15" s="75" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="B15" s="102"/>
       <c r="C15" s="103"/>
@@ -41749,7 +41710,7 @@
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A16" s="75" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="B16" s="102"/>
       <c r="C16" s="103"/>
@@ -41784,7 +41745,7 @@
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A17" s="75" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="B17" s="87" t="s">
         <v>160</v>
@@ -41813,7 +41774,7 @@
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A18" s="75" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="B18" s="87" t="s">
         <v>160</v>
@@ -41852,7 +41813,7 @@
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A19" s="75" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="B19" s="102"/>
       <c r="C19" s="103"/>
@@ -41881,15 +41842,15 @@
     </row>
     <row r="20" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A20" s="111" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="B20" s="112"/>
       <c r="C20" s="113"/>
       <c r="D20" s="114" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="E20" s="115" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="F20" s="103"/>
       <c r="G20" s="103"/>
@@ -42294,11 +42255,17 @@
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FE8C99E3-3621-4A94-B7E8-DFCD24F34FA6}">
   <ds:schemaRefs>
+    <ds:schemaRef ds:uri="b2778aaa-fd83-416e-8091-738aa96f6cd3"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="91455a6e-8899-4f67-a6e4-e187ec74b863"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="91455a6e-8899-4f67-a6e4-e187ec74b863"/>
-    <ds:schemaRef ds:uri="b2778aaa-fd83-416e-8091-738aa96f6cd3"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>